<commit_message>
open in colab para la clase 1
</commit_message>
<xml_diff>
--- a/9_asistencia_evaluacion/pivu_caucasia_notas_quices_asistencia.xlsx
+++ b/9_asistencia_evaluacion/pivu_caucasia_notas_quices_asistencia.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marco\Documentos\extension\camino-udea\9_asistencia_evaluacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB08A301-EBFA-4BC0-8F17-997991BE1BBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C25B41B2-1453-4561-84C4-CCD8E192695B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Inscritos" sheetId="2" r:id="rId1"/>
@@ -335,12 +335,6 @@
     <t>adrianamontanoherrera@gmail.com</t>
   </si>
   <si>
-    <t>carvajalrios1992@gmail.com</t>
-  </si>
-  <si>
-    <t>malejacc9209@gmail.com</t>
-  </si>
-  <si>
     <t>raquimus@hotmail.com</t>
   </si>
   <si>
@@ -357,6 +351,12 @@
   </si>
   <si>
     <t>semana_1</t>
+  </si>
+  <si>
+    <t>mariaalejandracuestacaldera@gmail.com</t>
+  </si>
+  <si>
+    <t>yeniferaguirrecarvajal2008@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -367,7 +367,7 @@
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="28" x14ac:knownFonts="1">
+  <fonts count="27" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -551,13 +551,6 @@
       <name val="Aptos Light"/>
       <family val="2"/>
     </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
-      <name val="Aptos Light"/>
-      <family val="2"/>
-    </font>
   </fonts>
   <fills count="13">
     <fill>
@@ -633,7 +626,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="18">
+  <borders count="19">
     <border>
       <left/>
       <right/>
@@ -840,6 +833,17 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -847,7 +851,7 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="140">
+  <cellXfs count="141">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -975,7 +979,6 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -991,113 +994,197 @@
     </xf>
     <xf numFmtId="0" fontId="23" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="22" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1126,15 +1213,6 @@
     <xf numFmtId="0" fontId="3" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1177,81 +1255,10 @@
     <xf numFmtId="0" fontId="3" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="2" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Hipervínculo" xfId="2" builtinId="8"/>
@@ -1733,46 +1740,46 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I38"/>
+  <dimension ref="A1:I39"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.109375" style="38" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="39.109375" style="46" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24.44140625" style="46" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.6640625" style="50" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="39.109375" style="45" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.44140625" style="45" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.6640625" style="49" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="12.88671875" style="38" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.6640625" style="46" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="40.33203125" style="46" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="6" style="47" customWidth="1"/>
+    <col min="6" max="6" width="13.6640625" style="45" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="40.33203125" style="45" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="6" style="46" customWidth="1"/>
     <col min="9" max="9" width="22.77734375" style="38" customWidth="1"/>
     <col min="10" max="16384" width="11.44140625" style="38"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="72" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="54" t="s">
+      <c r="A1" s="87" t="s">
         <v>27</v>
       </c>
-      <c r="B1" s="53"/>
-      <c r="C1" s="53"/>
-      <c r="D1" s="53"/>
-      <c r="E1" s="53"/>
-      <c r="F1" s="53"/>
-      <c r="G1" s="53"/>
-      <c r="H1" s="53"/>
+      <c r="B1" s="86"/>
+      <c r="C1" s="86"/>
+      <c r="D1" s="86"/>
+      <c r="E1" s="86"/>
+      <c r="F1" s="86"/>
+      <c r="G1" s="86"/>
+      <c r="H1" s="86"/>
     </row>
     <row r="2" spans="1:9" ht="19.8" x14ac:dyDescent="0.3">
-      <c r="A2" s="53" t="s">
+      <c r="A2" s="86" t="s">
         <v>26</v>
       </c>
-      <c r="B2" s="53"/>
-      <c r="C2" s="53"/>
-      <c r="D2" s="53"/>
-      <c r="E2" s="53"/>
-      <c r="F2" s="53"/>
-      <c r="G2" s="53"/>
-      <c r="H2" s="53"/>
-      <c r="I2" s="52" t="s">
-        <v>104</v>
+      <c r="B2" s="86"/>
+      <c r="C2" s="86"/>
+      <c r="D2" s="86"/>
+      <c r="E2" s="86"/>
+      <c r="F2" s="86"/>
+      <c r="G2" s="86"/>
+      <c r="H2" s="86"/>
+      <c r="I2" s="51" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
@@ -1785,7 +1792,7 @@
       <c r="C3" s="41" t="s">
         <v>57</v>
       </c>
-      <c r="D3" s="48" t="s">
+      <c r="D3" s="47" t="s">
         <v>14</v>
       </c>
       <c r="E3" s="39" t="s">
@@ -1811,7 +1818,7 @@
       <c r="C4" s="44" t="s">
         <v>28</v>
       </c>
-      <c r="D4" s="49">
+      <c r="D4" s="48">
         <v>1038110235</v>
       </c>
       <c r="E4" s="44">
@@ -1835,7 +1842,7 @@
       <c r="C5" s="44" t="s">
         <v>30</v>
       </c>
-      <c r="D5" s="49">
+      <c r="D5" s="48">
         <v>1038117202</v>
       </c>
       <c r="E5" s="44">
@@ -1859,7 +1866,7 @@
       <c r="C6" s="44" t="s">
         <v>28</v>
       </c>
-      <c r="D6" s="49">
+      <c r="D6" s="48">
         <v>1041633525</v>
       </c>
       <c r="E6" s="44">
@@ -1883,7 +1890,7 @@
       <c r="C7" s="44" t="s">
         <v>30</v>
       </c>
-      <c r="D7" s="49">
+      <c r="D7" s="48">
         <v>1038648794</v>
       </c>
       <c r="E7" s="44">
@@ -1907,7 +1914,7 @@
       <c r="C8" s="44" t="s">
         <v>28</v>
       </c>
-      <c r="D8" s="49">
+      <c r="D8" s="48">
         <v>1040505284</v>
       </c>
       <c r="E8" s="44">
@@ -1920,6 +1927,9 @@
         <v>78</v>
       </c>
       <c r="H8" s="44"/>
+      <c r="I8" s="38">
+        <v>1</v>
+      </c>
     </row>
     <row r="9" spans="1:9" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="42">
@@ -1931,7 +1941,7 @@
       <c r="C9" s="44" t="s">
         <v>28</v>
       </c>
-      <c r="D9" s="49">
+      <c r="D9" s="48">
         <v>1038110143</v>
       </c>
       <c r="E9" s="44">
@@ -1940,11 +1950,11 @@
       <c r="F9" s="44">
         <v>3203519315</v>
       </c>
-      <c r="G9" s="45" t="s">
+      <c r="G9" s="140" t="s">
         <v>95</v>
       </c>
-      <c r="H9" s="51" t="s">
-        <v>103</v>
+      <c r="H9" s="50" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -1957,7 +1967,7 @@
       <c r="C10" s="44" t="s">
         <v>28</v>
       </c>
-      <c r="D10" s="49">
+      <c r="D10" s="48">
         <v>1038114008</v>
       </c>
       <c r="E10" s="44">
@@ -1981,7 +1991,7 @@
       <c r="C11" s="44" t="s">
         <v>28</v>
       </c>
-      <c r="D11" s="49">
+      <c r="D11" s="48">
         <v>1038116790</v>
       </c>
       <c r="E11" s="44">
@@ -2005,7 +2015,7 @@
       <c r="C12" s="44" t="s">
         <v>28</v>
       </c>
-      <c r="D12" s="49">
+      <c r="D12" s="48">
         <v>1038111245</v>
       </c>
       <c r="E12" s="44">
@@ -2029,7 +2039,7 @@
       <c r="C13" s="44" t="s">
         <v>30</v>
       </c>
-      <c r="D13" s="49">
+      <c r="D13" s="48">
         <v>1038134078</v>
       </c>
       <c r="E13" s="44">
@@ -2038,11 +2048,11 @@
       <c r="F13" s="44">
         <v>3136630762</v>
       </c>
-      <c r="G13" s="44" t="s">
-        <v>100</v>
-      </c>
-      <c r="H13" s="51" t="s">
-        <v>103</v>
+      <c r="G13" s="140" t="s">
+        <v>98</v>
+      </c>
+      <c r="H13" s="50" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2055,7 +2065,7 @@
       <c r="C14" s="44" t="s">
         <v>30</v>
       </c>
-      <c r="D14" s="49">
+      <c r="D14" s="48">
         <v>1038647898</v>
       </c>
       <c r="E14" s="44">
@@ -2079,7 +2089,7 @@
       <c r="C15" s="44" t="s">
         <v>28</v>
       </c>
-      <c r="D15" s="49">
+      <c r="D15" s="48">
         <v>1038112414</v>
       </c>
       <c r="E15" s="44">
@@ -2103,7 +2113,7 @@
       <c r="C16" s="44" t="s">
         <v>30</v>
       </c>
-      <c r="D16" s="49">
+      <c r="D16" s="48">
         <v>1038109330</v>
       </c>
       <c r="E16" s="44">
@@ -2127,7 +2137,7 @@
       <c r="C17" s="44" t="s">
         <v>30</v>
       </c>
-      <c r="D17" s="49">
+      <c r="D17" s="48">
         <v>1038647796</v>
       </c>
       <c r="E17" s="44">
@@ -2151,7 +2161,7 @@
       <c r="C18" s="44" t="s">
         <v>30</v>
       </c>
-      <c r="D18" s="49">
+      <c r="D18" s="48">
         <v>1038105559</v>
       </c>
       <c r="E18" s="44">
@@ -2175,7 +2185,7 @@
       <c r="C19" s="44" t="s">
         <v>28</v>
       </c>
-      <c r="D19" s="49">
+      <c r="D19" s="48">
         <v>1011513720</v>
       </c>
       <c r="E19" s="44">
@@ -2184,11 +2194,11 @@
       <c r="F19" s="44">
         <v>3218798123</v>
       </c>
-      <c r="G19" s="44" t="s">
+      <c r="G19" s="140" t="s">
+        <v>104</v>
+      </c>
+      <c r="H19" s="50" t="s">
         <v>99</v>
-      </c>
-      <c r="H19" s="51" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="20" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2201,7 +2211,7 @@
       <c r="C20" s="44" t="s">
         <v>28</v>
       </c>
-      <c r="D20" s="49">
+      <c r="D20" s="48">
         <v>1038114154</v>
       </c>
       <c r="E20" s="44">
@@ -2225,7 +2235,7 @@
       <c r="C21" s="44" t="s">
         <v>28</v>
       </c>
-      <c r="D21" s="49">
+      <c r="D21" s="48">
         <v>1038113598</v>
       </c>
       <c r="E21" s="44">
@@ -2249,7 +2259,7 @@
       <c r="C22" s="44" t="s">
         <v>28</v>
       </c>
-      <c r="D22" s="49">
+      <c r="D22" s="48">
         <v>1038648337</v>
       </c>
       <c r="E22" s="44">
@@ -2259,8 +2269,8 @@
         <v>3145134544</v>
       </c>
       <c r="G22" s="44"/>
-      <c r="H22" s="51" t="s">
-        <v>102</v>
+      <c r="H22" s="50" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="23" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2273,7 +2283,7 @@
       <c r="C23" s="44" t="s">
         <v>28</v>
       </c>
-      <c r="D23" s="49">
+      <c r="D23" s="48">
         <v>1073690694</v>
       </c>
       <c r="E23" s="44">
@@ -2297,7 +2307,7 @@
       <c r="C24" s="44" t="s">
         <v>28</v>
       </c>
-      <c r="D24" s="49">
+      <c r="D24" s="48">
         <v>1066518419</v>
       </c>
       <c r="E24" s="44">
@@ -2321,7 +2331,7 @@
       <c r="C25" s="44" t="s">
         <v>28</v>
       </c>
-      <c r="D25" s="49">
+      <c r="D25" s="48">
         <v>1038114203</v>
       </c>
       <c r="E25" s="44">
@@ -2345,7 +2355,7 @@
       <c r="C26" s="44" t="s">
         <v>28</v>
       </c>
-      <c r="D26" s="49">
+      <c r="D26" s="48">
         <v>1038115554</v>
       </c>
       <c r="E26" s="44">
@@ -2369,7 +2379,7 @@
       <c r="C27" s="44" t="s">
         <v>28</v>
       </c>
-      <c r="D27" s="49">
+      <c r="D27" s="48">
         <v>1038109706</v>
       </c>
       <c r="E27" s="44">
@@ -2393,7 +2403,7 @@
       <c r="C28" s="44" t="s">
         <v>28</v>
       </c>
-      <c r="D28" s="49">
+      <c r="D28" s="48">
         <v>1038115449</v>
       </c>
       <c r="E28" s="44">
@@ -2417,7 +2427,7 @@
       <c r="C29" s="44" t="s">
         <v>28</v>
       </c>
-      <c r="D29" s="49">
+      <c r="D29" s="48">
         <v>1038112417</v>
       </c>
       <c r="E29" s="44">
@@ -2441,7 +2451,7 @@
       <c r="C30" s="44" t="s">
         <v>30</v>
       </c>
-      <c r="D30" s="49">
+      <c r="D30" s="48">
         <v>1038104210</v>
       </c>
       <c r="E30" s="44">
@@ -2465,7 +2475,7 @@
       <c r="C31" s="44" t="s">
         <v>28</v>
       </c>
-      <c r="D31" s="49">
+      <c r="D31" s="48">
         <v>1100016222</v>
       </c>
       <c r="E31" s="44">
@@ -2489,7 +2499,7 @@
       <c r="C32" s="44" t="s">
         <v>28</v>
       </c>
-      <c r="D32" s="49">
+      <c r="D32" s="48">
         <v>1038111917</v>
       </c>
       <c r="E32" s="44">
@@ -2513,7 +2523,7 @@
       <c r="C33" s="44" t="s">
         <v>28</v>
       </c>
-      <c r="D33" s="49">
+      <c r="D33" s="48">
         <v>1038115337</v>
       </c>
       <c r="E33" s="44">
@@ -2537,7 +2547,7 @@
       <c r="C34" s="44" t="s">
         <v>28</v>
       </c>
-      <c r="D34" s="49">
+      <c r="D34" s="48">
         <v>1116074065</v>
       </c>
       <c r="E34" s="44">
@@ -2561,7 +2571,7 @@
       <c r="C35" s="44" t="s">
         <v>28</v>
       </c>
-      <c r="D35" s="49">
+      <c r="D35" s="48">
         <v>1125368371</v>
       </c>
       <c r="E35" s="44">
@@ -2585,7 +2595,7 @@
       <c r="C36" s="44" t="s">
         <v>30</v>
       </c>
-      <c r="D36" s="49">
+      <c r="D36" s="48">
         <v>1038104997</v>
       </c>
       <c r="E36" s="44">
@@ -2609,7 +2619,7 @@
       <c r="C37" s="44" t="s">
         <v>28</v>
       </c>
-      <c r="D37" s="49">
+      <c r="D37" s="48">
         <v>1038113397</v>
       </c>
       <c r="E37" s="44">
@@ -2633,19 +2643,24 @@
       <c r="C38" s="44" t="s">
         <v>28</v>
       </c>
-      <c r="D38" s="49">
+      <c r="D38" s="48">
         <v>1038111032</v>
       </c>
       <c r="E38" s="44">
         <v>3209212858</v>
       </c>
       <c r="F38" s="44">
-        <v>3209212858</v>
-      </c>
-      <c r="G38" s="44" t="s">
-        <v>98</v>
+        <v>3212234096</v>
+      </c>
+      <c r="G38" s="140" t="s">
+        <v>105</v>
       </c>
       <c r="H38" s="44"/>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A39" s="38">
+        <v>36</v>
+      </c>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B4:G38">
@@ -2658,16 +2673,19 @@
   <phoneticPr fontId="2" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="G9" r:id="rId1" xr:uid="{4A79F488-B592-4729-8CEE-7BB35CBDDEFA}"/>
+    <hyperlink ref="G19" r:id="rId2" xr:uid="{0D63D482-2B15-4CBD-8A6E-32A20A7492DB}"/>
+    <hyperlink ref="G38" r:id="rId3" xr:uid="{F41688A5-1CDE-42E7-9CB3-E623ADE29950}"/>
+    <hyperlink ref="G13" r:id="rId4" xr:uid="{5EC44252-B9A4-45C6-9F57-A5A815D8FC04}"/>
   </hyperlinks>
   <pageMargins left="0.19685039370078741" right="0.19685039370078741" top="0.19685039370078741" bottom="0.19685039370078741" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup scale="80" orientation="landscape" r:id="rId2"/>
-  <drawing r:id="rId3"/>
+  <pageSetup scale="80" orientation="landscape" r:id="rId5"/>
+  <drawing r:id="rId6"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:AE39"/>
+  <dimension ref="A1:AE40"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="34.5546875" bestFit="1" customWidth="1"/>
@@ -2683,174 +2701,174 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:31" ht="66" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B1" s="62" t="s">
+      <c r="B1" s="59" t="s">
         <v>18</v>
       </c>
-      <c r="C1" s="62"/>
-      <c r="D1" s="62"/>
-      <c r="E1" s="62"/>
-      <c r="F1" s="62"/>
-      <c r="G1" s="62"/>
-      <c r="H1" s="62"/>
-      <c r="I1" s="62"/>
-      <c r="J1" s="62"/>
-      <c r="K1" s="62"/>
-      <c r="L1" s="62"/>
-      <c r="M1" s="62"/>
-      <c r="N1" s="62"/>
-      <c r="O1" s="62"/>
-      <c r="P1" s="62"/>
-      <c r="Q1" s="62"/>
-      <c r="R1" s="62"/>
-      <c r="S1" s="62"/>
-      <c r="T1" s="62"/>
-      <c r="U1" s="62"/>
-      <c r="V1" s="62"/>
-      <c r="W1" s="62"/>
-      <c r="X1" s="62"/>
-      <c r="Y1" s="62"/>
-      <c r="Z1" s="62"/>
-      <c r="AA1" s="62"/>
-      <c r="AB1" s="62"/>
-      <c r="AC1" s="62"/>
-      <c r="AD1" s="62"/>
-      <c r="AE1" s="62"/>
+      <c r="C1" s="59"/>
+      <c r="D1" s="59"/>
+      <c r="E1" s="59"/>
+      <c r="F1" s="59"/>
+      <c r="G1" s="59"/>
+      <c r="H1" s="59"/>
+      <c r="I1" s="59"/>
+      <c r="J1" s="59"/>
+      <c r="K1" s="59"/>
+      <c r="L1" s="59"/>
+      <c r="M1" s="59"/>
+      <c r="N1" s="59"/>
+      <c r="O1" s="59"/>
+      <c r="P1" s="59"/>
+      <c r="Q1" s="59"/>
+      <c r="R1" s="59"/>
+      <c r="S1" s="59"/>
+      <c r="T1" s="59"/>
+      <c r="U1" s="59"/>
+      <c r="V1" s="59"/>
+      <c r="W1" s="59"/>
+      <c r="X1" s="59"/>
+      <c r="Y1" s="59"/>
+      <c r="Z1" s="59"/>
+      <c r="AA1" s="59"/>
+      <c r="AB1" s="59"/>
+      <c r="AC1" s="59"/>
+      <c r="AD1" s="59"/>
+      <c r="AE1" s="59"/>
     </row>
     <row r="2" spans="1:31" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="63" t="s">
+      <c r="A2" s="60" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="87" t="s">
+      <c r="B2" s="84" t="s">
         <v>21</v>
       </c>
-      <c r="C2" s="63" t="s">
+      <c r="C2" s="60" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="80" t="s">
+      <c r="D2" s="77" t="s">
         <v>19</v>
       </c>
-      <c r="E2" s="81"/>
-      <c r="F2" s="81"/>
-      <c r="G2" s="81"/>
-      <c r="H2" s="82"/>
-      <c r="I2" s="65" t="s">
+      <c r="E2" s="78"/>
+      <c r="F2" s="78"/>
+      <c r="G2" s="78"/>
+      <c r="H2" s="79"/>
+      <c r="I2" s="62" t="s">
         <v>19</v>
       </c>
-      <c r="J2" s="66"/>
-      <c r="K2" s="66"/>
-      <c r="L2" s="66"/>
-      <c r="M2" s="66"/>
-      <c r="N2" s="66"/>
-      <c r="O2" s="66"/>
-      <c r="P2" s="66"/>
-      <c r="Q2" s="67"/>
-      <c r="R2" s="74" t="s">
+      <c r="J2" s="63"/>
+      <c r="K2" s="63"/>
+      <c r="L2" s="63"/>
+      <c r="M2" s="63"/>
+      <c r="N2" s="63"/>
+      <c r="O2" s="63"/>
+      <c r="P2" s="63"/>
+      <c r="Q2" s="64"/>
+      <c r="R2" s="71" t="s">
         <v>19</v>
       </c>
-      <c r="S2" s="75"/>
-      <c r="T2" s="75"/>
-      <c r="U2" s="75"/>
-      <c r="V2" s="75"/>
-      <c r="W2" s="75"/>
-      <c r="X2" s="75"/>
-      <c r="Y2" s="75"/>
-      <c r="Z2" s="76"/>
-      <c r="AA2" s="55" t="s">
+      <c r="S2" s="72"/>
+      <c r="T2" s="72"/>
+      <c r="U2" s="72"/>
+      <c r="V2" s="72"/>
+      <c r="W2" s="72"/>
+      <c r="X2" s="72"/>
+      <c r="Y2" s="72"/>
+      <c r="Z2" s="73"/>
+      <c r="AA2" s="52" t="s">
         <v>19</v>
       </c>
-      <c r="AB2" s="56"/>
-      <c r="AC2" s="56"/>
-      <c r="AD2" s="56"/>
-      <c r="AE2" s="57"/>
+      <c r="AB2" s="53"/>
+      <c r="AC2" s="53"/>
+      <c r="AD2" s="53"/>
+      <c r="AE2" s="54"/>
     </row>
     <row r="3" spans="1:31" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="64"/>
-      <c r="B3" s="88"/>
-      <c r="C3" s="64"/>
-      <c r="D3" s="83" t="s">
+      <c r="A3" s="61"/>
+      <c r="B3" s="85"/>
+      <c r="C3" s="61"/>
+      <c r="D3" s="80" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="84"/>
-      <c r="F3" s="84"/>
-      <c r="G3" s="84"/>
-      <c r="H3" s="85"/>
-      <c r="I3" s="68" t="s">
+      <c r="E3" s="81"/>
+      <c r="F3" s="81"/>
+      <c r="G3" s="81"/>
+      <c r="H3" s="82"/>
+      <c r="I3" s="65" t="s">
         <v>2</v>
       </c>
-      <c r="J3" s="69"/>
-      <c r="K3" s="69"/>
-      <c r="L3" s="69"/>
-      <c r="M3" s="69"/>
-      <c r="N3" s="69"/>
-      <c r="O3" s="69"/>
-      <c r="P3" s="69"/>
-      <c r="Q3" s="70"/>
-      <c r="R3" s="77" t="s">
+      <c r="J3" s="66"/>
+      <c r="K3" s="66"/>
+      <c r="L3" s="66"/>
+      <c r="M3" s="66"/>
+      <c r="N3" s="66"/>
+      <c r="O3" s="66"/>
+      <c r="P3" s="66"/>
+      <c r="Q3" s="67"/>
+      <c r="R3" s="74" t="s">
         <v>1</v>
       </c>
-      <c r="S3" s="78"/>
-      <c r="T3" s="78"/>
-      <c r="U3" s="78"/>
-      <c r="V3" s="78"/>
-      <c r="W3" s="78"/>
-      <c r="X3" s="78"/>
-      <c r="Y3" s="78"/>
-      <c r="Z3" s="79"/>
-      <c r="AA3" s="58" t="s">
-        <v>0</v>
-      </c>
-      <c r="AB3" s="59"/>
-      <c r="AC3" s="59"/>
-      <c r="AD3" s="59"/>
-      <c r="AE3" s="60"/>
+      <c r="S3" s="75"/>
+      <c r="T3" s="75"/>
+      <c r="U3" s="75"/>
+      <c r="V3" s="75"/>
+      <c r="W3" s="75"/>
+      <c r="X3" s="75"/>
+      <c r="Y3" s="75"/>
+      <c r="Z3" s="76"/>
+      <c r="AA3" s="55" t="s">
+        <v>0</v>
+      </c>
+      <c r="AB3" s="56"/>
+      <c r="AC3" s="56"/>
+      <c r="AD3" s="56"/>
+      <c r="AE3" s="57"/>
     </row>
     <row r="4" spans="1:31" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="64"/>
-      <c r="B4" s="88"/>
-      <c r="C4" s="64"/>
-      <c r="D4" s="86" t="s">
+      <c r="A4" s="61"/>
+      <c r="B4" s="85"/>
+      <c r="C4" s="61"/>
+      <c r="D4" s="83" t="s">
         <v>22</v>
       </c>
-      <c r="E4" s="72"/>
-      <c r="F4" s="72"/>
-      <c r="G4" s="73"/>
+      <c r="E4" s="69"/>
+      <c r="F4" s="69"/>
+      <c r="G4" s="70"/>
       <c r="H4" s="1"/>
-      <c r="I4" s="71" t="s">
+      <c r="I4" s="68" t="s">
         <v>23</v>
       </c>
-      <c r="J4" s="72"/>
-      <c r="K4" s="72"/>
-      <c r="L4" s="72"/>
-      <c r="M4" s="72"/>
-      <c r="N4" s="72"/>
-      <c r="O4" s="72"/>
-      <c r="P4" s="73"/>
+      <c r="J4" s="69"/>
+      <c r="K4" s="69"/>
+      <c r="L4" s="69"/>
+      <c r="M4" s="69"/>
+      <c r="N4" s="69"/>
+      <c r="O4" s="69"/>
+      <c r="P4" s="70"/>
       <c r="Q4" s="3"/>
-      <c r="R4" s="71" t="s">
+      <c r="R4" s="68" t="s">
         <v>23</v>
       </c>
-      <c r="S4" s="72"/>
-      <c r="T4" s="72"/>
-      <c r="U4" s="72"/>
-      <c r="V4" s="72"/>
-      <c r="W4" s="72"/>
-      <c r="X4" s="72"/>
-      <c r="Y4" s="73"/>
+      <c r="S4" s="69"/>
+      <c r="T4" s="69"/>
+      <c r="U4" s="69"/>
+      <c r="V4" s="69"/>
+      <c r="W4" s="69"/>
+      <c r="X4" s="69"/>
+      <c r="Y4" s="70"/>
       <c r="Z4" s="12"/>
-      <c r="AA4" s="61" t="s">
+      <c r="AA4" s="58" t="s">
         <v>23</v>
       </c>
-      <c r="AB4" s="61"/>
-      <c r="AC4" s="61"/>
-      <c r="AD4" s="61"/>
+      <c r="AB4" s="58"/>
+      <c r="AC4" s="58"/>
+      <c r="AD4" s="58"/>
       <c r="AE4" s="3"/>
     </row>
     <row r="5" spans="1:31" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="64"/>
-      <c r="B5" s="88"/>
-      <c r="C5" s="64"/>
+      <c r="A5" s="61"/>
+      <c r="B5" s="85"/>
+      <c r="C5" s="61"/>
       <c r="D5" s="28" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="E5" s="28"/>
       <c r="F5" s="28"/>
@@ -3112,13 +3130,15 @@
         <f>+Inscritos!D8</f>
         <v>1040505284</v>
       </c>
-      <c r="D10" s="13"/>
+      <c r="D10" s="13">
+        <v>1</v>
+      </c>
       <c r="E10" s="13"/>
       <c r="F10" s="13"/>
       <c r="G10" s="13"/>
       <c r="H10" s="32">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="I10" s="33"/>
       <c r="J10" s="33"/>
@@ -3642,13 +3662,15 @@
         <f>+Inscritos!D18</f>
         <v>1038105559</v>
       </c>
-      <c r="D20" s="13"/>
+      <c r="D20" s="13">
+        <v>1</v>
+      </c>
       <c r="E20" s="13"/>
       <c r="F20" s="13"/>
       <c r="G20" s="13"/>
       <c r="H20" s="32">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="I20" s="33"/>
       <c r="J20" s="33"/>
@@ -4278,13 +4300,15 @@
         <f>+Inscritos!D30</f>
         <v>1038104210</v>
       </c>
-      <c r="D32" s="13"/>
+      <c r="D32" s="13">
+        <v>1</v>
+      </c>
       <c r="E32" s="13"/>
       <c r="F32" s="13"/>
       <c r="G32" s="13"/>
       <c r="H32" s="32">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="I32" s="33"/>
       <c r="J32" s="33"/>
@@ -4332,14 +4356,14 @@
         <v>1100016222</v>
       </c>
       <c r="D33" s="13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E33" s="13"/>
       <c r="F33" s="13"/>
       <c r="G33" s="13"/>
       <c r="H33" s="32">
         <f t="shared" si="0"/>
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="I33" s="33"/>
       <c r="J33" s="33"/>
@@ -4492,13 +4516,15 @@
         <f>+Inscritos!D34</f>
         <v>1116074065</v>
       </c>
-      <c r="D36" s="13"/>
+      <c r="D36" s="13">
+        <v>1</v>
+      </c>
       <c r="E36" s="13"/>
       <c r="F36" s="13"/>
       <c r="G36" s="13"/>
       <c r="H36" s="32">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="I36" s="33"/>
       <c r="J36" s="33"/>
@@ -4690,6 +4716,11 @@
       <c r="AE39" s="32">
         <f t="shared" si="3"/>
         <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A40" s="139">
+        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -4744,123 +4775,123 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="72.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B1" s="115" t="s">
+      <c r="B1" s="88" t="s">
         <v>18</v>
       </c>
-      <c r="C1" s="115"/>
-      <c r="D1" s="115"/>
-      <c r="E1" s="115"/>
-      <c r="F1" s="115"/>
-      <c r="G1" s="115"/>
-      <c r="H1" s="115"/>
-      <c r="I1" s="115"/>
-      <c r="J1" s="115"/>
-      <c r="K1" s="115"/>
-      <c r="L1" s="115"/>
-      <c r="M1" s="115"/>
-      <c r="N1" s="115"/>
-      <c r="O1" s="115"/>
-      <c r="P1" s="115"/>
-      <c r="Q1" s="115"/>
-      <c r="R1" s="115"/>
-      <c r="S1" s="115"/>
-      <c r="T1" s="115"/>
+      <c r="C1" s="88"/>
+      <c r="D1" s="88"/>
+      <c r="E1" s="88"/>
+      <c r="F1" s="88"/>
+      <c r="G1" s="88"/>
+      <c r="H1" s="88"/>
+      <c r="I1" s="88"/>
+      <c r="J1" s="88"/>
+      <c r="K1" s="88"/>
+      <c r="L1" s="88"/>
+      <c r="M1" s="88"/>
+      <c r="N1" s="88"/>
+      <c r="O1" s="88"/>
+      <c r="P1" s="88"/>
+      <c r="Q1" s="88"/>
+      <c r="R1" s="88"/>
+      <c r="S1" s="88"/>
+      <c r="T1" s="88"/>
     </row>
     <row r="2" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="101" t="s">
+      <c r="A2" s="125" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="87" t="s">
+      <c r="B2" s="84" t="s">
         <v>21</v>
       </c>
-      <c r="C2" s="63" t="s">
+      <c r="C2" s="60" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="89" t="str">
+      <c r="D2" s="116" t="str">
         <f>Asistencia!D2</f>
         <v>NOMBRE DOCENTE</v>
       </c>
-      <c r="E2" s="90"/>
-      <c r="F2" s="91"/>
-      <c r="G2" s="89" t="str">
+      <c r="E2" s="117"/>
+      <c r="F2" s="118"/>
+      <c r="G2" s="116" t="str">
         <f>Asistencia!I2</f>
         <v>NOMBRE DOCENTE</v>
       </c>
-      <c r="H2" s="90"/>
-      <c r="I2" s="90"/>
-      <c r="J2" s="90"/>
-      <c r="K2" s="91"/>
-      <c r="L2" s="89" t="s">
+      <c r="H2" s="117"/>
+      <c r="I2" s="117"/>
+      <c r="J2" s="117"/>
+      <c r="K2" s="118"/>
+      <c r="L2" s="116" t="s">
         <v>19</v>
       </c>
-      <c r="M2" s="90"/>
-      <c r="N2" s="90"/>
-      <c r="O2" s="90"/>
-      <c r="P2" s="91"/>
-      <c r="Q2" s="89" t="str">
+      <c r="M2" s="117"/>
+      <c r="N2" s="117"/>
+      <c r="O2" s="117"/>
+      <c r="P2" s="118"/>
+      <c r="Q2" s="116" t="str">
         <f>Asistencia!AA2</f>
         <v>NOMBRE DOCENTE</v>
       </c>
-      <c r="R2" s="90"/>
-      <c r="S2" s="90"/>
-      <c r="T2" s="91"/>
+      <c r="R2" s="117"/>
+      <c r="S2" s="117"/>
+      <c r="T2" s="118"/>
     </row>
     <row r="3" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="102"/>
-      <c r="B3" s="88"/>
-      <c r="C3" s="64"/>
-      <c r="D3" s="109" t="s">
+      <c r="A3" s="126"/>
+      <c r="B3" s="85"/>
+      <c r="C3" s="61"/>
+      <c r="D3" s="133" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="110"/>
-      <c r="F3" s="111"/>
-      <c r="G3" s="103" t="s">
+      <c r="E3" s="134"/>
+      <c r="F3" s="135"/>
+      <c r="G3" s="127" t="s">
         <v>2</v>
       </c>
-      <c r="H3" s="104"/>
-      <c r="I3" s="104"/>
-      <c r="J3" s="104"/>
-      <c r="K3" s="105"/>
-      <c r="L3" s="134" t="s">
+      <c r="H3" s="128"/>
+      <c r="I3" s="128"/>
+      <c r="J3" s="128"/>
+      <c r="K3" s="129"/>
+      <c r="L3" s="110" t="s">
         <v>1</v>
       </c>
-      <c r="M3" s="135"/>
-      <c r="N3" s="135"/>
-      <c r="O3" s="135"/>
-      <c r="P3" s="136"/>
-      <c r="Q3" s="92" t="s">
-        <v>0</v>
-      </c>
-      <c r="R3" s="93"/>
-      <c r="S3" s="93"/>
-      <c r="T3" s="94"/>
+      <c r="M3" s="111"/>
+      <c r="N3" s="111"/>
+      <c r="O3" s="111"/>
+      <c r="P3" s="112"/>
+      <c r="Q3" s="119" t="s">
+        <v>0</v>
+      </c>
+      <c r="R3" s="120"/>
+      <c r="S3" s="120"/>
+      <c r="T3" s="121"/>
     </row>
     <row r="4" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="102"/>
-      <c r="B4" s="88"/>
-      <c r="C4" s="64"/>
-      <c r="D4" s="112"/>
-      <c r="E4" s="113"/>
-      <c r="F4" s="114"/>
-      <c r="G4" s="106"/>
-      <c r="H4" s="107"/>
-      <c r="I4" s="107"/>
-      <c r="J4" s="107"/>
-      <c r="K4" s="108"/>
-      <c r="L4" s="137"/>
-      <c r="M4" s="138"/>
-      <c r="N4" s="138"/>
-      <c r="O4" s="138"/>
-      <c r="P4" s="139"/>
-      <c r="Q4" s="95"/>
-      <c r="R4" s="96"/>
-      <c r="S4" s="96"/>
-      <c r="T4" s="97"/>
+      <c r="A4" s="126"/>
+      <c r="B4" s="85"/>
+      <c r="C4" s="61"/>
+      <c r="D4" s="136"/>
+      <c r="E4" s="137"/>
+      <c r="F4" s="138"/>
+      <c r="G4" s="130"/>
+      <c r="H4" s="131"/>
+      <c r="I4" s="131"/>
+      <c r="J4" s="131"/>
+      <c r="K4" s="132"/>
+      <c r="L4" s="113"/>
+      <c r="M4" s="114"/>
+      <c r="N4" s="114"/>
+      <c r="O4" s="114"/>
+      <c r="P4" s="115"/>
+      <c r="Q4" s="122"/>
+      <c r="R4" s="123"/>
+      <c r="S4" s="123"/>
+      <c r="T4" s="124"/>
     </row>
     <row r="5" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="102"/>
-      <c r="B5" s="88"/>
-      <c r="C5" s="64"/>
+      <c r="A5" s="126"/>
+      <c r="B5" s="85"/>
+      <c r="C5" s="61"/>
       <c r="D5" s="17">
         <v>0.75</v>
       </c>
@@ -7434,186 +7465,195 @@
       </c>
     </row>
     <row r="66" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D66" s="119" t="s">
+      <c r="D66" s="92" t="s">
         <v>24</v>
       </c>
-      <c r="E66" s="122" t="s">
+      <c r="E66" s="95" t="s">
         <v>12</v>
       </c>
-      <c r="G66" s="116" t="s">
+      <c r="G66" s="89" t="s">
         <v>8</v>
       </c>
-      <c r="H66" s="128" t="s">
+      <c r="H66" s="104" t="s">
         <v>9</v>
       </c>
-      <c r="I66" s="128" t="s">
+      <c r="I66" s="104" t="s">
         <v>10</v>
       </c>
-      <c r="J66" s="116" t="s">
+      <c r="J66" s="89" t="s">
         <v>11</v>
       </c>
       <c r="L66" s="98" t="s">
         <v>8</v>
       </c>
-      <c r="M66" s="125" t="s">
+      <c r="M66" s="101" t="s">
         <v>9</v>
       </c>
-      <c r="N66" s="125" t="s">
+      <c r="N66" s="101" t="s">
         <v>10</v>
       </c>
       <c r="O66" s="98" t="s">
         <v>11</v>
       </c>
-      <c r="Q66" s="131" t="s">
+      <c r="Q66" s="107" t="s">
         <v>24</v>
       </c>
-      <c r="R66" s="131" t="s">
+      <c r="R66" s="107" t="s">
         <v>4</v>
       </c>
-      <c r="S66" s="131" t="s">
+      <c r="S66" s="107" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="67" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D67" s="120"/>
-      <c r="E67" s="123"/>
-      <c r="G67" s="117"/>
-      <c r="H67" s="129"/>
-      <c r="I67" s="129"/>
-      <c r="J67" s="117"/>
+      <c r="D67" s="93"/>
+      <c r="E67" s="96"/>
+      <c r="G67" s="90"/>
+      <c r="H67" s="105"/>
+      <c r="I67" s="105"/>
+      <c r="J67" s="90"/>
       <c r="L67" s="99"/>
-      <c r="M67" s="126"/>
-      <c r="N67" s="126"/>
+      <c r="M67" s="102"/>
+      <c r="N67" s="102"/>
       <c r="O67" s="99"/>
-      <c r="Q67" s="132"/>
-      <c r="R67" s="132"/>
-      <c r="S67" s="132"/>
+      <c r="Q67" s="108"/>
+      <c r="R67" s="108"/>
+      <c r="S67" s="108"/>
     </row>
     <row r="68" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D68" s="120"/>
-      <c r="E68" s="123"/>
-      <c r="G68" s="117"/>
-      <c r="H68" s="129"/>
-      <c r="I68" s="129"/>
-      <c r="J68" s="117"/>
+      <c r="D68" s="93"/>
+      <c r="E68" s="96"/>
+      <c r="G68" s="90"/>
+      <c r="H68" s="105"/>
+      <c r="I68" s="105"/>
+      <c r="J68" s="90"/>
       <c r="L68" s="99"/>
-      <c r="M68" s="126"/>
-      <c r="N68" s="126"/>
+      <c r="M68" s="102"/>
+      <c r="N68" s="102"/>
       <c r="O68" s="99"/>
-      <c r="Q68" s="132"/>
-      <c r="R68" s="132"/>
-      <c r="S68" s="132"/>
+      <c r="Q68" s="108"/>
+      <c r="R68" s="108"/>
+      <c r="S68" s="108"/>
     </row>
     <row r="69" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D69" s="120"/>
-      <c r="E69" s="123"/>
-      <c r="G69" s="117"/>
-      <c r="H69" s="129"/>
-      <c r="I69" s="129"/>
-      <c r="J69" s="117"/>
+      <c r="D69" s="93"/>
+      <c r="E69" s="96"/>
+      <c r="G69" s="90"/>
+      <c r="H69" s="105"/>
+      <c r="I69" s="105"/>
+      <c r="J69" s="90"/>
       <c r="L69" s="99"/>
-      <c r="M69" s="126"/>
-      <c r="N69" s="126"/>
+      <c r="M69" s="102"/>
+      <c r="N69" s="102"/>
       <c r="O69" s="99"/>
-      <c r="Q69" s="132"/>
-      <c r="R69" s="132"/>
-      <c r="S69" s="132"/>
+      <c r="Q69" s="108"/>
+      <c r="R69" s="108"/>
+      <c r="S69" s="108"/>
     </row>
     <row r="70" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D70" s="120"/>
-      <c r="E70" s="123"/>
-      <c r="G70" s="117"/>
-      <c r="H70" s="129"/>
-      <c r="I70" s="129"/>
-      <c r="J70" s="117"/>
+      <c r="D70" s="93"/>
+      <c r="E70" s="96"/>
+      <c r="G70" s="90"/>
+      <c r="H70" s="105"/>
+      <c r="I70" s="105"/>
+      <c r="J70" s="90"/>
       <c r="L70" s="99"/>
-      <c r="M70" s="126"/>
-      <c r="N70" s="126"/>
+      <c r="M70" s="102"/>
+      <c r="N70" s="102"/>
       <c r="O70" s="99"/>
-      <c r="Q70" s="132"/>
-      <c r="R70" s="132"/>
-      <c r="S70" s="132"/>
+      <c r="Q70" s="108"/>
+      <c r="R70" s="108"/>
+      <c r="S70" s="108"/>
     </row>
     <row r="71" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D71" s="120"/>
-      <c r="E71" s="123"/>
-      <c r="G71" s="117"/>
-      <c r="H71" s="129"/>
-      <c r="I71" s="129"/>
-      <c r="J71" s="117"/>
+      <c r="D71" s="93"/>
+      <c r="E71" s="96"/>
+      <c r="G71" s="90"/>
+      <c r="H71" s="105"/>
+      <c r="I71" s="105"/>
+      <c r="J71" s="90"/>
       <c r="L71" s="99"/>
-      <c r="M71" s="126"/>
-      <c r="N71" s="126"/>
+      <c r="M71" s="102"/>
+      <c r="N71" s="102"/>
       <c r="O71" s="99"/>
-      <c r="Q71" s="132"/>
-      <c r="R71" s="132"/>
-      <c r="S71" s="132"/>
+      <c r="Q71" s="108"/>
+      <c r="R71" s="108"/>
+      <c r="S71" s="108"/>
     </row>
     <row r="72" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D72" s="120"/>
-      <c r="E72" s="123"/>
-      <c r="G72" s="117"/>
-      <c r="H72" s="129"/>
-      <c r="I72" s="129"/>
-      <c r="J72" s="117"/>
+      <c r="D72" s="93"/>
+      <c r="E72" s="96"/>
+      <c r="G72" s="90"/>
+      <c r="H72" s="105"/>
+      <c r="I72" s="105"/>
+      <c r="J72" s="90"/>
       <c r="L72" s="99"/>
-      <c r="M72" s="126"/>
-      <c r="N72" s="126"/>
+      <c r="M72" s="102"/>
+      <c r="N72" s="102"/>
       <c r="O72" s="99"/>
-      <c r="Q72" s="132"/>
-      <c r="R72" s="132"/>
-      <c r="S72" s="132"/>
+      <c r="Q72" s="108"/>
+      <c r="R72" s="108"/>
+      <c r="S72" s="108"/>
     </row>
     <row r="73" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D73" s="120"/>
-      <c r="E73" s="123"/>
-      <c r="G73" s="117"/>
-      <c r="H73" s="129"/>
-      <c r="I73" s="129"/>
-      <c r="J73" s="117"/>
+      <c r="D73" s="93"/>
+      <c r="E73" s="96"/>
+      <c r="G73" s="90"/>
+      <c r="H73" s="105"/>
+      <c r="I73" s="105"/>
+      <c r="J73" s="90"/>
       <c r="L73" s="99"/>
-      <c r="M73" s="126"/>
-      <c r="N73" s="126"/>
+      <c r="M73" s="102"/>
+      <c r="N73" s="102"/>
       <c r="O73" s="99"/>
-      <c r="Q73" s="132"/>
-      <c r="R73" s="132"/>
-      <c r="S73" s="132"/>
+      <c r="Q73" s="108"/>
+      <c r="R73" s="108"/>
+      <c r="S73" s="108"/>
     </row>
     <row r="74" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D74" s="120"/>
-      <c r="E74" s="123"/>
-      <c r="G74" s="117"/>
-      <c r="H74" s="129"/>
-      <c r="I74" s="129"/>
-      <c r="J74" s="117"/>
+      <c r="D74" s="93"/>
+      <c r="E74" s="96"/>
+      <c r="G74" s="90"/>
+      <c r="H74" s="105"/>
+      <c r="I74" s="105"/>
+      <c r="J74" s="90"/>
       <c r="L74" s="99"/>
-      <c r="M74" s="126"/>
-      <c r="N74" s="126"/>
+      <c r="M74" s="102"/>
+      <c r="N74" s="102"/>
       <c r="O74" s="99"/>
-      <c r="Q74" s="132"/>
-      <c r="R74" s="132"/>
-      <c r="S74" s="132"/>
+      <c r="Q74" s="108"/>
+      <c r="R74" s="108"/>
+      <c r="S74" s="108"/>
     </row>
     <row r="75" spans="1:20" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D75" s="121"/>
-      <c r="E75" s="124"/>
-      <c r="G75" s="118"/>
-      <c r="H75" s="130"/>
-      <c r="I75" s="130"/>
-      <c r="J75" s="118"/>
+      <c r="D75" s="94"/>
+      <c r="E75" s="97"/>
+      <c r="G75" s="91"/>
+      <c r="H75" s="106"/>
+      <c r="I75" s="106"/>
+      <c r="J75" s="91"/>
       <c r="L75" s="100"/>
-      <c r="M75" s="127"/>
-      <c r="N75" s="127"/>
+      <c r="M75" s="103"/>
+      <c r="N75" s="103"/>
       <c r="O75" s="100"/>
-      <c r="Q75" s="133"/>
-      <c r="R75" s="133"/>
-      <c r="S75" s="133"/>
+      <c r="Q75" s="109"/>
+      <c r="R75" s="109"/>
+      <c r="S75" s="109"/>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B6:T60">
     <sortCondition ref="B6"/>
   </sortState>
   <mergeCells count="25">
+    <mergeCell ref="G2:K2"/>
+    <mergeCell ref="D2:F2"/>
+    <mergeCell ref="Q3:T4"/>
+    <mergeCell ref="O66:O75"/>
+    <mergeCell ref="A2:A5"/>
+    <mergeCell ref="G3:K4"/>
+    <mergeCell ref="D3:F4"/>
+    <mergeCell ref="B2:B5"/>
+    <mergeCell ref="C2:C5"/>
     <mergeCell ref="B1:T1"/>
     <mergeCell ref="J66:J75"/>
     <mergeCell ref="D66:D75"/>
@@ -7630,15 +7670,6 @@
     <mergeCell ref="I66:I75"/>
     <mergeCell ref="Q2:T2"/>
     <mergeCell ref="L2:P2"/>
-    <mergeCell ref="G2:K2"/>
-    <mergeCell ref="D2:F2"/>
-    <mergeCell ref="Q3:T4"/>
-    <mergeCell ref="O66:O75"/>
-    <mergeCell ref="A2:A5"/>
-    <mergeCell ref="G3:K4"/>
-    <mergeCell ref="D3:F4"/>
-    <mergeCell ref="B2:B5"/>
-    <mergeCell ref="C2:C5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
llamada a participar lista
</commit_message>
<xml_diff>
--- a/9_asistencia_evaluacion/pivu_caucasia_notas_quices_asistencia.xlsx
+++ b/9_asistencia_evaluacion/pivu_caucasia_notas_quices_asistencia.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marco\Documentos\extension\camino-udea\9_asistencia_evaluacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C25B41B2-1453-4561-84C4-CCD8E192695B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CB8F5E9-1628-4181-9D54-A2A9C501AB55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="107">
   <si>
     <t>METODOLOGÍA DE ESTUDIO</t>
   </si>
@@ -357,6 +357,9 @@
   </si>
   <si>
     <t>yeniferaguirrecarvajal2008@gmail.com</t>
+  </si>
+  <si>
+    <t>mariallno0716@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -994,6 +997,16 @@
     </xf>
     <xf numFmtId="0" fontId="23" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="22" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="19" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1096,11 +1109,83 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1132,15 +1217,6 @@
     <xf numFmtId="0" fontId="7" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
@@ -1186,79 +1262,6 @@
     <xf numFmtId="0" fontId="3" fillId="9" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="2" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Hipervínculo" xfId="2" builtinId="8"/>
@@ -1756,28 +1759,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="72" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="87" t="s">
+      <c r="A1" s="55" t="s">
         <v>27</v>
       </c>
-      <c r="B1" s="86"/>
-      <c r="C1" s="86"/>
-      <c r="D1" s="86"/>
-      <c r="E1" s="86"/>
-      <c r="F1" s="86"/>
-      <c r="G1" s="86"/>
-      <c r="H1" s="86"/>
+      <c r="B1" s="54"/>
+      <c r="C1" s="54"/>
+      <c r="D1" s="54"/>
+      <c r="E1" s="54"/>
+      <c r="F1" s="54"/>
+      <c r="G1" s="54"/>
+      <c r="H1" s="54"/>
     </row>
     <row r="2" spans="1:9" ht="19.8" x14ac:dyDescent="0.3">
-      <c r="A2" s="86" t="s">
+      <c r="A2" s="54" t="s">
         <v>26</v>
       </c>
-      <c r="B2" s="86"/>
-      <c r="C2" s="86"/>
-      <c r="D2" s="86"/>
-      <c r="E2" s="86"/>
-      <c r="F2" s="86"/>
-      <c r="G2" s="86"/>
-      <c r="H2" s="86"/>
+      <c r="B2" s="54"/>
+      <c r="C2" s="54"/>
+      <c r="D2" s="54"/>
+      <c r="E2" s="54"/>
+      <c r="F2" s="54"/>
+      <c r="G2" s="54"/>
+      <c r="H2" s="54"/>
       <c r="I2" s="51" t="s">
         <v>102</v>
       </c>
@@ -1950,7 +1953,7 @@
       <c r="F9" s="44">
         <v>3203519315</v>
       </c>
-      <c r="G9" s="140" t="s">
+      <c r="G9" s="53" t="s">
         <v>95</v>
       </c>
       <c r="H9" s="50" t="s">
@@ -2048,7 +2051,7 @@
       <c r="F13" s="44">
         <v>3136630762</v>
       </c>
-      <c r="G13" s="140" t="s">
+      <c r="G13" s="53" t="s">
         <v>98</v>
       </c>
       <c r="H13" s="50" t="s">
@@ -2194,7 +2197,7 @@
       <c r="F19" s="44">
         <v>3218798123</v>
       </c>
-      <c r="G19" s="140" t="s">
+      <c r="G19" s="53" t="s">
         <v>104</v>
       </c>
       <c r="H19" s="50" t="s">
@@ -2268,7 +2271,9 @@
       <c r="F22" s="44">
         <v>3145134544</v>
       </c>
-      <c r="G22" s="44"/>
+      <c r="G22" s="53" t="s">
+        <v>106</v>
+      </c>
       <c r="H22" s="50" t="s">
         <v>100</v>
       </c>
@@ -2652,7 +2657,7 @@
       <c r="F38" s="44">
         <v>3212234096</v>
       </c>
-      <c r="G38" s="140" t="s">
+      <c r="G38" s="53" t="s">
         <v>105</v>
       </c>
       <c r="H38" s="44"/>
@@ -2676,10 +2681,11 @@
     <hyperlink ref="G19" r:id="rId2" xr:uid="{0D63D482-2B15-4CBD-8A6E-32A20A7492DB}"/>
     <hyperlink ref="G38" r:id="rId3" xr:uid="{F41688A5-1CDE-42E7-9CB3-E623ADE29950}"/>
     <hyperlink ref="G13" r:id="rId4" xr:uid="{5EC44252-B9A4-45C6-9F57-A5A815D8FC04}"/>
+    <hyperlink ref="G22" r:id="rId5" xr:uid="{05E3B9BD-D2ED-4CAA-BA6F-0462EAED9919}"/>
   </hyperlinks>
   <pageMargins left="0.19685039370078741" right="0.19685039370078741" top="0.19685039370078741" bottom="0.19685039370078741" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup scale="80" orientation="landscape" r:id="rId5"/>
-  <drawing r:id="rId6"/>
+  <pageSetup scale="80" orientation="landscape" r:id="rId6"/>
+  <drawing r:id="rId7"/>
 </worksheet>
 </file>
 
@@ -2701,172 +2707,172 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:31" ht="66" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B1" s="59" t="s">
+      <c r="B1" s="63" t="s">
         <v>18</v>
       </c>
-      <c r="C1" s="59"/>
-      <c r="D1" s="59"/>
-      <c r="E1" s="59"/>
-      <c r="F1" s="59"/>
-      <c r="G1" s="59"/>
-      <c r="H1" s="59"/>
-      <c r="I1" s="59"/>
-      <c r="J1" s="59"/>
-      <c r="K1" s="59"/>
-      <c r="L1" s="59"/>
-      <c r="M1" s="59"/>
-      <c r="N1" s="59"/>
-      <c r="O1" s="59"/>
-      <c r="P1" s="59"/>
-      <c r="Q1" s="59"/>
-      <c r="R1" s="59"/>
-      <c r="S1" s="59"/>
-      <c r="T1" s="59"/>
-      <c r="U1" s="59"/>
-      <c r="V1" s="59"/>
-      <c r="W1" s="59"/>
-      <c r="X1" s="59"/>
-      <c r="Y1" s="59"/>
-      <c r="Z1" s="59"/>
-      <c r="AA1" s="59"/>
-      <c r="AB1" s="59"/>
-      <c r="AC1" s="59"/>
-      <c r="AD1" s="59"/>
-      <c r="AE1" s="59"/>
+      <c r="C1" s="63"/>
+      <c r="D1" s="63"/>
+      <c r="E1" s="63"/>
+      <c r="F1" s="63"/>
+      <c r="G1" s="63"/>
+      <c r="H1" s="63"/>
+      <c r="I1" s="63"/>
+      <c r="J1" s="63"/>
+      <c r="K1" s="63"/>
+      <c r="L1" s="63"/>
+      <c r="M1" s="63"/>
+      <c r="N1" s="63"/>
+      <c r="O1" s="63"/>
+      <c r="P1" s="63"/>
+      <c r="Q1" s="63"/>
+      <c r="R1" s="63"/>
+      <c r="S1" s="63"/>
+      <c r="T1" s="63"/>
+      <c r="U1" s="63"/>
+      <c r="V1" s="63"/>
+      <c r="W1" s="63"/>
+      <c r="X1" s="63"/>
+      <c r="Y1" s="63"/>
+      <c r="Z1" s="63"/>
+      <c r="AA1" s="63"/>
+      <c r="AB1" s="63"/>
+      <c r="AC1" s="63"/>
+      <c r="AD1" s="63"/>
+      <c r="AE1" s="63"/>
     </row>
     <row r="2" spans="1:31" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="60" t="s">
+      <c r="A2" s="64" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="84" t="s">
+      <c r="B2" s="88" t="s">
         <v>21</v>
       </c>
-      <c r="C2" s="60" t="s">
+      <c r="C2" s="64" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="77" t="s">
+      <c r="D2" s="81" t="s">
         <v>19</v>
       </c>
-      <c r="E2" s="78"/>
-      <c r="F2" s="78"/>
-      <c r="G2" s="78"/>
-      <c r="H2" s="79"/>
-      <c r="I2" s="62" t="s">
+      <c r="E2" s="82"/>
+      <c r="F2" s="82"/>
+      <c r="G2" s="82"/>
+      <c r="H2" s="83"/>
+      <c r="I2" s="66" t="s">
         <v>19</v>
       </c>
-      <c r="J2" s="63"/>
-      <c r="K2" s="63"/>
-      <c r="L2" s="63"/>
-      <c r="M2" s="63"/>
-      <c r="N2" s="63"/>
-      <c r="O2" s="63"/>
-      <c r="P2" s="63"/>
-      <c r="Q2" s="64"/>
-      <c r="R2" s="71" t="s">
+      <c r="J2" s="67"/>
+      <c r="K2" s="67"/>
+      <c r="L2" s="67"/>
+      <c r="M2" s="67"/>
+      <c r="N2" s="67"/>
+      <c r="O2" s="67"/>
+      <c r="P2" s="67"/>
+      <c r="Q2" s="68"/>
+      <c r="R2" s="75" t="s">
         <v>19</v>
       </c>
-      <c r="S2" s="72"/>
-      <c r="T2" s="72"/>
-      <c r="U2" s="72"/>
-      <c r="V2" s="72"/>
-      <c r="W2" s="72"/>
-      <c r="X2" s="72"/>
-      <c r="Y2" s="72"/>
-      <c r="Z2" s="73"/>
-      <c r="AA2" s="52" t="s">
+      <c r="S2" s="76"/>
+      <c r="T2" s="76"/>
+      <c r="U2" s="76"/>
+      <c r="V2" s="76"/>
+      <c r="W2" s="76"/>
+      <c r="X2" s="76"/>
+      <c r="Y2" s="76"/>
+      <c r="Z2" s="77"/>
+      <c r="AA2" s="56" t="s">
         <v>19</v>
       </c>
-      <c r="AB2" s="53"/>
-      <c r="AC2" s="53"/>
-      <c r="AD2" s="53"/>
-      <c r="AE2" s="54"/>
+      <c r="AB2" s="57"/>
+      <c r="AC2" s="57"/>
+      <c r="AD2" s="57"/>
+      <c r="AE2" s="58"/>
     </row>
     <row r="3" spans="1:31" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="61"/>
-      <c r="B3" s="85"/>
-      <c r="C3" s="61"/>
-      <c r="D3" s="80" t="s">
+      <c r="A3" s="65"/>
+      <c r="B3" s="89"/>
+      <c r="C3" s="65"/>
+      <c r="D3" s="84" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="81"/>
-      <c r="F3" s="81"/>
-      <c r="G3" s="81"/>
-      <c r="H3" s="82"/>
-      <c r="I3" s="65" t="s">
+      <c r="E3" s="85"/>
+      <c r="F3" s="85"/>
+      <c r="G3" s="85"/>
+      <c r="H3" s="86"/>
+      <c r="I3" s="69" t="s">
         <v>2</v>
       </c>
-      <c r="J3" s="66"/>
-      <c r="K3" s="66"/>
-      <c r="L3" s="66"/>
-      <c r="M3" s="66"/>
-      <c r="N3" s="66"/>
-      <c r="O3" s="66"/>
-      <c r="P3" s="66"/>
-      <c r="Q3" s="67"/>
-      <c r="R3" s="74" t="s">
+      <c r="J3" s="70"/>
+      <c r="K3" s="70"/>
+      <c r="L3" s="70"/>
+      <c r="M3" s="70"/>
+      <c r="N3" s="70"/>
+      <c r="O3" s="70"/>
+      <c r="P3" s="70"/>
+      <c r="Q3" s="71"/>
+      <c r="R3" s="78" t="s">
         <v>1</v>
       </c>
-      <c r="S3" s="75"/>
-      <c r="T3" s="75"/>
-      <c r="U3" s="75"/>
-      <c r="V3" s="75"/>
-      <c r="W3" s="75"/>
-      <c r="X3" s="75"/>
-      <c r="Y3" s="75"/>
-      <c r="Z3" s="76"/>
-      <c r="AA3" s="55" t="s">
-        <v>0</v>
-      </c>
-      <c r="AB3" s="56"/>
-      <c r="AC3" s="56"/>
-      <c r="AD3" s="56"/>
-      <c r="AE3" s="57"/>
+      <c r="S3" s="79"/>
+      <c r="T3" s="79"/>
+      <c r="U3" s="79"/>
+      <c r="V3" s="79"/>
+      <c r="W3" s="79"/>
+      <c r="X3" s="79"/>
+      <c r="Y3" s="79"/>
+      <c r="Z3" s="80"/>
+      <c r="AA3" s="59" t="s">
+        <v>0</v>
+      </c>
+      <c r="AB3" s="60"/>
+      <c r="AC3" s="60"/>
+      <c r="AD3" s="60"/>
+      <c r="AE3" s="61"/>
     </row>
     <row r="4" spans="1:31" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="61"/>
-      <c r="B4" s="85"/>
-      <c r="C4" s="61"/>
-      <c r="D4" s="83" t="s">
+      <c r="A4" s="65"/>
+      <c r="B4" s="89"/>
+      <c r="C4" s="65"/>
+      <c r="D4" s="87" t="s">
         <v>22</v>
       </c>
-      <c r="E4" s="69"/>
-      <c r="F4" s="69"/>
-      <c r="G4" s="70"/>
+      <c r="E4" s="73"/>
+      <c r="F4" s="73"/>
+      <c r="G4" s="74"/>
       <c r="H4" s="1"/>
-      <c r="I4" s="68" t="s">
+      <c r="I4" s="72" t="s">
         <v>23</v>
       </c>
-      <c r="J4" s="69"/>
-      <c r="K4" s="69"/>
-      <c r="L4" s="69"/>
-      <c r="M4" s="69"/>
-      <c r="N4" s="69"/>
-      <c r="O4" s="69"/>
-      <c r="P4" s="70"/>
+      <c r="J4" s="73"/>
+      <c r="K4" s="73"/>
+      <c r="L4" s="73"/>
+      <c r="M4" s="73"/>
+      <c r="N4" s="73"/>
+      <c r="O4" s="73"/>
+      <c r="P4" s="74"/>
       <c r="Q4" s="3"/>
-      <c r="R4" s="68" t="s">
+      <c r="R4" s="72" t="s">
         <v>23</v>
       </c>
-      <c r="S4" s="69"/>
-      <c r="T4" s="69"/>
-      <c r="U4" s="69"/>
-      <c r="V4" s="69"/>
-      <c r="W4" s="69"/>
-      <c r="X4" s="69"/>
-      <c r="Y4" s="70"/>
+      <c r="S4" s="73"/>
+      <c r="T4" s="73"/>
+      <c r="U4" s="73"/>
+      <c r="V4" s="73"/>
+      <c r="W4" s="73"/>
+      <c r="X4" s="73"/>
+      <c r="Y4" s="74"/>
       <c r="Z4" s="12"/>
-      <c r="AA4" s="58" t="s">
+      <c r="AA4" s="62" t="s">
         <v>23</v>
       </c>
-      <c r="AB4" s="58"/>
-      <c r="AC4" s="58"/>
-      <c r="AD4" s="58"/>
+      <c r="AB4" s="62"/>
+      <c r="AC4" s="62"/>
+      <c r="AD4" s="62"/>
       <c r="AE4" s="3"/>
     </row>
     <row r="5" spans="1:31" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="61"/>
-      <c r="B5" s="85"/>
-      <c r="C5" s="61"/>
+      <c r="A5" s="65"/>
+      <c r="B5" s="89"/>
+      <c r="C5" s="65"/>
       <c r="D5" s="28" t="s">
         <v>103</v>
       </c>
@@ -2918,13 +2924,15 @@
         <f>+Inscritos!D4</f>
         <v>1038110235</v>
       </c>
-      <c r="D6" s="13"/>
+      <c r="D6" s="13">
+        <v>1</v>
+      </c>
       <c r="E6" s="13"/>
       <c r="F6" s="13"/>
       <c r="G6" s="13"/>
       <c r="H6" s="32">
         <f>+SUM(D6:G6)/4</f>
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="I6" s="33"/>
       <c r="J6" s="33"/>
@@ -3185,13 +3193,15 @@
         <f>+Inscritos!D9</f>
         <v>1038110143</v>
       </c>
-      <c r="D11" s="13"/>
+      <c r="D11" s="13">
+        <v>1</v>
+      </c>
       <c r="E11" s="13"/>
       <c r="F11" s="13"/>
       <c r="G11" s="13"/>
       <c r="H11" s="32">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="I11" s="33"/>
       <c r="J11" s="33"/>
@@ -3344,13 +3354,15 @@
         <f>+Inscritos!D12</f>
         <v>1038111245</v>
       </c>
-      <c r="D14" s="13"/>
+      <c r="D14" s="13">
+        <v>1</v>
+      </c>
       <c r="E14" s="13"/>
       <c r="F14" s="13"/>
       <c r="G14" s="13"/>
       <c r="H14" s="32">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="I14" s="33"/>
       <c r="J14" s="33"/>
@@ -4194,13 +4206,15 @@
         <f>+Inscritos!D28</f>
         <v>1038115449</v>
       </c>
-      <c r="D30" s="13"/>
+      <c r="D30" s="13">
+        <v>1</v>
+      </c>
       <c r="E30" s="13"/>
       <c r="F30" s="13"/>
       <c r="G30" s="13"/>
       <c r="H30" s="32">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="I30" s="33"/>
       <c r="J30" s="33"/>
@@ -4301,14 +4315,14 @@
         <v>1038104210</v>
       </c>
       <c r="D32" s="13">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E32" s="13"/>
       <c r="F32" s="13"/>
       <c r="G32" s="13"/>
       <c r="H32" s="32">
         <f t="shared" si="0"/>
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="I32" s="33"/>
       <c r="J32" s="33"/>
@@ -4719,7 +4733,7 @@
       </c>
     </row>
     <row r="40" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A40" s="139">
+      <c r="A40" s="52">
         <v>35</v>
       </c>
     </row>
@@ -4775,123 +4789,123 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="72.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B1" s="88" t="s">
+      <c r="B1" s="116" t="s">
         <v>18</v>
       </c>
-      <c r="C1" s="88"/>
-      <c r="D1" s="88"/>
-      <c r="E1" s="88"/>
-      <c r="F1" s="88"/>
-      <c r="G1" s="88"/>
-      <c r="H1" s="88"/>
-      <c r="I1" s="88"/>
-      <c r="J1" s="88"/>
-      <c r="K1" s="88"/>
-      <c r="L1" s="88"/>
-      <c r="M1" s="88"/>
-      <c r="N1" s="88"/>
-      <c r="O1" s="88"/>
-      <c r="P1" s="88"/>
-      <c r="Q1" s="88"/>
-      <c r="R1" s="88"/>
-      <c r="S1" s="88"/>
-      <c r="T1" s="88"/>
+      <c r="C1" s="116"/>
+      <c r="D1" s="116"/>
+      <c r="E1" s="116"/>
+      <c r="F1" s="116"/>
+      <c r="G1" s="116"/>
+      <c r="H1" s="116"/>
+      <c r="I1" s="116"/>
+      <c r="J1" s="116"/>
+      <c r="K1" s="116"/>
+      <c r="L1" s="116"/>
+      <c r="M1" s="116"/>
+      <c r="N1" s="116"/>
+      <c r="O1" s="116"/>
+      <c r="P1" s="116"/>
+      <c r="Q1" s="116"/>
+      <c r="R1" s="116"/>
+      <c r="S1" s="116"/>
+      <c r="T1" s="116"/>
     </row>
     <row r="2" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="125" t="s">
+      <c r="A2" s="102" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="84" t="s">
+      <c r="B2" s="88" t="s">
         <v>21</v>
       </c>
-      <c r="C2" s="60" t="s">
+      <c r="C2" s="64" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="116" t="str">
+      <c r="D2" s="90" t="str">
         <f>Asistencia!D2</f>
         <v>NOMBRE DOCENTE</v>
       </c>
-      <c r="E2" s="117"/>
-      <c r="F2" s="118"/>
-      <c r="G2" s="116" t="str">
+      <c r="E2" s="91"/>
+      <c r="F2" s="92"/>
+      <c r="G2" s="90" t="str">
         <f>Asistencia!I2</f>
         <v>NOMBRE DOCENTE</v>
       </c>
-      <c r="H2" s="117"/>
-      <c r="I2" s="117"/>
-      <c r="J2" s="117"/>
-      <c r="K2" s="118"/>
-      <c r="L2" s="116" t="s">
+      <c r="H2" s="91"/>
+      <c r="I2" s="91"/>
+      <c r="J2" s="91"/>
+      <c r="K2" s="92"/>
+      <c r="L2" s="90" t="s">
         <v>19</v>
       </c>
-      <c r="M2" s="117"/>
-      <c r="N2" s="117"/>
-      <c r="O2" s="117"/>
-      <c r="P2" s="118"/>
-      <c r="Q2" s="116" t="str">
+      <c r="M2" s="91"/>
+      <c r="N2" s="91"/>
+      <c r="O2" s="91"/>
+      <c r="P2" s="92"/>
+      <c r="Q2" s="90" t="str">
         <f>Asistencia!AA2</f>
         <v>NOMBRE DOCENTE</v>
       </c>
-      <c r="R2" s="117"/>
-      <c r="S2" s="117"/>
-      <c r="T2" s="118"/>
+      <c r="R2" s="91"/>
+      <c r="S2" s="91"/>
+      <c r="T2" s="92"/>
     </row>
     <row r="3" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="126"/>
-      <c r="B3" s="85"/>
-      <c r="C3" s="61"/>
-      <c r="D3" s="133" t="s">
+      <c r="A3" s="103"/>
+      <c r="B3" s="89"/>
+      <c r="C3" s="65"/>
+      <c r="D3" s="110" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="134"/>
-      <c r="F3" s="135"/>
-      <c r="G3" s="127" t="s">
+      <c r="E3" s="111"/>
+      <c r="F3" s="112"/>
+      <c r="G3" s="104" t="s">
         <v>2</v>
       </c>
-      <c r="H3" s="128"/>
-      <c r="I3" s="128"/>
-      <c r="J3" s="128"/>
-      <c r="K3" s="129"/>
-      <c r="L3" s="110" t="s">
+      <c r="H3" s="105"/>
+      <c r="I3" s="105"/>
+      <c r="J3" s="105"/>
+      <c r="K3" s="106"/>
+      <c r="L3" s="135" t="s">
         <v>1</v>
       </c>
-      <c r="M3" s="111"/>
-      <c r="N3" s="111"/>
-      <c r="O3" s="111"/>
-      <c r="P3" s="112"/>
-      <c r="Q3" s="119" t="s">
-        <v>0</v>
-      </c>
-      <c r="R3" s="120"/>
-      <c r="S3" s="120"/>
-      <c r="T3" s="121"/>
+      <c r="M3" s="136"/>
+      <c r="N3" s="136"/>
+      <c r="O3" s="136"/>
+      <c r="P3" s="137"/>
+      <c r="Q3" s="93" t="s">
+        <v>0</v>
+      </c>
+      <c r="R3" s="94"/>
+      <c r="S3" s="94"/>
+      <c r="T3" s="95"/>
     </row>
     <row r="4" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="126"/>
-      <c r="B4" s="85"/>
-      <c r="C4" s="61"/>
-      <c r="D4" s="136"/>
-      <c r="E4" s="137"/>
-      <c r="F4" s="138"/>
-      <c r="G4" s="130"/>
-      <c r="H4" s="131"/>
-      <c r="I4" s="131"/>
-      <c r="J4" s="131"/>
-      <c r="K4" s="132"/>
-      <c r="L4" s="113"/>
-      <c r="M4" s="114"/>
-      <c r="N4" s="114"/>
-      <c r="O4" s="114"/>
-      <c r="P4" s="115"/>
-      <c r="Q4" s="122"/>
-      <c r="R4" s="123"/>
-      <c r="S4" s="123"/>
-      <c r="T4" s="124"/>
+      <c r="A4" s="103"/>
+      <c r="B4" s="89"/>
+      <c r="C4" s="65"/>
+      <c r="D4" s="113"/>
+      <c r="E4" s="114"/>
+      <c r="F4" s="115"/>
+      <c r="G4" s="107"/>
+      <c r="H4" s="108"/>
+      <c r="I4" s="108"/>
+      <c r="J4" s="108"/>
+      <c r="K4" s="109"/>
+      <c r="L4" s="138"/>
+      <c r="M4" s="139"/>
+      <c r="N4" s="139"/>
+      <c r="O4" s="139"/>
+      <c r="P4" s="140"/>
+      <c r="Q4" s="96"/>
+      <c r="R4" s="97"/>
+      <c r="S4" s="97"/>
+      <c r="T4" s="98"/>
     </row>
     <row r="5" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="126"/>
-      <c r="B5" s="85"/>
-      <c r="C5" s="61"/>
+      <c r="A5" s="103"/>
+      <c r="B5" s="89"/>
+      <c r="C5" s="65"/>
       <c r="D5" s="17">
         <v>0.75</v>
       </c>
@@ -7465,195 +7479,186 @@
       </c>
     </row>
     <row r="66" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D66" s="92" t="s">
+      <c r="D66" s="120" t="s">
         <v>24</v>
       </c>
-      <c r="E66" s="95" t="s">
+      <c r="E66" s="123" t="s">
         <v>12</v>
       </c>
-      <c r="G66" s="89" t="s">
+      <c r="G66" s="117" t="s">
         <v>8</v>
       </c>
-      <c r="H66" s="104" t="s">
+      <c r="H66" s="129" t="s">
         <v>9</v>
       </c>
-      <c r="I66" s="104" t="s">
+      <c r="I66" s="129" t="s">
         <v>10</v>
       </c>
-      <c r="J66" s="89" t="s">
+      <c r="J66" s="117" t="s">
         <v>11</v>
       </c>
-      <c r="L66" s="98" t="s">
+      <c r="L66" s="99" t="s">
         <v>8</v>
       </c>
-      <c r="M66" s="101" t="s">
+      <c r="M66" s="126" t="s">
         <v>9</v>
       </c>
-      <c r="N66" s="101" t="s">
+      <c r="N66" s="126" t="s">
         <v>10</v>
       </c>
-      <c r="O66" s="98" t="s">
+      <c r="O66" s="99" t="s">
         <v>11</v>
       </c>
-      <c r="Q66" s="107" t="s">
+      <c r="Q66" s="132" t="s">
         <v>24</v>
       </c>
-      <c r="R66" s="107" t="s">
+      <c r="R66" s="132" t="s">
         <v>4</v>
       </c>
-      <c r="S66" s="107" t="s">
+      <c r="S66" s="132" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="67" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D67" s="93"/>
-      <c r="E67" s="96"/>
-      <c r="G67" s="90"/>
-      <c r="H67" s="105"/>
-      <c r="I67" s="105"/>
-      <c r="J67" s="90"/>
-      <c r="L67" s="99"/>
-      <c r="M67" s="102"/>
-      <c r="N67" s="102"/>
-      <c r="O67" s="99"/>
-      <c r="Q67" s="108"/>
-      <c r="R67" s="108"/>
-      <c r="S67" s="108"/>
+      <c r="D67" s="121"/>
+      <c r="E67" s="124"/>
+      <c r="G67" s="118"/>
+      <c r="H67" s="130"/>
+      <c r="I67" s="130"/>
+      <c r="J67" s="118"/>
+      <c r="L67" s="100"/>
+      <c r="M67" s="127"/>
+      <c r="N67" s="127"/>
+      <c r="O67" s="100"/>
+      <c r="Q67" s="133"/>
+      <c r="R67" s="133"/>
+      <c r="S67" s="133"/>
     </row>
     <row r="68" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D68" s="93"/>
-      <c r="E68" s="96"/>
-      <c r="G68" s="90"/>
-      <c r="H68" s="105"/>
-      <c r="I68" s="105"/>
-      <c r="J68" s="90"/>
-      <c r="L68" s="99"/>
-      <c r="M68" s="102"/>
-      <c r="N68" s="102"/>
-      <c r="O68" s="99"/>
-      <c r="Q68" s="108"/>
-      <c r="R68" s="108"/>
-      <c r="S68" s="108"/>
+      <c r="D68" s="121"/>
+      <c r="E68" s="124"/>
+      <c r="G68" s="118"/>
+      <c r="H68" s="130"/>
+      <c r="I68" s="130"/>
+      <c r="J68" s="118"/>
+      <c r="L68" s="100"/>
+      <c r="M68" s="127"/>
+      <c r="N68" s="127"/>
+      <c r="O68" s="100"/>
+      <c r="Q68" s="133"/>
+      <c r="R68" s="133"/>
+      <c r="S68" s="133"/>
     </row>
     <row r="69" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D69" s="93"/>
-      <c r="E69" s="96"/>
-      <c r="G69" s="90"/>
-      <c r="H69" s="105"/>
-      <c r="I69" s="105"/>
-      <c r="J69" s="90"/>
-      <c r="L69" s="99"/>
-      <c r="M69" s="102"/>
-      <c r="N69" s="102"/>
-      <c r="O69" s="99"/>
-      <c r="Q69" s="108"/>
-      <c r="R69" s="108"/>
-      <c r="S69" s="108"/>
+      <c r="D69" s="121"/>
+      <c r="E69" s="124"/>
+      <c r="G69" s="118"/>
+      <c r="H69" s="130"/>
+      <c r="I69" s="130"/>
+      <c r="J69" s="118"/>
+      <c r="L69" s="100"/>
+      <c r="M69" s="127"/>
+      <c r="N69" s="127"/>
+      <c r="O69" s="100"/>
+      <c r="Q69" s="133"/>
+      <c r="R69" s="133"/>
+      <c r="S69" s="133"/>
     </row>
     <row r="70" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D70" s="93"/>
-      <c r="E70" s="96"/>
-      <c r="G70" s="90"/>
-      <c r="H70" s="105"/>
-      <c r="I70" s="105"/>
-      <c r="J70" s="90"/>
-      <c r="L70" s="99"/>
-      <c r="M70" s="102"/>
-      <c r="N70" s="102"/>
-      <c r="O70" s="99"/>
-      <c r="Q70" s="108"/>
-      <c r="R70" s="108"/>
-      <c r="S70" s="108"/>
+      <c r="D70" s="121"/>
+      <c r="E70" s="124"/>
+      <c r="G70" s="118"/>
+      <c r="H70" s="130"/>
+      <c r="I70" s="130"/>
+      <c r="J70" s="118"/>
+      <c r="L70" s="100"/>
+      <c r="M70" s="127"/>
+      <c r="N70" s="127"/>
+      <c r="O70" s="100"/>
+      <c r="Q70" s="133"/>
+      <c r="R70" s="133"/>
+      <c r="S70" s="133"/>
     </row>
     <row r="71" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D71" s="93"/>
-      <c r="E71" s="96"/>
-      <c r="G71" s="90"/>
-      <c r="H71" s="105"/>
-      <c r="I71" s="105"/>
-      <c r="J71" s="90"/>
-      <c r="L71" s="99"/>
-      <c r="M71" s="102"/>
-      <c r="N71" s="102"/>
-      <c r="O71" s="99"/>
-      <c r="Q71" s="108"/>
-      <c r="R71" s="108"/>
-      <c r="S71" s="108"/>
+      <c r="D71" s="121"/>
+      <c r="E71" s="124"/>
+      <c r="G71" s="118"/>
+      <c r="H71" s="130"/>
+      <c r="I71" s="130"/>
+      <c r="J71" s="118"/>
+      <c r="L71" s="100"/>
+      <c r="M71" s="127"/>
+      <c r="N71" s="127"/>
+      <c r="O71" s="100"/>
+      <c r="Q71" s="133"/>
+      <c r="R71" s="133"/>
+      <c r="S71" s="133"/>
     </row>
     <row r="72" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D72" s="93"/>
-      <c r="E72" s="96"/>
-      <c r="G72" s="90"/>
-      <c r="H72" s="105"/>
-      <c r="I72" s="105"/>
-      <c r="J72" s="90"/>
-      <c r="L72" s="99"/>
-      <c r="M72" s="102"/>
-      <c r="N72" s="102"/>
-      <c r="O72" s="99"/>
-      <c r="Q72" s="108"/>
-      <c r="R72" s="108"/>
-      <c r="S72" s="108"/>
+      <c r="D72" s="121"/>
+      <c r="E72" s="124"/>
+      <c r="G72" s="118"/>
+      <c r="H72" s="130"/>
+      <c r="I72" s="130"/>
+      <c r="J72" s="118"/>
+      <c r="L72" s="100"/>
+      <c r="M72" s="127"/>
+      <c r="N72" s="127"/>
+      <c r="O72" s="100"/>
+      <c r="Q72" s="133"/>
+      <c r="R72" s="133"/>
+      <c r="S72" s="133"/>
     </row>
     <row r="73" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D73" s="93"/>
-      <c r="E73" s="96"/>
-      <c r="G73" s="90"/>
-      <c r="H73" s="105"/>
-      <c r="I73" s="105"/>
-      <c r="J73" s="90"/>
-      <c r="L73" s="99"/>
-      <c r="M73" s="102"/>
-      <c r="N73" s="102"/>
-      <c r="O73" s="99"/>
-      <c r="Q73" s="108"/>
-      <c r="R73" s="108"/>
-      <c r="S73" s="108"/>
+      <c r="D73" s="121"/>
+      <c r="E73" s="124"/>
+      <c r="G73" s="118"/>
+      <c r="H73" s="130"/>
+      <c r="I73" s="130"/>
+      <c r="J73" s="118"/>
+      <c r="L73" s="100"/>
+      <c r="M73" s="127"/>
+      <c r="N73" s="127"/>
+      <c r="O73" s="100"/>
+      <c r="Q73" s="133"/>
+      <c r="R73" s="133"/>
+      <c r="S73" s="133"/>
     </row>
     <row r="74" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D74" s="93"/>
-      <c r="E74" s="96"/>
-      <c r="G74" s="90"/>
-      <c r="H74" s="105"/>
-      <c r="I74" s="105"/>
-      <c r="J74" s="90"/>
-      <c r="L74" s="99"/>
-      <c r="M74" s="102"/>
-      <c r="N74" s="102"/>
-      <c r="O74" s="99"/>
-      <c r="Q74" s="108"/>
-      <c r="R74" s="108"/>
-      <c r="S74" s="108"/>
+      <c r="D74" s="121"/>
+      <c r="E74" s="124"/>
+      <c r="G74" s="118"/>
+      <c r="H74" s="130"/>
+      <c r="I74" s="130"/>
+      <c r="J74" s="118"/>
+      <c r="L74" s="100"/>
+      <c r="M74" s="127"/>
+      <c r="N74" s="127"/>
+      <c r="O74" s="100"/>
+      <c r="Q74" s="133"/>
+      <c r="R74" s="133"/>
+      <c r="S74" s="133"/>
     </row>
     <row r="75" spans="1:20" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D75" s="94"/>
-      <c r="E75" s="97"/>
-      <c r="G75" s="91"/>
-      <c r="H75" s="106"/>
-      <c r="I75" s="106"/>
-      <c r="J75" s="91"/>
-      <c r="L75" s="100"/>
-      <c r="M75" s="103"/>
-      <c r="N75" s="103"/>
-      <c r="O75" s="100"/>
-      <c r="Q75" s="109"/>
-      <c r="R75" s="109"/>
-      <c r="S75" s="109"/>
+      <c r="D75" s="122"/>
+      <c r="E75" s="125"/>
+      <c r="G75" s="119"/>
+      <c r="H75" s="131"/>
+      <c r="I75" s="131"/>
+      <c r="J75" s="119"/>
+      <c r="L75" s="101"/>
+      <c r="M75" s="128"/>
+      <c r="N75" s="128"/>
+      <c r="O75" s="101"/>
+      <c r="Q75" s="134"/>
+      <c r="R75" s="134"/>
+      <c r="S75" s="134"/>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B6:T60">
     <sortCondition ref="B6"/>
   </sortState>
   <mergeCells count="25">
-    <mergeCell ref="G2:K2"/>
-    <mergeCell ref="D2:F2"/>
-    <mergeCell ref="Q3:T4"/>
-    <mergeCell ref="O66:O75"/>
-    <mergeCell ref="A2:A5"/>
-    <mergeCell ref="G3:K4"/>
-    <mergeCell ref="D3:F4"/>
-    <mergeCell ref="B2:B5"/>
-    <mergeCell ref="C2:C5"/>
     <mergeCell ref="B1:T1"/>
     <mergeCell ref="J66:J75"/>
     <mergeCell ref="D66:D75"/>
@@ -7670,6 +7675,15 @@
     <mergeCell ref="I66:I75"/>
     <mergeCell ref="Q2:T2"/>
     <mergeCell ref="L2:P2"/>
+    <mergeCell ref="G2:K2"/>
+    <mergeCell ref="D2:F2"/>
+    <mergeCell ref="Q3:T4"/>
+    <mergeCell ref="O66:O75"/>
+    <mergeCell ref="A2:A5"/>
+    <mergeCell ref="G3:K4"/>
+    <mergeCell ref="D3:F4"/>
+    <mergeCell ref="B2:B5"/>
+    <mergeCell ref="C2:C5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
hola ayuda a sara
</commit_message>
<xml_diff>
--- a/9_asistencia_evaluacion/pivu_caucasia_notas_quices_asistencia.xlsx
+++ b/9_asistencia_evaluacion/pivu_caucasia_notas_quices_asistencia.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marco\Documentos\extension\camino-udea\9_asistencia_evaluacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CB8F5E9-1628-4181-9D54-A2A9C501AB55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F253509-3F91-4A7E-A048-A3F9C3C6C4C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="104">
   <si>
     <t>METODOLOGÍA DE ESTUDIO</t>
   </si>
@@ -336,15 +336,6 @@
   </si>
   <si>
     <t>raquimus@hotmail.com</t>
-  </si>
-  <si>
-    <t>ojo: verificar correo</t>
-  </si>
-  <si>
-    <t>preguntar correo</t>
-  </si>
-  <si>
-    <t>Ojo: verificar correo</t>
   </si>
   <si>
     <t>Asistencia_lunes_6_abril</t>
@@ -995,7 +986,6 @@
     <xf numFmtId="164" fontId="23" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1109,6 +1099,90 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1136,15 +1210,6 @@
     <xf numFmtId="0" fontId="3" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1187,81 +1252,7 @@
     <xf numFmtId="0" fontId="3" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="23" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Hipervínculo" xfId="2" builtinId="8"/>
@@ -1759,30 +1750,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="72" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="55" t="s">
+      <c r="A1" s="54" t="s">
         <v>27</v>
       </c>
-      <c r="B1" s="54"/>
-      <c r="C1" s="54"/>
-      <c r="D1" s="54"/>
-      <c r="E1" s="54"/>
-      <c r="F1" s="54"/>
-      <c r="G1" s="54"/>
-      <c r="H1" s="54"/>
+      <c r="B1" s="53"/>
+      <c r="C1" s="53"/>
+      <c r="D1" s="53"/>
+      <c r="E1" s="53"/>
+      <c r="F1" s="53"/>
+      <c r="G1" s="53"/>
+      <c r="H1" s="53"/>
     </row>
     <row r="2" spans="1:9" ht="19.8" x14ac:dyDescent="0.3">
-      <c r="A2" s="54" t="s">
+      <c r="A2" s="53" t="s">
         <v>26</v>
       </c>
-      <c r="B2" s="54"/>
-      <c r="C2" s="54"/>
-      <c r="D2" s="54"/>
-      <c r="E2" s="54"/>
-      <c r="F2" s="54"/>
-      <c r="G2" s="54"/>
-      <c r="H2" s="54"/>
-      <c r="I2" s="51" t="s">
-        <v>102</v>
+      <c r="B2" s="53"/>
+      <c r="C2" s="53"/>
+      <c r="D2" s="53"/>
+      <c r="E2" s="53"/>
+      <c r="F2" s="53"/>
+      <c r="G2" s="53"/>
+      <c r="H2" s="53"/>
+      <c r="I2" s="50" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
@@ -1953,12 +1944,10 @@
       <c r="F9" s="44">
         <v>3203519315</v>
       </c>
-      <c r="G9" s="53" t="s">
+      <c r="G9" s="52" t="s">
         <v>95</v>
       </c>
-      <c r="H9" s="50" t="s">
-        <v>101</v>
-      </c>
+      <c r="H9" s="140"/>
     </row>
     <row r="10" spans="1:9" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="42">
@@ -2051,12 +2040,10 @@
       <c r="F13" s="44">
         <v>3136630762</v>
       </c>
-      <c r="G13" s="53" t="s">
+      <c r="G13" s="52" t="s">
         <v>98</v>
       </c>
-      <c r="H13" s="50" t="s">
-        <v>101</v>
-      </c>
+      <c r="H13" s="140"/>
     </row>
     <row r="14" spans="1:9" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="42">
@@ -2197,12 +2184,10 @@
       <c r="F19" s="44">
         <v>3218798123</v>
       </c>
-      <c r="G19" s="53" t="s">
-        <v>104</v>
-      </c>
-      <c r="H19" s="50" t="s">
-        <v>99</v>
-      </c>
+      <c r="G19" s="52" t="s">
+        <v>101</v>
+      </c>
+      <c r="H19" s="140"/>
     </row>
     <row r="20" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="42">
@@ -2271,12 +2256,10 @@
       <c r="F22" s="44">
         <v>3145134544</v>
       </c>
-      <c r="G22" s="53" t="s">
-        <v>106</v>
-      </c>
-      <c r="H22" s="50" t="s">
-        <v>100</v>
-      </c>
+      <c r="G22" s="52" t="s">
+        <v>103</v>
+      </c>
+      <c r="H22" s="140"/>
     </row>
     <row r="23" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="42">
@@ -2657,8 +2640,8 @@
       <c r="F38" s="44">
         <v>3212234096</v>
       </c>
-      <c r="G38" s="53" t="s">
-        <v>105</v>
+      <c r="G38" s="52" t="s">
+        <v>102</v>
       </c>
       <c r="H38" s="44"/>
     </row>
@@ -2707,174 +2690,174 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:31" ht="66" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B1" s="63" t="s">
+      <c r="B1" s="62" t="s">
         <v>18</v>
       </c>
-      <c r="C1" s="63"/>
-      <c r="D1" s="63"/>
-      <c r="E1" s="63"/>
-      <c r="F1" s="63"/>
-      <c r="G1" s="63"/>
-      <c r="H1" s="63"/>
-      <c r="I1" s="63"/>
-      <c r="J1" s="63"/>
-      <c r="K1" s="63"/>
-      <c r="L1" s="63"/>
-      <c r="M1" s="63"/>
-      <c r="N1" s="63"/>
-      <c r="O1" s="63"/>
-      <c r="P1" s="63"/>
-      <c r="Q1" s="63"/>
-      <c r="R1" s="63"/>
-      <c r="S1" s="63"/>
-      <c r="T1" s="63"/>
-      <c r="U1" s="63"/>
-      <c r="V1" s="63"/>
-      <c r="W1" s="63"/>
-      <c r="X1" s="63"/>
-      <c r="Y1" s="63"/>
-      <c r="Z1" s="63"/>
-      <c r="AA1" s="63"/>
-      <c r="AB1" s="63"/>
-      <c r="AC1" s="63"/>
-      <c r="AD1" s="63"/>
-      <c r="AE1" s="63"/>
+      <c r="C1" s="62"/>
+      <c r="D1" s="62"/>
+      <c r="E1" s="62"/>
+      <c r="F1" s="62"/>
+      <c r="G1" s="62"/>
+      <c r="H1" s="62"/>
+      <c r="I1" s="62"/>
+      <c r="J1" s="62"/>
+      <c r="K1" s="62"/>
+      <c r="L1" s="62"/>
+      <c r="M1" s="62"/>
+      <c r="N1" s="62"/>
+      <c r="O1" s="62"/>
+      <c r="P1" s="62"/>
+      <c r="Q1" s="62"/>
+      <c r="R1" s="62"/>
+      <c r="S1" s="62"/>
+      <c r="T1" s="62"/>
+      <c r="U1" s="62"/>
+      <c r="V1" s="62"/>
+      <c r="W1" s="62"/>
+      <c r="X1" s="62"/>
+      <c r="Y1" s="62"/>
+      <c r="Z1" s="62"/>
+      <c r="AA1" s="62"/>
+      <c r="AB1" s="62"/>
+      <c r="AC1" s="62"/>
+      <c r="AD1" s="62"/>
+      <c r="AE1" s="62"/>
     </row>
     <row r="2" spans="1:31" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="64" t="s">
+      <c r="A2" s="63" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="88" t="s">
+      <c r="B2" s="87" t="s">
         <v>21</v>
       </c>
-      <c r="C2" s="64" t="s">
+      <c r="C2" s="63" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="81" t="s">
+      <c r="D2" s="80" t="s">
         <v>19</v>
       </c>
-      <c r="E2" s="82"/>
-      <c r="F2" s="82"/>
-      <c r="G2" s="82"/>
-      <c r="H2" s="83"/>
-      <c r="I2" s="66" t="s">
+      <c r="E2" s="81"/>
+      <c r="F2" s="81"/>
+      <c r="G2" s="81"/>
+      <c r="H2" s="82"/>
+      <c r="I2" s="65" t="s">
         <v>19</v>
       </c>
-      <c r="J2" s="67"/>
-      <c r="K2" s="67"/>
-      <c r="L2" s="67"/>
-      <c r="M2" s="67"/>
-      <c r="N2" s="67"/>
-      <c r="O2" s="67"/>
-      <c r="P2" s="67"/>
-      <c r="Q2" s="68"/>
-      <c r="R2" s="75" t="s">
+      <c r="J2" s="66"/>
+      <c r="K2" s="66"/>
+      <c r="L2" s="66"/>
+      <c r="M2" s="66"/>
+      <c r="N2" s="66"/>
+      <c r="O2" s="66"/>
+      <c r="P2" s="66"/>
+      <c r="Q2" s="67"/>
+      <c r="R2" s="74" t="s">
         <v>19</v>
       </c>
-      <c r="S2" s="76"/>
-      <c r="T2" s="76"/>
-      <c r="U2" s="76"/>
-      <c r="V2" s="76"/>
-      <c r="W2" s="76"/>
-      <c r="X2" s="76"/>
-      <c r="Y2" s="76"/>
-      <c r="Z2" s="77"/>
-      <c r="AA2" s="56" t="s">
+      <c r="S2" s="75"/>
+      <c r="T2" s="75"/>
+      <c r="U2" s="75"/>
+      <c r="V2" s="75"/>
+      <c r="W2" s="75"/>
+      <c r="X2" s="75"/>
+      <c r="Y2" s="75"/>
+      <c r="Z2" s="76"/>
+      <c r="AA2" s="55" t="s">
         <v>19</v>
       </c>
-      <c r="AB2" s="57"/>
-      <c r="AC2" s="57"/>
-      <c r="AD2" s="57"/>
-      <c r="AE2" s="58"/>
+      <c r="AB2" s="56"/>
+      <c r="AC2" s="56"/>
+      <c r="AD2" s="56"/>
+      <c r="AE2" s="57"/>
     </row>
     <row r="3" spans="1:31" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="65"/>
-      <c r="B3" s="89"/>
-      <c r="C3" s="65"/>
-      <c r="D3" s="84" t="s">
+      <c r="A3" s="64"/>
+      <c r="B3" s="88"/>
+      <c r="C3" s="64"/>
+      <c r="D3" s="83" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="85"/>
-      <c r="F3" s="85"/>
-      <c r="G3" s="85"/>
-      <c r="H3" s="86"/>
-      <c r="I3" s="69" t="s">
+      <c r="E3" s="84"/>
+      <c r="F3" s="84"/>
+      <c r="G3" s="84"/>
+      <c r="H3" s="85"/>
+      <c r="I3" s="68" t="s">
         <v>2</v>
       </c>
-      <c r="J3" s="70"/>
-      <c r="K3" s="70"/>
-      <c r="L3" s="70"/>
-      <c r="M3" s="70"/>
-      <c r="N3" s="70"/>
-      <c r="O3" s="70"/>
-      <c r="P3" s="70"/>
-      <c r="Q3" s="71"/>
-      <c r="R3" s="78" t="s">
+      <c r="J3" s="69"/>
+      <c r="K3" s="69"/>
+      <c r="L3" s="69"/>
+      <c r="M3" s="69"/>
+      <c r="N3" s="69"/>
+      <c r="O3" s="69"/>
+      <c r="P3" s="69"/>
+      <c r="Q3" s="70"/>
+      <c r="R3" s="77" t="s">
         <v>1</v>
       </c>
-      <c r="S3" s="79"/>
-      <c r="T3" s="79"/>
-      <c r="U3" s="79"/>
-      <c r="V3" s="79"/>
-      <c r="W3" s="79"/>
-      <c r="X3" s="79"/>
-      <c r="Y3" s="79"/>
-      <c r="Z3" s="80"/>
-      <c r="AA3" s="59" t="s">
-        <v>0</v>
-      </c>
-      <c r="AB3" s="60"/>
-      <c r="AC3" s="60"/>
-      <c r="AD3" s="60"/>
-      <c r="AE3" s="61"/>
+      <c r="S3" s="78"/>
+      <c r="T3" s="78"/>
+      <c r="U3" s="78"/>
+      <c r="V3" s="78"/>
+      <c r="W3" s="78"/>
+      <c r="X3" s="78"/>
+      <c r="Y3" s="78"/>
+      <c r="Z3" s="79"/>
+      <c r="AA3" s="58" t="s">
+        <v>0</v>
+      </c>
+      <c r="AB3" s="59"/>
+      <c r="AC3" s="59"/>
+      <c r="AD3" s="59"/>
+      <c r="AE3" s="60"/>
     </row>
     <row r="4" spans="1:31" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="65"/>
-      <c r="B4" s="89"/>
-      <c r="C4" s="65"/>
-      <c r="D4" s="87" t="s">
+      <c r="A4" s="64"/>
+      <c r="B4" s="88"/>
+      <c r="C4" s="64"/>
+      <c r="D4" s="86" t="s">
         <v>22</v>
       </c>
-      <c r="E4" s="73"/>
-      <c r="F4" s="73"/>
-      <c r="G4" s="74"/>
+      <c r="E4" s="72"/>
+      <c r="F4" s="72"/>
+      <c r="G4" s="73"/>
       <c r="H4" s="1"/>
-      <c r="I4" s="72" t="s">
+      <c r="I4" s="71" t="s">
         <v>23</v>
       </c>
-      <c r="J4" s="73"/>
-      <c r="K4" s="73"/>
-      <c r="L4" s="73"/>
-      <c r="M4" s="73"/>
-      <c r="N4" s="73"/>
-      <c r="O4" s="73"/>
-      <c r="P4" s="74"/>
+      <c r="J4" s="72"/>
+      <c r="K4" s="72"/>
+      <c r="L4" s="72"/>
+      <c r="M4" s="72"/>
+      <c r="N4" s="72"/>
+      <c r="O4" s="72"/>
+      <c r="P4" s="73"/>
       <c r="Q4" s="3"/>
-      <c r="R4" s="72" t="s">
+      <c r="R4" s="71" t="s">
         <v>23</v>
       </c>
-      <c r="S4" s="73"/>
-      <c r="T4" s="73"/>
-      <c r="U4" s="73"/>
-      <c r="V4" s="73"/>
-      <c r="W4" s="73"/>
-      <c r="X4" s="73"/>
-      <c r="Y4" s="74"/>
+      <c r="S4" s="72"/>
+      <c r="T4" s="72"/>
+      <c r="U4" s="72"/>
+      <c r="V4" s="72"/>
+      <c r="W4" s="72"/>
+      <c r="X4" s="72"/>
+      <c r="Y4" s="73"/>
       <c r="Z4" s="12"/>
-      <c r="AA4" s="62" t="s">
+      <c r="AA4" s="61" t="s">
         <v>23</v>
       </c>
-      <c r="AB4" s="62"/>
-      <c r="AC4" s="62"/>
-      <c r="AD4" s="62"/>
+      <c r="AB4" s="61"/>
+      <c r="AC4" s="61"/>
+      <c r="AD4" s="61"/>
       <c r="AE4" s="3"/>
     </row>
     <row r="5" spans="1:31" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="65"/>
-      <c r="B5" s="89"/>
-      <c r="C5" s="65"/>
+      <c r="A5" s="64"/>
+      <c r="B5" s="88"/>
+      <c r="C5" s="64"/>
       <c r="D5" s="28" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="E5" s="28"/>
       <c r="F5" s="28"/>
@@ -4733,7 +4716,7 @@
       </c>
     </row>
     <row r="40" spans="1:31" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A40" s="52">
+      <c r="A40" s="51">
         <v>35</v>
       </c>
     </row>
@@ -4789,123 +4772,123 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="72.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B1" s="116" t="s">
+      <c r="B1" s="89" t="s">
         <v>18</v>
       </c>
-      <c r="C1" s="116"/>
-      <c r="D1" s="116"/>
-      <c r="E1" s="116"/>
-      <c r="F1" s="116"/>
-      <c r="G1" s="116"/>
-      <c r="H1" s="116"/>
-      <c r="I1" s="116"/>
-      <c r="J1" s="116"/>
-      <c r="K1" s="116"/>
-      <c r="L1" s="116"/>
-      <c r="M1" s="116"/>
-      <c r="N1" s="116"/>
-      <c r="O1" s="116"/>
-      <c r="P1" s="116"/>
-      <c r="Q1" s="116"/>
-      <c r="R1" s="116"/>
-      <c r="S1" s="116"/>
-      <c r="T1" s="116"/>
+      <c r="C1" s="89"/>
+      <c r="D1" s="89"/>
+      <c r="E1" s="89"/>
+      <c r="F1" s="89"/>
+      <c r="G1" s="89"/>
+      <c r="H1" s="89"/>
+      <c r="I1" s="89"/>
+      <c r="J1" s="89"/>
+      <c r="K1" s="89"/>
+      <c r="L1" s="89"/>
+      <c r="M1" s="89"/>
+      <c r="N1" s="89"/>
+      <c r="O1" s="89"/>
+      <c r="P1" s="89"/>
+      <c r="Q1" s="89"/>
+      <c r="R1" s="89"/>
+      <c r="S1" s="89"/>
+      <c r="T1" s="89"/>
     </row>
     <row r="2" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="102" t="s">
+      <c r="A2" s="126" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="88" t="s">
+      <c r="B2" s="87" t="s">
         <v>21</v>
       </c>
-      <c r="C2" s="64" t="s">
+      <c r="C2" s="63" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="90" t="str">
+      <c r="D2" s="117" t="str">
         <f>Asistencia!D2</f>
         <v>NOMBRE DOCENTE</v>
       </c>
-      <c r="E2" s="91"/>
-      <c r="F2" s="92"/>
-      <c r="G2" s="90" t="str">
+      <c r="E2" s="118"/>
+      <c r="F2" s="119"/>
+      <c r="G2" s="117" t="str">
         <f>Asistencia!I2</f>
         <v>NOMBRE DOCENTE</v>
       </c>
-      <c r="H2" s="91"/>
-      <c r="I2" s="91"/>
-      <c r="J2" s="91"/>
-      <c r="K2" s="92"/>
-      <c r="L2" s="90" t="s">
+      <c r="H2" s="118"/>
+      <c r="I2" s="118"/>
+      <c r="J2" s="118"/>
+      <c r="K2" s="119"/>
+      <c r="L2" s="117" t="s">
         <v>19</v>
       </c>
-      <c r="M2" s="91"/>
-      <c r="N2" s="91"/>
-      <c r="O2" s="91"/>
-      <c r="P2" s="92"/>
-      <c r="Q2" s="90" t="str">
+      <c r="M2" s="118"/>
+      <c r="N2" s="118"/>
+      <c r="O2" s="118"/>
+      <c r="P2" s="119"/>
+      <c r="Q2" s="117" t="str">
         <f>Asistencia!AA2</f>
         <v>NOMBRE DOCENTE</v>
       </c>
-      <c r="R2" s="91"/>
-      <c r="S2" s="91"/>
-      <c r="T2" s="92"/>
+      <c r="R2" s="118"/>
+      <c r="S2" s="118"/>
+      <c r="T2" s="119"/>
     </row>
     <row r="3" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="103"/>
-      <c r="B3" s="89"/>
-      <c r="C3" s="65"/>
-      <c r="D3" s="110" t="s">
+      <c r="A3" s="127"/>
+      <c r="B3" s="88"/>
+      <c r="C3" s="64"/>
+      <c r="D3" s="134" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="111"/>
-      <c r="F3" s="112"/>
-      <c r="G3" s="104" t="s">
+      <c r="E3" s="135"/>
+      <c r="F3" s="136"/>
+      <c r="G3" s="128" t="s">
         <v>2</v>
       </c>
-      <c r="H3" s="105"/>
-      <c r="I3" s="105"/>
-      <c r="J3" s="105"/>
-      <c r="K3" s="106"/>
-      <c r="L3" s="135" t="s">
+      <c r="H3" s="129"/>
+      <c r="I3" s="129"/>
+      <c r="J3" s="129"/>
+      <c r="K3" s="130"/>
+      <c r="L3" s="111" t="s">
         <v>1</v>
       </c>
-      <c r="M3" s="136"/>
-      <c r="N3" s="136"/>
-      <c r="O3" s="136"/>
-      <c r="P3" s="137"/>
-      <c r="Q3" s="93" t="s">
-        <v>0</v>
-      </c>
-      <c r="R3" s="94"/>
-      <c r="S3" s="94"/>
-      <c r="T3" s="95"/>
+      <c r="M3" s="112"/>
+      <c r="N3" s="112"/>
+      <c r="O3" s="112"/>
+      <c r="P3" s="113"/>
+      <c r="Q3" s="120" t="s">
+        <v>0</v>
+      </c>
+      <c r="R3" s="121"/>
+      <c r="S3" s="121"/>
+      <c r="T3" s="122"/>
     </row>
     <row r="4" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="103"/>
-      <c r="B4" s="89"/>
-      <c r="C4" s="65"/>
-      <c r="D4" s="113"/>
-      <c r="E4" s="114"/>
-      <c r="F4" s="115"/>
-      <c r="G4" s="107"/>
-      <c r="H4" s="108"/>
-      <c r="I4" s="108"/>
-      <c r="J4" s="108"/>
-      <c r="K4" s="109"/>
-      <c r="L4" s="138"/>
-      <c r="M4" s="139"/>
-      <c r="N4" s="139"/>
-      <c r="O4" s="139"/>
-      <c r="P4" s="140"/>
-      <c r="Q4" s="96"/>
-      <c r="R4" s="97"/>
-      <c r="S4" s="97"/>
-      <c r="T4" s="98"/>
+      <c r="A4" s="127"/>
+      <c r="B4" s="88"/>
+      <c r="C4" s="64"/>
+      <c r="D4" s="137"/>
+      <c r="E4" s="138"/>
+      <c r="F4" s="139"/>
+      <c r="G4" s="131"/>
+      <c r="H4" s="132"/>
+      <c r="I4" s="132"/>
+      <c r="J4" s="132"/>
+      <c r="K4" s="133"/>
+      <c r="L4" s="114"/>
+      <c r="M4" s="115"/>
+      <c r="N4" s="115"/>
+      <c r="O4" s="115"/>
+      <c r="P4" s="116"/>
+      <c r="Q4" s="123"/>
+      <c r="R4" s="124"/>
+      <c r="S4" s="124"/>
+      <c r="T4" s="125"/>
     </row>
     <row r="5" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="103"/>
-      <c r="B5" s="89"/>
-      <c r="C5" s="65"/>
+      <c r="A5" s="127"/>
+      <c r="B5" s="88"/>
+      <c r="C5" s="64"/>
       <c r="D5" s="17">
         <v>0.75</v>
       </c>
@@ -7479,186 +7462,195 @@
       </c>
     </row>
     <row r="66" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D66" s="120" t="s">
+      <c r="D66" s="93" t="s">
         <v>24</v>
       </c>
-      <c r="E66" s="123" t="s">
+      <c r="E66" s="96" t="s">
         <v>12</v>
       </c>
-      <c r="G66" s="117" t="s">
+      <c r="G66" s="90" t="s">
         <v>8</v>
       </c>
-      <c r="H66" s="129" t="s">
+      <c r="H66" s="105" t="s">
         <v>9</v>
       </c>
-      <c r="I66" s="129" t="s">
+      <c r="I66" s="105" t="s">
         <v>10</v>
       </c>
-      <c r="J66" s="117" t="s">
+      <c r="J66" s="90" t="s">
         <v>11</v>
       </c>
       <c r="L66" s="99" t="s">
         <v>8</v>
       </c>
-      <c r="M66" s="126" t="s">
+      <c r="M66" s="102" t="s">
         <v>9</v>
       </c>
-      <c r="N66" s="126" t="s">
+      <c r="N66" s="102" t="s">
         <v>10</v>
       </c>
       <c r="O66" s="99" t="s">
         <v>11</v>
       </c>
-      <c r="Q66" s="132" t="s">
+      <c r="Q66" s="108" t="s">
         <v>24</v>
       </c>
-      <c r="R66" s="132" t="s">
+      <c r="R66" s="108" t="s">
         <v>4</v>
       </c>
-      <c r="S66" s="132" t="s">
+      <c r="S66" s="108" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="67" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D67" s="121"/>
-      <c r="E67" s="124"/>
-      <c r="G67" s="118"/>
-      <c r="H67" s="130"/>
-      <c r="I67" s="130"/>
-      <c r="J67" s="118"/>
+      <c r="D67" s="94"/>
+      <c r="E67" s="97"/>
+      <c r="G67" s="91"/>
+      <c r="H67" s="106"/>
+      <c r="I67" s="106"/>
+      <c r="J67" s="91"/>
       <c r="L67" s="100"/>
-      <c r="M67" s="127"/>
-      <c r="N67" s="127"/>
+      <c r="M67" s="103"/>
+      <c r="N67" s="103"/>
       <c r="O67" s="100"/>
-      <c r="Q67" s="133"/>
-      <c r="R67" s="133"/>
-      <c r="S67" s="133"/>
+      <c r="Q67" s="109"/>
+      <c r="R67" s="109"/>
+      <c r="S67" s="109"/>
     </row>
     <row r="68" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D68" s="121"/>
-      <c r="E68" s="124"/>
-      <c r="G68" s="118"/>
-      <c r="H68" s="130"/>
-      <c r="I68" s="130"/>
-      <c r="J68" s="118"/>
+      <c r="D68" s="94"/>
+      <c r="E68" s="97"/>
+      <c r="G68" s="91"/>
+      <c r="H68" s="106"/>
+      <c r="I68" s="106"/>
+      <c r="J68" s="91"/>
       <c r="L68" s="100"/>
-      <c r="M68" s="127"/>
-      <c r="N68" s="127"/>
+      <c r="M68" s="103"/>
+      <c r="N68" s="103"/>
       <c r="O68" s="100"/>
-      <c r="Q68" s="133"/>
-      <c r="R68" s="133"/>
-      <c r="S68" s="133"/>
+      <c r="Q68" s="109"/>
+      <c r="R68" s="109"/>
+      <c r="S68" s="109"/>
     </row>
     <row r="69" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D69" s="121"/>
-      <c r="E69" s="124"/>
-      <c r="G69" s="118"/>
-      <c r="H69" s="130"/>
-      <c r="I69" s="130"/>
-      <c r="J69" s="118"/>
+      <c r="D69" s="94"/>
+      <c r="E69" s="97"/>
+      <c r="G69" s="91"/>
+      <c r="H69" s="106"/>
+      <c r="I69" s="106"/>
+      <c r="J69" s="91"/>
       <c r="L69" s="100"/>
-      <c r="M69" s="127"/>
-      <c r="N69" s="127"/>
+      <c r="M69" s="103"/>
+      <c r="N69" s="103"/>
       <c r="O69" s="100"/>
-      <c r="Q69" s="133"/>
-      <c r="R69" s="133"/>
-      <c r="S69" s="133"/>
+      <c r="Q69" s="109"/>
+      <c r="R69" s="109"/>
+      <c r="S69" s="109"/>
     </row>
     <row r="70" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D70" s="121"/>
-      <c r="E70" s="124"/>
-      <c r="G70" s="118"/>
-      <c r="H70" s="130"/>
-      <c r="I70" s="130"/>
-      <c r="J70" s="118"/>
+      <c r="D70" s="94"/>
+      <c r="E70" s="97"/>
+      <c r="G70" s="91"/>
+      <c r="H70" s="106"/>
+      <c r="I70" s="106"/>
+      <c r="J70" s="91"/>
       <c r="L70" s="100"/>
-      <c r="M70" s="127"/>
-      <c r="N70" s="127"/>
+      <c r="M70" s="103"/>
+      <c r="N70" s="103"/>
       <c r="O70" s="100"/>
-      <c r="Q70" s="133"/>
-      <c r="R70" s="133"/>
-      <c r="S70" s="133"/>
+      <c r="Q70" s="109"/>
+      <c r="R70" s="109"/>
+      <c r="S70" s="109"/>
     </row>
     <row r="71" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D71" s="121"/>
-      <c r="E71" s="124"/>
-      <c r="G71" s="118"/>
-      <c r="H71" s="130"/>
-      <c r="I71" s="130"/>
-      <c r="J71" s="118"/>
+      <c r="D71" s="94"/>
+      <c r="E71" s="97"/>
+      <c r="G71" s="91"/>
+      <c r="H71" s="106"/>
+      <c r="I71" s="106"/>
+      <c r="J71" s="91"/>
       <c r="L71" s="100"/>
-      <c r="M71" s="127"/>
-      <c r="N71" s="127"/>
+      <c r="M71" s="103"/>
+      <c r="N71" s="103"/>
       <c r="O71" s="100"/>
-      <c r="Q71" s="133"/>
-      <c r="R71" s="133"/>
-      <c r="S71" s="133"/>
+      <c r="Q71" s="109"/>
+      <c r="R71" s="109"/>
+      <c r="S71" s="109"/>
     </row>
     <row r="72" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D72" s="121"/>
-      <c r="E72" s="124"/>
-      <c r="G72" s="118"/>
-      <c r="H72" s="130"/>
-      <c r="I72" s="130"/>
-      <c r="J72" s="118"/>
+      <c r="D72" s="94"/>
+      <c r="E72" s="97"/>
+      <c r="G72" s="91"/>
+      <c r="H72" s="106"/>
+      <c r="I72" s="106"/>
+      <c r="J72" s="91"/>
       <c r="L72" s="100"/>
-      <c r="M72" s="127"/>
-      <c r="N72" s="127"/>
+      <c r="M72" s="103"/>
+      <c r="N72" s="103"/>
       <c r="O72" s="100"/>
-      <c r="Q72" s="133"/>
-      <c r="R72" s="133"/>
-      <c r="S72" s="133"/>
+      <c r="Q72" s="109"/>
+      <c r="R72" s="109"/>
+      <c r="S72" s="109"/>
     </row>
     <row r="73" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D73" s="121"/>
-      <c r="E73" s="124"/>
-      <c r="G73" s="118"/>
-      <c r="H73" s="130"/>
-      <c r="I73" s="130"/>
-      <c r="J73" s="118"/>
+      <c r="D73" s="94"/>
+      <c r="E73" s="97"/>
+      <c r="G73" s="91"/>
+      <c r="H73" s="106"/>
+      <c r="I73" s="106"/>
+      <c r="J73" s="91"/>
       <c r="L73" s="100"/>
-      <c r="M73" s="127"/>
-      <c r="N73" s="127"/>
+      <c r="M73" s="103"/>
+      <c r="N73" s="103"/>
       <c r="O73" s="100"/>
-      <c r="Q73" s="133"/>
-      <c r="R73" s="133"/>
-      <c r="S73" s="133"/>
+      <c r="Q73" s="109"/>
+      <c r="R73" s="109"/>
+      <c r="S73" s="109"/>
     </row>
     <row r="74" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D74" s="121"/>
-      <c r="E74" s="124"/>
-      <c r="G74" s="118"/>
-      <c r="H74" s="130"/>
-      <c r="I74" s="130"/>
-      <c r="J74" s="118"/>
+      <c r="D74" s="94"/>
+      <c r="E74" s="97"/>
+      <c r="G74" s="91"/>
+      <c r="H74" s="106"/>
+      <c r="I74" s="106"/>
+      <c r="J74" s="91"/>
       <c r="L74" s="100"/>
-      <c r="M74" s="127"/>
-      <c r="N74" s="127"/>
+      <c r="M74" s="103"/>
+      <c r="N74" s="103"/>
       <c r="O74" s="100"/>
-      <c r="Q74" s="133"/>
-      <c r="R74" s="133"/>
-      <c r="S74" s="133"/>
+      <c r="Q74" s="109"/>
+      <c r="R74" s="109"/>
+      <c r="S74" s="109"/>
     </row>
     <row r="75" spans="1:20" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D75" s="122"/>
-      <c r="E75" s="125"/>
-      <c r="G75" s="119"/>
-      <c r="H75" s="131"/>
-      <c r="I75" s="131"/>
-      <c r="J75" s="119"/>
+      <c r="D75" s="95"/>
+      <c r="E75" s="98"/>
+      <c r="G75" s="92"/>
+      <c r="H75" s="107"/>
+      <c r="I75" s="107"/>
+      <c r="J75" s="92"/>
       <c r="L75" s="101"/>
-      <c r="M75" s="128"/>
-      <c r="N75" s="128"/>
+      <c r="M75" s="104"/>
+      <c r="N75" s="104"/>
       <c r="O75" s="101"/>
-      <c r="Q75" s="134"/>
-      <c r="R75" s="134"/>
-      <c r="S75" s="134"/>
+      <c r="Q75" s="110"/>
+      <c r="R75" s="110"/>
+      <c r="S75" s="110"/>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B6:T60">
     <sortCondition ref="B6"/>
   </sortState>
   <mergeCells count="25">
+    <mergeCell ref="G2:K2"/>
+    <mergeCell ref="D2:F2"/>
+    <mergeCell ref="Q3:T4"/>
+    <mergeCell ref="O66:O75"/>
+    <mergeCell ref="A2:A5"/>
+    <mergeCell ref="G3:K4"/>
+    <mergeCell ref="D3:F4"/>
+    <mergeCell ref="B2:B5"/>
+    <mergeCell ref="C2:C5"/>
     <mergeCell ref="B1:T1"/>
     <mergeCell ref="J66:J75"/>
     <mergeCell ref="D66:D75"/>
@@ -7675,15 +7667,6 @@
     <mergeCell ref="I66:I75"/>
     <mergeCell ref="Q2:T2"/>
     <mergeCell ref="L2:P2"/>
-    <mergeCell ref="G2:K2"/>
-    <mergeCell ref="D2:F2"/>
-    <mergeCell ref="Q3:T4"/>
-    <mergeCell ref="O66:O75"/>
-    <mergeCell ref="A2:A5"/>
-    <mergeCell ref="G3:K4"/>
-    <mergeCell ref="D3:F4"/>
-    <mergeCell ref="B2:B5"/>
-    <mergeCell ref="C2:C5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
inicio de preparación de la clase 7
</commit_message>
<xml_diff>
--- a/9_asistencia_evaluacion/pivu_caucasia_notas_quices_asistencia.xlsx
+++ b/9_asistencia_evaluacion/pivu_caucasia_notas_quices_asistencia.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marco\Documentos\extension\camino-udea\9_asistencia_evaluacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F253509-3F91-4A7E-A048-A3F9C3C6C4C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4EC5795-A1F6-4380-B3CB-5A38912B0CF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="105">
   <si>
     <t>METODOLOGÍA DE ESTUDIO</t>
   </si>
@@ -351,6 +351,9 @@
   </si>
   <si>
     <t>mariallno0716@gmail.com</t>
+  </si>
+  <si>
+    <t>resolver problema con su correo</t>
   </si>
 </sst>
 </file>
@@ -845,7 +848,7 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="141">
+  <cellXfs count="142">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -991,6 +994,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="23" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="22" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1099,6 +1103,84 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1129,15 +1211,6 @@
     <xf numFmtId="0" fontId="7" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
@@ -1183,76 +1256,7 @@
     <xf numFmtId="0" fontId="3" fillId="9" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="23" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Hipervínculo" xfId="2" builtinId="8"/>
@@ -1744,34 +1748,34 @@
     <col min="5" max="5" width="12.88671875" style="38" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="13.6640625" style="45" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="40.33203125" style="45" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="6" style="46" customWidth="1"/>
+    <col min="8" max="8" width="29.21875" style="46" customWidth="1"/>
     <col min="9" max="9" width="22.77734375" style="38" customWidth="1"/>
     <col min="10" max="16384" width="11.44140625" style="38"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="72" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="54" t="s">
+      <c r="A1" s="55" t="s">
         <v>27</v>
       </c>
-      <c r="B1" s="53"/>
-      <c r="C1" s="53"/>
-      <c r="D1" s="53"/>
-      <c r="E1" s="53"/>
-      <c r="F1" s="53"/>
-      <c r="G1" s="53"/>
-      <c r="H1" s="53"/>
+      <c r="B1" s="54"/>
+      <c r="C1" s="54"/>
+      <c r="D1" s="54"/>
+      <c r="E1" s="54"/>
+      <c r="F1" s="54"/>
+      <c r="G1" s="54"/>
+      <c r="H1" s="54"/>
     </row>
     <row r="2" spans="1:9" ht="19.8" x14ac:dyDescent="0.3">
-      <c r="A2" s="53" t="s">
+      <c r="A2" s="54" t="s">
         <v>26</v>
       </c>
-      <c r="B2" s="53"/>
-      <c r="C2" s="53"/>
-      <c r="D2" s="53"/>
-      <c r="E2" s="53"/>
-      <c r="F2" s="53"/>
-      <c r="G2" s="53"/>
-      <c r="H2" s="53"/>
+      <c r="B2" s="54"/>
+      <c r="C2" s="54"/>
+      <c r="D2" s="54"/>
+      <c r="E2" s="54"/>
+      <c r="F2" s="54"/>
+      <c r="G2" s="54"/>
+      <c r="H2" s="54"/>
       <c r="I2" s="50" t="s">
         <v>99</v>
       </c>
@@ -1947,7 +1951,9 @@
       <c r="G9" s="52" t="s">
         <v>95</v>
       </c>
-      <c r="H9" s="140"/>
+      <c r="H9" s="141" t="s">
+        <v>104</v>
+      </c>
     </row>
     <row r="10" spans="1:9" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="42">
@@ -2043,7 +2049,7 @@
       <c r="G13" s="52" t="s">
         <v>98</v>
       </c>
-      <c r="H13" s="140"/>
+      <c r="H13" s="53"/>
     </row>
     <row r="14" spans="1:9" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="42">
@@ -2187,7 +2193,7 @@
       <c r="G19" s="52" t="s">
         <v>101</v>
       </c>
-      <c r="H19" s="140"/>
+      <c r="H19" s="53"/>
     </row>
     <row r="20" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="42">
@@ -2259,7 +2265,7 @@
       <c r="G22" s="52" t="s">
         <v>103</v>
       </c>
-      <c r="H22" s="140"/>
+      <c r="H22" s="53"/>
     </row>
     <row r="23" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="42">
@@ -2690,172 +2696,172 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:31" ht="66" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B1" s="62" t="s">
+      <c r="B1" s="63" t="s">
         <v>18</v>
       </c>
-      <c r="C1" s="62"/>
-      <c r="D1" s="62"/>
-      <c r="E1" s="62"/>
-      <c r="F1" s="62"/>
-      <c r="G1" s="62"/>
-      <c r="H1" s="62"/>
-      <c r="I1" s="62"/>
-      <c r="J1" s="62"/>
-      <c r="K1" s="62"/>
-      <c r="L1" s="62"/>
-      <c r="M1" s="62"/>
-      <c r="N1" s="62"/>
-      <c r="O1" s="62"/>
-      <c r="P1" s="62"/>
-      <c r="Q1" s="62"/>
-      <c r="R1" s="62"/>
-      <c r="S1" s="62"/>
-      <c r="T1" s="62"/>
-      <c r="U1" s="62"/>
-      <c r="V1" s="62"/>
-      <c r="W1" s="62"/>
-      <c r="X1" s="62"/>
-      <c r="Y1" s="62"/>
-      <c r="Z1" s="62"/>
-      <c r="AA1" s="62"/>
-      <c r="AB1" s="62"/>
-      <c r="AC1" s="62"/>
-      <c r="AD1" s="62"/>
-      <c r="AE1" s="62"/>
+      <c r="C1" s="63"/>
+      <c r="D1" s="63"/>
+      <c r="E1" s="63"/>
+      <c r="F1" s="63"/>
+      <c r="G1" s="63"/>
+      <c r="H1" s="63"/>
+      <c r="I1" s="63"/>
+      <c r="J1" s="63"/>
+      <c r="K1" s="63"/>
+      <c r="L1" s="63"/>
+      <c r="M1" s="63"/>
+      <c r="N1" s="63"/>
+      <c r="O1" s="63"/>
+      <c r="P1" s="63"/>
+      <c r="Q1" s="63"/>
+      <c r="R1" s="63"/>
+      <c r="S1" s="63"/>
+      <c r="T1" s="63"/>
+      <c r="U1" s="63"/>
+      <c r="V1" s="63"/>
+      <c r="W1" s="63"/>
+      <c r="X1" s="63"/>
+      <c r="Y1" s="63"/>
+      <c r="Z1" s="63"/>
+      <c r="AA1" s="63"/>
+      <c r="AB1" s="63"/>
+      <c r="AC1" s="63"/>
+      <c r="AD1" s="63"/>
+      <c r="AE1" s="63"/>
     </row>
     <row r="2" spans="1:31" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="63" t="s">
+      <c r="A2" s="64" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="87" t="s">
+      <c r="B2" s="88" t="s">
         <v>21</v>
       </c>
-      <c r="C2" s="63" t="s">
+      <c r="C2" s="64" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="80" t="s">
+      <c r="D2" s="81" t="s">
         <v>19</v>
       </c>
-      <c r="E2" s="81"/>
-      <c r="F2" s="81"/>
-      <c r="G2" s="81"/>
-      <c r="H2" s="82"/>
-      <c r="I2" s="65" t="s">
+      <c r="E2" s="82"/>
+      <c r="F2" s="82"/>
+      <c r="G2" s="82"/>
+      <c r="H2" s="83"/>
+      <c r="I2" s="66" t="s">
         <v>19</v>
       </c>
-      <c r="J2" s="66"/>
-      <c r="K2" s="66"/>
-      <c r="L2" s="66"/>
-      <c r="M2" s="66"/>
-      <c r="N2" s="66"/>
-      <c r="O2" s="66"/>
-      <c r="P2" s="66"/>
-      <c r="Q2" s="67"/>
-      <c r="R2" s="74" t="s">
+      <c r="J2" s="67"/>
+      <c r="K2" s="67"/>
+      <c r="L2" s="67"/>
+      <c r="M2" s="67"/>
+      <c r="N2" s="67"/>
+      <c r="O2" s="67"/>
+      <c r="P2" s="67"/>
+      <c r="Q2" s="68"/>
+      <c r="R2" s="75" t="s">
         <v>19</v>
       </c>
-      <c r="S2" s="75"/>
-      <c r="T2" s="75"/>
-      <c r="U2" s="75"/>
-      <c r="V2" s="75"/>
-      <c r="W2" s="75"/>
-      <c r="X2" s="75"/>
-      <c r="Y2" s="75"/>
-      <c r="Z2" s="76"/>
-      <c r="AA2" s="55" t="s">
+      <c r="S2" s="76"/>
+      <c r="T2" s="76"/>
+      <c r="U2" s="76"/>
+      <c r="V2" s="76"/>
+      <c r="W2" s="76"/>
+      <c r="X2" s="76"/>
+      <c r="Y2" s="76"/>
+      <c r="Z2" s="77"/>
+      <c r="AA2" s="56" t="s">
         <v>19</v>
       </c>
-      <c r="AB2" s="56"/>
-      <c r="AC2" s="56"/>
-      <c r="AD2" s="56"/>
-      <c r="AE2" s="57"/>
+      <c r="AB2" s="57"/>
+      <c r="AC2" s="57"/>
+      <c r="AD2" s="57"/>
+      <c r="AE2" s="58"/>
     </row>
     <row r="3" spans="1:31" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="64"/>
-      <c r="B3" s="88"/>
-      <c r="C3" s="64"/>
-      <c r="D3" s="83" t="s">
+      <c r="A3" s="65"/>
+      <c r="B3" s="89"/>
+      <c r="C3" s="65"/>
+      <c r="D3" s="84" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="84"/>
-      <c r="F3" s="84"/>
-      <c r="G3" s="84"/>
-      <c r="H3" s="85"/>
-      <c r="I3" s="68" t="s">
+      <c r="E3" s="85"/>
+      <c r="F3" s="85"/>
+      <c r="G3" s="85"/>
+      <c r="H3" s="86"/>
+      <c r="I3" s="69" t="s">
         <v>2</v>
       </c>
-      <c r="J3" s="69"/>
-      <c r="K3" s="69"/>
-      <c r="L3" s="69"/>
-      <c r="M3" s="69"/>
-      <c r="N3" s="69"/>
-      <c r="O3" s="69"/>
-      <c r="P3" s="69"/>
-      <c r="Q3" s="70"/>
-      <c r="R3" s="77" t="s">
+      <c r="J3" s="70"/>
+      <c r="K3" s="70"/>
+      <c r="L3" s="70"/>
+      <c r="M3" s="70"/>
+      <c r="N3" s="70"/>
+      <c r="O3" s="70"/>
+      <c r="P3" s="70"/>
+      <c r="Q3" s="71"/>
+      <c r="R3" s="78" t="s">
         <v>1</v>
       </c>
-      <c r="S3" s="78"/>
-      <c r="T3" s="78"/>
-      <c r="U3" s="78"/>
-      <c r="V3" s="78"/>
-      <c r="W3" s="78"/>
-      <c r="X3" s="78"/>
-      <c r="Y3" s="78"/>
-      <c r="Z3" s="79"/>
-      <c r="AA3" s="58" t="s">
-        <v>0</v>
-      </c>
-      <c r="AB3" s="59"/>
-      <c r="AC3" s="59"/>
-      <c r="AD3" s="59"/>
-      <c r="AE3" s="60"/>
+      <c r="S3" s="79"/>
+      <c r="T3" s="79"/>
+      <c r="U3" s="79"/>
+      <c r="V3" s="79"/>
+      <c r="W3" s="79"/>
+      <c r="X3" s="79"/>
+      <c r="Y3" s="79"/>
+      <c r="Z3" s="80"/>
+      <c r="AA3" s="59" t="s">
+        <v>0</v>
+      </c>
+      <c r="AB3" s="60"/>
+      <c r="AC3" s="60"/>
+      <c r="AD3" s="60"/>
+      <c r="AE3" s="61"/>
     </row>
     <row r="4" spans="1:31" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="64"/>
-      <c r="B4" s="88"/>
-      <c r="C4" s="64"/>
-      <c r="D4" s="86" t="s">
+      <c r="A4" s="65"/>
+      <c r="B4" s="89"/>
+      <c r="C4" s="65"/>
+      <c r="D4" s="87" t="s">
         <v>22</v>
       </c>
-      <c r="E4" s="72"/>
-      <c r="F4" s="72"/>
-      <c r="G4" s="73"/>
+      <c r="E4" s="73"/>
+      <c r="F4" s="73"/>
+      <c r="G4" s="74"/>
       <c r="H4" s="1"/>
-      <c r="I4" s="71" t="s">
+      <c r="I4" s="72" t="s">
         <v>23</v>
       </c>
-      <c r="J4" s="72"/>
-      <c r="K4" s="72"/>
-      <c r="L4" s="72"/>
-      <c r="M4" s="72"/>
-      <c r="N4" s="72"/>
-      <c r="O4" s="72"/>
-      <c r="P4" s="73"/>
+      <c r="J4" s="73"/>
+      <c r="K4" s="73"/>
+      <c r="L4" s="73"/>
+      <c r="M4" s="73"/>
+      <c r="N4" s="73"/>
+      <c r="O4" s="73"/>
+      <c r="P4" s="74"/>
       <c r="Q4" s="3"/>
-      <c r="R4" s="71" t="s">
+      <c r="R4" s="72" t="s">
         <v>23</v>
       </c>
-      <c r="S4" s="72"/>
-      <c r="T4" s="72"/>
-      <c r="U4" s="72"/>
-      <c r="V4" s="72"/>
-      <c r="W4" s="72"/>
-      <c r="X4" s="72"/>
-      <c r="Y4" s="73"/>
+      <c r="S4" s="73"/>
+      <c r="T4" s="73"/>
+      <c r="U4" s="73"/>
+      <c r="V4" s="73"/>
+      <c r="W4" s="73"/>
+      <c r="X4" s="73"/>
+      <c r="Y4" s="74"/>
       <c r="Z4" s="12"/>
-      <c r="AA4" s="61" t="s">
+      <c r="AA4" s="62" t="s">
         <v>23</v>
       </c>
-      <c r="AB4" s="61"/>
-      <c r="AC4" s="61"/>
-      <c r="AD4" s="61"/>
+      <c r="AB4" s="62"/>
+      <c r="AC4" s="62"/>
+      <c r="AD4" s="62"/>
       <c r="AE4" s="3"/>
     </row>
     <row r="5" spans="1:31" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="64"/>
-      <c r="B5" s="88"/>
-      <c r="C5" s="64"/>
+      <c r="A5" s="65"/>
+      <c r="B5" s="89"/>
+      <c r="C5" s="65"/>
       <c r="D5" s="28" t="s">
         <v>100</v>
       </c>
@@ -4772,123 +4778,123 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="72.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B1" s="89" t="s">
+      <c r="B1" s="116" t="s">
         <v>18</v>
       </c>
-      <c r="C1" s="89"/>
-      <c r="D1" s="89"/>
-      <c r="E1" s="89"/>
-      <c r="F1" s="89"/>
-      <c r="G1" s="89"/>
-      <c r="H1" s="89"/>
-      <c r="I1" s="89"/>
-      <c r="J1" s="89"/>
-      <c r="K1" s="89"/>
-      <c r="L1" s="89"/>
-      <c r="M1" s="89"/>
-      <c r="N1" s="89"/>
-      <c r="O1" s="89"/>
-      <c r="P1" s="89"/>
-      <c r="Q1" s="89"/>
-      <c r="R1" s="89"/>
-      <c r="S1" s="89"/>
-      <c r="T1" s="89"/>
+      <c r="C1" s="116"/>
+      <c r="D1" s="116"/>
+      <c r="E1" s="116"/>
+      <c r="F1" s="116"/>
+      <c r="G1" s="116"/>
+      <c r="H1" s="116"/>
+      <c r="I1" s="116"/>
+      <c r="J1" s="116"/>
+      <c r="K1" s="116"/>
+      <c r="L1" s="116"/>
+      <c r="M1" s="116"/>
+      <c r="N1" s="116"/>
+      <c r="O1" s="116"/>
+      <c r="P1" s="116"/>
+      <c r="Q1" s="116"/>
+      <c r="R1" s="116"/>
+      <c r="S1" s="116"/>
+      <c r="T1" s="116"/>
     </row>
     <row r="2" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="126" t="s">
+      <c r="A2" s="102" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="87" t="s">
+      <c r="B2" s="88" t="s">
         <v>21</v>
       </c>
-      <c r="C2" s="63" t="s">
+      <c r="C2" s="64" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="117" t="str">
+      <c r="D2" s="90" t="str">
         <f>Asistencia!D2</f>
         <v>NOMBRE DOCENTE</v>
       </c>
-      <c r="E2" s="118"/>
-      <c r="F2" s="119"/>
-      <c r="G2" s="117" t="str">
+      <c r="E2" s="91"/>
+      <c r="F2" s="92"/>
+      <c r="G2" s="90" t="str">
         <f>Asistencia!I2</f>
         <v>NOMBRE DOCENTE</v>
       </c>
-      <c r="H2" s="118"/>
-      <c r="I2" s="118"/>
-      <c r="J2" s="118"/>
-      <c r="K2" s="119"/>
-      <c r="L2" s="117" t="s">
+      <c r="H2" s="91"/>
+      <c r="I2" s="91"/>
+      <c r="J2" s="91"/>
+      <c r="K2" s="92"/>
+      <c r="L2" s="90" t="s">
         <v>19</v>
       </c>
-      <c r="M2" s="118"/>
-      <c r="N2" s="118"/>
-      <c r="O2" s="118"/>
-      <c r="P2" s="119"/>
-      <c r="Q2" s="117" t="str">
+      <c r="M2" s="91"/>
+      <c r="N2" s="91"/>
+      <c r="O2" s="91"/>
+      <c r="P2" s="92"/>
+      <c r="Q2" s="90" t="str">
         <f>Asistencia!AA2</f>
         <v>NOMBRE DOCENTE</v>
       </c>
-      <c r="R2" s="118"/>
-      <c r="S2" s="118"/>
-      <c r="T2" s="119"/>
+      <c r="R2" s="91"/>
+      <c r="S2" s="91"/>
+      <c r="T2" s="92"/>
     </row>
     <row r="3" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="127"/>
-      <c r="B3" s="88"/>
-      <c r="C3" s="64"/>
-      <c r="D3" s="134" t="s">
+      <c r="A3" s="103"/>
+      <c r="B3" s="89"/>
+      <c r="C3" s="65"/>
+      <c r="D3" s="110" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="135"/>
-      <c r="F3" s="136"/>
-      <c r="G3" s="128" t="s">
+      <c r="E3" s="111"/>
+      <c r="F3" s="112"/>
+      <c r="G3" s="104" t="s">
         <v>2</v>
       </c>
-      <c r="H3" s="129"/>
-      <c r="I3" s="129"/>
-      <c r="J3" s="129"/>
-      <c r="K3" s="130"/>
-      <c r="L3" s="111" t="s">
+      <c r="H3" s="105"/>
+      <c r="I3" s="105"/>
+      <c r="J3" s="105"/>
+      <c r="K3" s="106"/>
+      <c r="L3" s="135" t="s">
         <v>1</v>
       </c>
-      <c r="M3" s="112"/>
-      <c r="N3" s="112"/>
-      <c r="O3" s="112"/>
-      <c r="P3" s="113"/>
-      <c r="Q3" s="120" t="s">
-        <v>0</v>
-      </c>
-      <c r="R3" s="121"/>
-      <c r="S3" s="121"/>
-      <c r="T3" s="122"/>
+      <c r="M3" s="136"/>
+      <c r="N3" s="136"/>
+      <c r="O3" s="136"/>
+      <c r="P3" s="137"/>
+      <c r="Q3" s="93" t="s">
+        <v>0</v>
+      </c>
+      <c r="R3" s="94"/>
+      <c r="S3" s="94"/>
+      <c r="T3" s="95"/>
     </row>
     <row r="4" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="127"/>
-      <c r="B4" s="88"/>
-      <c r="C4" s="64"/>
-      <c r="D4" s="137"/>
-      <c r="E4" s="138"/>
-      <c r="F4" s="139"/>
-      <c r="G4" s="131"/>
-      <c r="H4" s="132"/>
-      <c r="I4" s="132"/>
-      <c r="J4" s="132"/>
-      <c r="K4" s="133"/>
-      <c r="L4" s="114"/>
-      <c r="M4" s="115"/>
-      <c r="N4" s="115"/>
-      <c r="O4" s="115"/>
-      <c r="P4" s="116"/>
-      <c r="Q4" s="123"/>
-      <c r="R4" s="124"/>
-      <c r="S4" s="124"/>
-      <c r="T4" s="125"/>
+      <c r="A4" s="103"/>
+      <c r="B4" s="89"/>
+      <c r="C4" s="65"/>
+      <c r="D4" s="113"/>
+      <c r="E4" s="114"/>
+      <c r="F4" s="115"/>
+      <c r="G4" s="107"/>
+      <c r="H4" s="108"/>
+      <c r="I4" s="108"/>
+      <c r="J4" s="108"/>
+      <c r="K4" s="109"/>
+      <c r="L4" s="138"/>
+      <c r="M4" s="139"/>
+      <c r="N4" s="139"/>
+      <c r="O4" s="139"/>
+      <c r="P4" s="140"/>
+      <c r="Q4" s="96"/>
+      <c r="R4" s="97"/>
+      <c r="S4" s="97"/>
+      <c r="T4" s="98"/>
     </row>
     <row r="5" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="127"/>
-      <c r="B5" s="88"/>
-      <c r="C5" s="64"/>
+      <c r="A5" s="103"/>
+      <c r="B5" s="89"/>
+      <c r="C5" s="65"/>
       <c r="D5" s="17">
         <v>0.75</v>
       </c>
@@ -7462,195 +7468,186 @@
       </c>
     </row>
     <row r="66" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D66" s="93" t="s">
+      <c r="D66" s="120" t="s">
         <v>24</v>
       </c>
-      <c r="E66" s="96" t="s">
+      <c r="E66" s="123" t="s">
         <v>12</v>
       </c>
-      <c r="G66" s="90" t="s">
+      <c r="G66" s="117" t="s">
         <v>8</v>
       </c>
-      <c r="H66" s="105" t="s">
+      <c r="H66" s="129" t="s">
         <v>9</v>
       </c>
-      <c r="I66" s="105" t="s">
+      <c r="I66" s="129" t="s">
         <v>10</v>
       </c>
-      <c r="J66" s="90" t="s">
+      <c r="J66" s="117" t="s">
         <v>11</v>
       </c>
       <c r="L66" s="99" t="s">
         <v>8</v>
       </c>
-      <c r="M66" s="102" t="s">
+      <c r="M66" s="126" t="s">
         <v>9</v>
       </c>
-      <c r="N66" s="102" t="s">
+      <c r="N66" s="126" t="s">
         <v>10</v>
       </c>
       <c r="O66" s="99" t="s">
         <v>11</v>
       </c>
-      <c r="Q66" s="108" t="s">
+      <c r="Q66" s="132" t="s">
         <v>24</v>
       </c>
-      <c r="R66" s="108" t="s">
+      <c r="R66" s="132" t="s">
         <v>4</v>
       </c>
-      <c r="S66" s="108" t="s">
+      <c r="S66" s="132" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="67" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D67" s="94"/>
-      <c r="E67" s="97"/>
-      <c r="G67" s="91"/>
-      <c r="H67" s="106"/>
-      <c r="I67" s="106"/>
-      <c r="J67" s="91"/>
+      <c r="D67" s="121"/>
+      <c r="E67" s="124"/>
+      <c r="G67" s="118"/>
+      <c r="H67" s="130"/>
+      <c r="I67" s="130"/>
+      <c r="J67" s="118"/>
       <c r="L67" s="100"/>
-      <c r="M67" s="103"/>
-      <c r="N67" s="103"/>
+      <c r="M67" s="127"/>
+      <c r="N67" s="127"/>
       <c r="O67" s="100"/>
-      <c r="Q67" s="109"/>
-      <c r="R67" s="109"/>
-      <c r="S67" s="109"/>
+      <c r="Q67" s="133"/>
+      <c r="R67" s="133"/>
+      <c r="S67" s="133"/>
     </row>
     <row r="68" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D68" s="94"/>
-      <c r="E68" s="97"/>
-      <c r="G68" s="91"/>
-      <c r="H68" s="106"/>
-      <c r="I68" s="106"/>
-      <c r="J68" s="91"/>
+      <c r="D68" s="121"/>
+      <c r="E68" s="124"/>
+      <c r="G68" s="118"/>
+      <c r="H68" s="130"/>
+      <c r="I68" s="130"/>
+      <c r="J68" s="118"/>
       <c r="L68" s="100"/>
-      <c r="M68" s="103"/>
-      <c r="N68" s="103"/>
+      <c r="M68" s="127"/>
+      <c r="N68" s="127"/>
       <c r="O68" s="100"/>
-      <c r="Q68" s="109"/>
-      <c r="R68" s="109"/>
-      <c r="S68" s="109"/>
+      <c r="Q68" s="133"/>
+      <c r="R68" s="133"/>
+      <c r="S68" s="133"/>
     </row>
     <row r="69" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D69" s="94"/>
-      <c r="E69" s="97"/>
-      <c r="G69" s="91"/>
-      <c r="H69" s="106"/>
-      <c r="I69" s="106"/>
-      <c r="J69" s="91"/>
+      <c r="D69" s="121"/>
+      <c r="E69" s="124"/>
+      <c r="G69" s="118"/>
+      <c r="H69" s="130"/>
+      <c r="I69" s="130"/>
+      <c r="J69" s="118"/>
       <c r="L69" s="100"/>
-      <c r="M69" s="103"/>
-      <c r="N69" s="103"/>
+      <c r="M69" s="127"/>
+      <c r="N69" s="127"/>
       <c r="O69" s="100"/>
-      <c r="Q69" s="109"/>
-      <c r="R69" s="109"/>
-      <c r="S69" s="109"/>
+      <c r="Q69" s="133"/>
+      <c r="R69" s="133"/>
+      <c r="S69" s="133"/>
     </row>
     <row r="70" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D70" s="94"/>
-      <c r="E70" s="97"/>
-      <c r="G70" s="91"/>
-      <c r="H70" s="106"/>
-      <c r="I70" s="106"/>
-      <c r="J70" s="91"/>
+      <c r="D70" s="121"/>
+      <c r="E70" s="124"/>
+      <c r="G70" s="118"/>
+      <c r="H70" s="130"/>
+      <c r="I70" s="130"/>
+      <c r="J70" s="118"/>
       <c r="L70" s="100"/>
-      <c r="M70" s="103"/>
-      <c r="N70" s="103"/>
+      <c r="M70" s="127"/>
+      <c r="N70" s="127"/>
       <c r="O70" s="100"/>
-      <c r="Q70" s="109"/>
-      <c r="R70" s="109"/>
-      <c r="S70" s="109"/>
+      <c r="Q70" s="133"/>
+      <c r="R70" s="133"/>
+      <c r="S70" s="133"/>
     </row>
     <row r="71" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D71" s="94"/>
-      <c r="E71" s="97"/>
-      <c r="G71" s="91"/>
-      <c r="H71" s="106"/>
-      <c r="I71" s="106"/>
-      <c r="J71" s="91"/>
+      <c r="D71" s="121"/>
+      <c r="E71" s="124"/>
+      <c r="G71" s="118"/>
+      <c r="H71" s="130"/>
+      <c r="I71" s="130"/>
+      <c r="J71" s="118"/>
       <c r="L71" s="100"/>
-      <c r="M71" s="103"/>
-      <c r="N71" s="103"/>
+      <c r="M71" s="127"/>
+      <c r="N71" s="127"/>
       <c r="O71" s="100"/>
-      <c r="Q71" s="109"/>
-      <c r="R71" s="109"/>
-      <c r="S71" s="109"/>
+      <c r="Q71" s="133"/>
+      <c r="R71" s="133"/>
+      <c r="S71" s="133"/>
     </row>
     <row r="72" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D72" s="94"/>
-      <c r="E72" s="97"/>
-      <c r="G72" s="91"/>
-      <c r="H72" s="106"/>
-      <c r="I72" s="106"/>
-      <c r="J72" s="91"/>
+      <c r="D72" s="121"/>
+      <c r="E72" s="124"/>
+      <c r="G72" s="118"/>
+      <c r="H72" s="130"/>
+      <c r="I72" s="130"/>
+      <c r="J72" s="118"/>
       <c r="L72" s="100"/>
-      <c r="M72" s="103"/>
-      <c r="N72" s="103"/>
+      <c r="M72" s="127"/>
+      <c r="N72" s="127"/>
       <c r="O72" s="100"/>
-      <c r="Q72" s="109"/>
-      <c r="R72" s="109"/>
-      <c r="S72" s="109"/>
+      <c r="Q72" s="133"/>
+      <c r="R72" s="133"/>
+      <c r="S72" s="133"/>
     </row>
     <row r="73" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D73" s="94"/>
-      <c r="E73" s="97"/>
-      <c r="G73" s="91"/>
-      <c r="H73" s="106"/>
-      <c r="I73" s="106"/>
-      <c r="J73" s="91"/>
+      <c r="D73" s="121"/>
+      <c r="E73" s="124"/>
+      <c r="G73" s="118"/>
+      <c r="H73" s="130"/>
+      <c r="I73" s="130"/>
+      <c r="J73" s="118"/>
       <c r="L73" s="100"/>
-      <c r="M73" s="103"/>
-      <c r="N73" s="103"/>
+      <c r="M73" s="127"/>
+      <c r="N73" s="127"/>
       <c r="O73" s="100"/>
-      <c r="Q73" s="109"/>
-      <c r="R73" s="109"/>
-      <c r="S73" s="109"/>
+      <c r="Q73" s="133"/>
+      <c r="R73" s="133"/>
+      <c r="S73" s="133"/>
     </row>
     <row r="74" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D74" s="94"/>
-      <c r="E74" s="97"/>
-      <c r="G74" s="91"/>
-      <c r="H74" s="106"/>
-      <c r="I74" s="106"/>
-      <c r="J74" s="91"/>
+      <c r="D74" s="121"/>
+      <c r="E74" s="124"/>
+      <c r="G74" s="118"/>
+      <c r="H74" s="130"/>
+      <c r="I74" s="130"/>
+      <c r="J74" s="118"/>
       <c r="L74" s="100"/>
-      <c r="M74" s="103"/>
-      <c r="N74" s="103"/>
+      <c r="M74" s="127"/>
+      <c r="N74" s="127"/>
       <c r="O74" s="100"/>
-      <c r="Q74" s="109"/>
-      <c r="R74" s="109"/>
-      <c r="S74" s="109"/>
+      <c r="Q74" s="133"/>
+      <c r="R74" s="133"/>
+      <c r="S74" s="133"/>
     </row>
     <row r="75" spans="1:20" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D75" s="95"/>
-      <c r="E75" s="98"/>
-      <c r="G75" s="92"/>
-      <c r="H75" s="107"/>
-      <c r="I75" s="107"/>
-      <c r="J75" s="92"/>
+      <c r="D75" s="122"/>
+      <c r="E75" s="125"/>
+      <c r="G75" s="119"/>
+      <c r="H75" s="131"/>
+      <c r="I75" s="131"/>
+      <c r="J75" s="119"/>
       <c r="L75" s="101"/>
-      <c r="M75" s="104"/>
-      <c r="N75" s="104"/>
+      <c r="M75" s="128"/>
+      <c r="N75" s="128"/>
       <c r="O75" s="101"/>
-      <c r="Q75" s="110"/>
-      <c r="R75" s="110"/>
-      <c r="S75" s="110"/>
+      <c r="Q75" s="134"/>
+      <c r="R75" s="134"/>
+      <c r="S75" s="134"/>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B6:T60">
     <sortCondition ref="B6"/>
   </sortState>
   <mergeCells count="25">
-    <mergeCell ref="G2:K2"/>
-    <mergeCell ref="D2:F2"/>
-    <mergeCell ref="Q3:T4"/>
-    <mergeCell ref="O66:O75"/>
-    <mergeCell ref="A2:A5"/>
-    <mergeCell ref="G3:K4"/>
-    <mergeCell ref="D3:F4"/>
-    <mergeCell ref="B2:B5"/>
-    <mergeCell ref="C2:C5"/>
     <mergeCell ref="B1:T1"/>
     <mergeCell ref="J66:J75"/>
     <mergeCell ref="D66:D75"/>
@@ -7667,6 +7664,15 @@
     <mergeCell ref="I66:I75"/>
     <mergeCell ref="Q2:T2"/>
     <mergeCell ref="L2:P2"/>
+    <mergeCell ref="G2:K2"/>
+    <mergeCell ref="D2:F2"/>
+    <mergeCell ref="Q3:T4"/>
+    <mergeCell ref="O66:O75"/>
+    <mergeCell ref="A2:A5"/>
+    <mergeCell ref="G3:K4"/>
+    <mergeCell ref="D3:F4"/>
+    <mergeCell ref="B2:B5"/>
+    <mergeCell ref="C2:C5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
gestión de datos para diagnostico uniciado
</commit_message>
<xml_diff>
--- a/9_asistencia_evaluacion/pivu_caucasia_notas_quices_asistencia.xlsx
+++ b/9_asistencia_evaluacion/pivu_caucasia_notas_quices_asistencia.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marco\Documentos\extension\camino-udea\9_asistencia_evaluacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{056D1C83-67BA-4B54-A0A9-0A1164B86189}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C51AA121-A4C0-4B93-A344-E4CAD4B441A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1025,6 +1025,12 @@
     <xf numFmtId="0" fontId="28" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="22" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="19" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1127,11 +1133,89 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1160,15 +1244,6 @@
     <xf numFmtId="0" fontId="3" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1209,81 +1284,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1767,7 +1767,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I41"/>
+  <dimension ref="A1:I38"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.109375" style="38" bestFit="1" customWidth="1"/>
@@ -1783,28 +1783,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="72" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="92" t="s">
+      <c r="A1" s="58" t="s">
         <v>27</v>
       </c>
-      <c r="B1" s="91"/>
-      <c r="C1" s="91"/>
-      <c r="D1" s="91"/>
-      <c r="E1" s="91"/>
-      <c r="F1" s="91"/>
-      <c r="G1" s="91"/>
-      <c r="H1" s="91"/>
+      <c r="B1" s="57"/>
+      <c r="C1" s="57"/>
+      <c r="D1" s="57"/>
+      <c r="E1" s="57"/>
+      <c r="F1" s="57"/>
+      <c r="G1" s="57"/>
+      <c r="H1" s="57"/>
     </row>
     <row r="2" spans="1:9" ht="19.8" x14ac:dyDescent="0.3">
-      <c r="A2" s="91" t="s">
+      <c r="A2" s="57" t="s">
         <v>26</v>
       </c>
-      <c r="B2" s="91"/>
-      <c r="C2" s="91"/>
-      <c r="D2" s="91"/>
-      <c r="E2" s="91"/>
-      <c r="F2" s="91"/>
-      <c r="G2" s="91"/>
-      <c r="H2" s="91"/>
+      <c r="B2" s="57"/>
+      <c r="C2" s="57"/>
+      <c r="D2" s="57"/>
+      <c r="E2" s="57"/>
+      <c r="F2" s="57"/>
+      <c r="G2" s="57"/>
+      <c r="H2" s="57"/>
       <c r="I2" s="50" t="s">
         <v>99</v>
       </c>
@@ -2536,7 +2536,7 @@
       </c>
       <c r="H32" s="44"/>
     </row>
-    <row r="33" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:9" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="42">
         <v>30</v>
       </c>
@@ -2560,7 +2560,7 @@
       </c>
       <c r="H33" s="44"/>
     </row>
-    <row r="34" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:9" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="42">
         <v>31</v>
       </c>
@@ -2584,7 +2584,7 @@
       </c>
       <c r="H34" s="44"/>
     </row>
-    <row r="35" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:9" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="42">
         <v>32</v>
       </c>
@@ -2608,7 +2608,7 @@
       </c>
       <c r="H35" s="44"/>
     </row>
-    <row r="36" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:9" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="42">
         <v>33</v>
       </c>
@@ -2632,7 +2632,7 @@
       </c>
       <c r="H36" s="44"/>
     </row>
-    <row r="37" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:9" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="42">
         <v>34</v>
       </c>
@@ -2655,8 +2655,11 @@
         <v>59</v>
       </c>
       <c r="H37" s="44"/>
-    </row>
-    <row r="38" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="I37" s="45" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="42">
         <v>35</v>
       </c>
@@ -2679,18 +2682,8 @@
         <v>102</v>
       </c>
       <c r="H38" s="44"/>
-    </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A39" s="38">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="B41" s="45" t="s">
+      <c r="I38" s="45" t="s">
         <v>106</v>
-      </c>
-      <c r="C41" s="45" t="s">
-        <v>107</v>
       </c>
     </row>
   </sheetData>
@@ -2733,172 +2726,172 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:31" ht="66" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B1" s="64" t="s">
+      <c r="B1" s="66" t="s">
         <v>18</v>
       </c>
-      <c r="C1" s="64"/>
-      <c r="D1" s="64"/>
-      <c r="E1" s="64"/>
-      <c r="F1" s="64"/>
-      <c r="G1" s="64"/>
-      <c r="H1" s="64"/>
-      <c r="I1" s="64"/>
-      <c r="J1" s="64"/>
-      <c r="K1" s="64"/>
-      <c r="L1" s="64"/>
-      <c r="M1" s="64"/>
-      <c r="N1" s="64"/>
-      <c r="O1" s="64"/>
-      <c r="P1" s="64"/>
-      <c r="Q1" s="64"/>
-      <c r="R1" s="64"/>
-      <c r="S1" s="64"/>
-      <c r="T1" s="64"/>
-      <c r="U1" s="64"/>
-      <c r="V1" s="64"/>
-      <c r="W1" s="64"/>
-      <c r="X1" s="64"/>
-      <c r="Y1" s="64"/>
-      <c r="Z1" s="64"/>
-      <c r="AA1" s="64"/>
-      <c r="AB1" s="64"/>
-      <c r="AC1" s="64"/>
-      <c r="AD1" s="64"/>
-      <c r="AE1" s="64"/>
+      <c r="C1" s="66"/>
+      <c r="D1" s="66"/>
+      <c r="E1" s="66"/>
+      <c r="F1" s="66"/>
+      <c r="G1" s="66"/>
+      <c r="H1" s="66"/>
+      <c r="I1" s="66"/>
+      <c r="J1" s="66"/>
+      <c r="K1" s="66"/>
+      <c r="L1" s="66"/>
+      <c r="M1" s="66"/>
+      <c r="N1" s="66"/>
+      <c r="O1" s="66"/>
+      <c r="P1" s="66"/>
+      <c r="Q1" s="66"/>
+      <c r="R1" s="66"/>
+      <c r="S1" s="66"/>
+      <c r="T1" s="66"/>
+      <c r="U1" s="66"/>
+      <c r="V1" s="66"/>
+      <c r="W1" s="66"/>
+      <c r="X1" s="66"/>
+      <c r="Y1" s="66"/>
+      <c r="Z1" s="66"/>
+      <c r="AA1" s="66"/>
+      <c r="AB1" s="66"/>
+      <c r="AC1" s="66"/>
+      <c r="AD1" s="66"/>
+      <c r="AE1" s="66"/>
     </row>
     <row r="2" spans="1:31" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="65" t="s">
+      <c r="A2" s="67" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="89" t="s">
+      <c r="B2" s="91" t="s">
         <v>21</v>
       </c>
-      <c r="C2" s="65" t="s">
+      <c r="C2" s="67" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="82" t="s">
+      <c r="D2" s="84" t="s">
         <v>19</v>
       </c>
-      <c r="E2" s="83"/>
-      <c r="F2" s="83"/>
-      <c r="G2" s="83"/>
-      <c r="H2" s="84"/>
-      <c r="I2" s="67" t="s">
+      <c r="E2" s="85"/>
+      <c r="F2" s="85"/>
+      <c r="G2" s="85"/>
+      <c r="H2" s="86"/>
+      <c r="I2" s="69" t="s">
         <v>19</v>
       </c>
-      <c r="J2" s="68"/>
-      <c r="K2" s="68"/>
-      <c r="L2" s="68"/>
-      <c r="M2" s="68"/>
-      <c r="N2" s="68"/>
-      <c r="O2" s="68"/>
-      <c r="P2" s="68"/>
-      <c r="Q2" s="69"/>
-      <c r="R2" s="76" t="s">
+      <c r="J2" s="70"/>
+      <c r="K2" s="70"/>
+      <c r="L2" s="70"/>
+      <c r="M2" s="70"/>
+      <c r="N2" s="70"/>
+      <c r="O2" s="70"/>
+      <c r="P2" s="70"/>
+      <c r="Q2" s="71"/>
+      <c r="R2" s="78" t="s">
         <v>19</v>
       </c>
-      <c r="S2" s="77"/>
-      <c r="T2" s="77"/>
-      <c r="U2" s="77"/>
-      <c r="V2" s="77"/>
-      <c r="W2" s="77"/>
-      <c r="X2" s="77"/>
-      <c r="Y2" s="77"/>
-      <c r="Z2" s="78"/>
-      <c r="AA2" s="57" t="s">
+      <c r="S2" s="79"/>
+      <c r="T2" s="79"/>
+      <c r="U2" s="79"/>
+      <c r="V2" s="79"/>
+      <c r="W2" s="79"/>
+      <c r="X2" s="79"/>
+      <c r="Y2" s="79"/>
+      <c r="Z2" s="80"/>
+      <c r="AA2" s="59" t="s">
         <v>19</v>
       </c>
-      <c r="AB2" s="58"/>
-      <c r="AC2" s="58"/>
-      <c r="AD2" s="58"/>
-      <c r="AE2" s="59"/>
+      <c r="AB2" s="60"/>
+      <c r="AC2" s="60"/>
+      <c r="AD2" s="60"/>
+      <c r="AE2" s="61"/>
     </row>
     <row r="3" spans="1:31" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="66"/>
-      <c r="B3" s="90"/>
-      <c r="C3" s="66"/>
-      <c r="D3" s="85" t="s">
+      <c r="A3" s="68"/>
+      <c r="B3" s="92"/>
+      <c r="C3" s="68"/>
+      <c r="D3" s="87" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="86"/>
-      <c r="F3" s="86"/>
-      <c r="G3" s="86"/>
-      <c r="H3" s="87"/>
-      <c r="I3" s="70" t="s">
+      <c r="E3" s="88"/>
+      <c r="F3" s="88"/>
+      <c r="G3" s="88"/>
+      <c r="H3" s="89"/>
+      <c r="I3" s="72" t="s">
         <v>2</v>
       </c>
-      <c r="J3" s="71"/>
-      <c r="K3" s="71"/>
-      <c r="L3" s="71"/>
-      <c r="M3" s="71"/>
-      <c r="N3" s="71"/>
-      <c r="O3" s="71"/>
-      <c r="P3" s="71"/>
-      <c r="Q3" s="72"/>
-      <c r="R3" s="79" t="s">
+      <c r="J3" s="73"/>
+      <c r="K3" s="73"/>
+      <c r="L3" s="73"/>
+      <c r="M3" s="73"/>
+      <c r="N3" s="73"/>
+      <c r="O3" s="73"/>
+      <c r="P3" s="73"/>
+      <c r="Q3" s="74"/>
+      <c r="R3" s="81" t="s">
         <v>1</v>
       </c>
-      <c r="S3" s="80"/>
-      <c r="T3" s="80"/>
-      <c r="U3" s="80"/>
-      <c r="V3" s="80"/>
-      <c r="W3" s="80"/>
-      <c r="X3" s="80"/>
-      <c r="Y3" s="80"/>
-      <c r="Z3" s="81"/>
-      <c r="AA3" s="60" t="s">
-        <v>0</v>
-      </c>
-      <c r="AB3" s="61"/>
-      <c r="AC3" s="61"/>
-      <c r="AD3" s="61"/>
-      <c r="AE3" s="62"/>
+      <c r="S3" s="82"/>
+      <c r="T3" s="82"/>
+      <c r="U3" s="82"/>
+      <c r="V3" s="82"/>
+      <c r="W3" s="82"/>
+      <c r="X3" s="82"/>
+      <c r="Y3" s="82"/>
+      <c r="Z3" s="83"/>
+      <c r="AA3" s="62" t="s">
+        <v>0</v>
+      </c>
+      <c r="AB3" s="63"/>
+      <c r="AC3" s="63"/>
+      <c r="AD3" s="63"/>
+      <c r="AE3" s="64"/>
     </row>
     <row r="4" spans="1:31" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="66"/>
-      <c r="B4" s="90"/>
-      <c r="C4" s="66"/>
-      <c r="D4" s="88" t="s">
+      <c r="A4" s="68"/>
+      <c r="B4" s="92"/>
+      <c r="C4" s="68"/>
+      <c r="D4" s="90" t="s">
         <v>22</v>
       </c>
-      <c r="E4" s="74"/>
-      <c r="F4" s="74"/>
-      <c r="G4" s="75"/>
+      <c r="E4" s="76"/>
+      <c r="F4" s="76"/>
+      <c r="G4" s="77"/>
       <c r="H4" s="1"/>
-      <c r="I4" s="73" t="s">
+      <c r="I4" s="75" t="s">
         <v>23</v>
       </c>
-      <c r="J4" s="74"/>
-      <c r="K4" s="74"/>
-      <c r="L4" s="74"/>
-      <c r="M4" s="74"/>
-      <c r="N4" s="74"/>
-      <c r="O4" s="74"/>
-      <c r="P4" s="75"/>
+      <c r="J4" s="76"/>
+      <c r="K4" s="76"/>
+      <c r="L4" s="76"/>
+      <c r="M4" s="76"/>
+      <c r="N4" s="76"/>
+      <c r="O4" s="76"/>
+      <c r="P4" s="77"/>
       <c r="Q4" s="3"/>
-      <c r="R4" s="73" t="s">
+      <c r="R4" s="75" t="s">
         <v>23</v>
       </c>
-      <c r="S4" s="74"/>
-      <c r="T4" s="74"/>
-      <c r="U4" s="74"/>
-      <c r="V4" s="74"/>
-      <c r="W4" s="74"/>
-      <c r="X4" s="74"/>
-      <c r="Y4" s="75"/>
+      <c r="S4" s="76"/>
+      <c r="T4" s="76"/>
+      <c r="U4" s="76"/>
+      <c r="V4" s="76"/>
+      <c r="W4" s="76"/>
+      <c r="X4" s="76"/>
+      <c r="Y4" s="77"/>
       <c r="Z4" s="12"/>
-      <c r="AA4" s="63" t="s">
+      <c r="AA4" s="65" t="s">
         <v>23</v>
       </c>
-      <c r="AB4" s="63"/>
-      <c r="AC4" s="63"/>
-      <c r="AD4" s="63"/>
+      <c r="AB4" s="65"/>
+      <c r="AC4" s="65"/>
+      <c r="AD4" s="65"/>
       <c r="AE4" s="3"/>
     </row>
     <row r="5" spans="1:31" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="66"/>
-      <c r="B5" s="90"/>
-      <c r="C5" s="66"/>
+      <c r="A5" s="68"/>
+      <c r="B5" s="92"/>
+      <c r="C5" s="68"/>
       <c r="D5" s="28" t="s">
         <v>100</v>
       </c>
@@ -4820,123 +4813,123 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="72.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B1" s="119" t="s">
+      <c r="B1" s="93" t="s">
         <v>18</v>
       </c>
-      <c r="C1" s="119"/>
-      <c r="D1" s="119"/>
-      <c r="E1" s="119"/>
-      <c r="F1" s="119"/>
-      <c r="G1" s="119"/>
-      <c r="H1" s="119"/>
-      <c r="I1" s="119"/>
-      <c r="J1" s="119"/>
-      <c r="K1" s="119"/>
-      <c r="L1" s="119"/>
-      <c r="M1" s="119"/>
-      <c r="N1" s="119"/>
-      <c r="O1" s="119"/>
-      <c r="P1" s="119"/>
-      <c r="Q1" s="119"/>
-      <c r="R1" s="119"/>
-      <c r="S1" s="119"/>
-      <c r="T1" s="119"/>
+      <c r="C1" s="93"/>
+      <c r="D1" s="93"/>
+      <c r="E1" s="93"/>
+      <c r="F1" s="93"/>
+      <c r="G1" s="93"/>
+      <c r="H1" s="93"/>
+      <c r="I1" s="93"/>
+      <c r="J1" s="93"/>
+      <c r="K1" s="93"/>
+      <c r="L1" s="93"/>
+      <c r="M1" s="93"/>
+      <c r="N1" s="93"/>
+      <c r="O1" s="93"/>
+      <c r="P1" s="93"/>
+      <c r="Q1" s="93"/>
+      <c r="R1" s="93"/>
+      <c r="S1" s="93"/>
+      <c r="T1" s="93"/>
     </row>
     <row r="2" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="105" t="s">
+      <c r="A2" s="130" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="89" t="s">
+      <c r="B2" s="91" t="s">
         <v>21</v>
       </c>
-      <c r="C2" s="65" t="s">
+      <c r="C2" s="67" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="93" t="str">
+      <c r="D2" s="121" t="str">
         <f>Asistencia!D2</f>
         <v>NOMBRE DOCENTE</v>
       </c>
-      <c r="E2" s="94"/>
-      <c r="F2" s="95"/>
-      <c r="G2" s="93" t="str">
+      <c r="E2" s="122"/>
+      <c r="F2" s="123"/>
+      <c r="G2" s="121" t="str">
         <f>Asistencia!I2</f>
         <v>NOMBRE DOCENTE</v>
       </c>
-      <c r="H2" s="94"/>
-      <c r="I2" s="94"/>
-      <c r="J2" s="94"/>
-      <c r="K2" s="95"/>
-      <c r="L2" s="93" t="s">
+      <c r="H2" s="122"/>
+      <c r="I2" s="122"/>
+      <c r="J2" s="122"/>
+      <c r="K2" s="123"/>
+      <c r="L2" s="121" t="s">
         <v>19</v>
       </c>
-      <c r="M2" s="94"/>
-      <c r="N2" s="94"/>
-      <c r="O2" s="94"/>
-      <c r="P2" s="95"/>
-      <c r="Q2" s="93" t="str">
+      <c r="M2" s="122"/>
+      <c r="N2" s="122"/>
+      <c r="O2" s="122"/>
+      <c r="P2" s="123"/>
+      <c r="Q2" s="121" t="str">
         <f>Asistencia!AA2</f>
         <v>NOMBRE DOCENTE</v>
       </c>
-      <c r="R2" s="94"/>
-      <c r="S2" s="94"/>
-      <c r="T2" s="95"/>
+      <c r="R2" s="122"/>
+      <c r="S2" s="122"/>
+      <c r="T2" s="123"/>
     </row>
     <row r="3" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="106"/>
-      <c r="B3" s="90"/>
-      <c r="C3" s="66"/>
-      <c r="D3" s="113" t="s">
+      <c r="A3" s="131"/>
+      <c r="B3" s="92"/>
+      <c r="C3" s="68"/>
+      <c r="D3" s="138" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="114"/>
-      <c r="F3" s="115"/>
-      <c r="G3" s="107" t="s">
+      <c r="E3" s="139"/>
+      <c r="F3" s="140"/>
+      <c r="G3" s="132" t="s">
         <v>2</v>
       </c>
-      <c r="H3" s="108"/>
-      <c r="I3" s="108"/>
-      <c r="J3" s="108"/>
-      <c r="K3" s="109"/>
-      <c r="L3" s="138" t="s">
+      <c r="H3" s="133"/>
+      <c r="I3" s="133"/>
+      <c r="J3" s="133"/>
+      <c r="K3" s="134"/>
+      <c r="L3" s="115" t="s">
         <v>1</v>
       </c>
-      <c r="M3" s="139"/>
-      <c r="N3" s="139"/>
-      <c r="O3" s="139"/>
-      <c r="P3" s="140"/>
-      <c r="Q3" s="96" t="s">
-        <v>0</v>
-      </c>
-      <c r="R3" s="97"/>
-      <c r="S3" s="97"/>
-      <c r="T3" s="98"/>
+      <c r="M3" s="116"/>
+      <c r="N3" s="116"/>
+      <c r="O3" s="116"/>
+      <c r="P3" s="117"/>
+      <c r="Q3" s="124" t="s">
+        <v>0</v>
+      </c>
+      <c r="R3" s="125"/>
+      <c r="S3" s="125"/>
+      <c r="T3" s="126"/>
     </row>
     <row r="4" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="106"/>
-      <c r="B4" s="90"/>
-      <c r="C4" s="66"/>
-      <c r="D4" s="116"/>
-      <c r="E4" s="117"/>
-      <c r="F4" s="118"/>
-      <c r="G4" s="110"/>
-      <c r="H4" s="111"/>
-      <c r="I4" s="111"/>
-      <c r="J4" s="111"/>
-      <c r="K4" s="112"/>
-      <c r="L4" s="141"/>
-      <c r="M4" s="142"/>
-      <c r="N4" s="142"/>
-      <c r="O4" s="142"/>
-      <c r="P4" s="143"/>
-      <c r="Q4" s="99"/>
-      <c r="R4" s="100"/>
-      <c r="S4" s="100"/>
-      <c r="T4" s="101"/>
+      <c r="A4" s="131"/>
+      <c r="B4" s="92"/>
+      <c r="C4" s="68"/>
+      <c r="D4" s="141"/>
+      <c r="E4" s="142"/>
+      <c r="F4" s="143"/>
+      <c r="G4" s="135"/>
+      <c r="H4" s="136"/>
+      <c r="I4" s="136"/>
+      <c r="J4" s="136"/>
+      <c r="K4" s="137"/>
+      <c r="L4" s="118"/>
+      <c r="M4" s="119"/>
+      <c r="N4" s="119"/>
+      <c r="O4" s="119"/>
+      <c r="P4" s="120"/>
+      <c r="Q4" s="127"/>
+      <c r="R4" s="128"/>
+      <c r="S4" s="128"/>
+      <c r="T4" s="129"/>
     </row>
     <row r="5" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="106"/>
-      <c r="B5" s="90"/>
-      <c r="C5" s="66"/>
+      <c r="A5" s="131"/>
+      <c r="B5" s="92"/>
+      <c r="C5" s="68"/>
       <c r="D5" s="17">
         <v>0.75</v>
       </c>
@@ -6463,13 +6456,13 @@
       <c r="A41" s="10">
         <v>36</v>
       </c>
-      <c r="B41" s="14">
-        <f>Inscritos!B39</f>
-        <v>0</v>
-      </c>
-      <c r="C41" s="14">
-        <f>+Inscritos!D39</f>
-        <v>0</v>
+      <c r="B41" s="14" t="e">
+        <f>Inscritos!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="C41" s="14" t="e">
+        <f>+Inscritos!#REF!</f>
+        <v>#REF!</v>
       </c>
       <c r="D41" s="7"/>
       <c r="E41" s="7"/>
@@ -6505,13 +6498,13 @@
       <c r="A42" s="10">
         <v>37</v>
       </c>
-      <c r="B42" s="14">
-        <f>Inscritos!B40</f>
-        <v>0</v>
-      </c>
-      <c r="C42" s="14">
-        <f>+Inscritos!D40</f>
-        <v>0</v>
+      <c r="B42" s="14" t="e">
+        <f>Inscritos!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="C42" s="14" t="e">
+        <f>+Inscritos!#REF!</f>
+        <v>#REF!</v>
       </c>
       <c r="D42" s="7"/>
       <c r="E42" s="7"/>
@@ -6548,11 +6541,11 @@
         <v>38</v>
       </c>
       <c r="B43" s="14" t="str">
-        <f>Inscritos!B41</f>
+        <f>Inscritos!I38</f>
         <v>Vinculo para reportar resultados del PIVU</v>
       </c>
       <c r="C43" s="14">
-        <f>+Inscritos!D41</f>
+        <f>+Inscritos!D39</f>
         <v>0</v>
       </c>
       <c r="D43" s="7"/>
@@ -6590,11 +6583,11 @@
         <v>39</v>
       </c>
       <c r="B44" s="14">
-        <f>Inscritos!B42</f>
+        <f>Inscritos!B40</f>
         <v>0</v>
       </c>
       <c r="C44" s="14">
-        <f>+Inscritos!D42</f>
+        <f>+Inscritos!D40</f>
         <v>0</v>
       </c>
       <c r="D44" s="7"/>
@@ -6632,11 +6625,11 @@
         <v>40</v>
       </c>
       <c r="B45" s="14">
-        <f>Inscritos!B43</f>
+        <f>Inscritos!B41</f>
         <v>0</v>
       </c>
       <c r="C45" s="14">
-        <f>+Inscritos!D43</f>
+        <f>+Inscritos!D41</f>
         <v>0</v>
       </c>
       <c r="D45" s="7"/>
@@ -6674,11 +6667,11 @@
         <v>41</v>
       </c>
       <c r="B46" s="14">
-        <f>Inscritos!B44</f>
+        <f>Inscritos!B42</f>
         <v>0</v>
       </c>
       <c r="C46" s="14">
-        <f>+Inscritos!D44</f>
+        <f>+Inscritos!D42</f>
         <v>0</v>
       </c>
       <c r="D46" s="7"/>
@@ -6716,11 +6709,11 @@
         <v>42</v>
       </c>
       <c r="B47" s="14">
-        <f>Inscritos!B45</f>
+        <f>Inscritos!B43</f>
         <v>0</v>
       </c>
       <c r="C47" s="14">
-        <f>+Inscritos!D45</f>
+        <f>+Inscritos!D43</f>
         <v>0</v>
       </c>
       <c r="D47" s="7"/>
@@ -6758,11 +6751,11 @@
         <v>43</v>
       </c>
       <c r="B48" s="14">
-        <f>Inscritos!B46</f>
+        <f>Inscritos!B44</f>
         <v>0</v>
       </c>
       <c r="C48" s="14">
-        <f>+Inscritos!D46</f>
+        <f>+Inscritos!D44</f>
         <v>0</v>
       </c>
       <c r="D48" s="7"/>
@@ -6800,11 +6793,11 @@
         <v>44</v>
       </c>
       <c r="B49" s="14">
-        <f>Inscritos!B47</f>
+        <f>Inscritos!B45</f>
         <v>0</v>
       </c>
       <c r="C49" s="14">
-        <f>+Inscritos!D47</f>
+        <f>+Inscritos!D45</f>
         <v>0</v>
       </c>
       <c r="D49" s="7"/>
@@ -6842,11 +6835,11 @@
         <v>45</v>
       </c>
       <c r="B50" s="14">
-        <f>Inscritos!B48</f>
+        <f>Inscritos!B46</f>
         <v>0</v>
       </c>
       <c r="C50" s="14">
-        <f>+Inscritos!D48</f>
+        <f>+Inscritos!D46</f>
         <v>0</v>
       </c>
       <c r="D50" s="7"/>
@@ -6884,11 +6877,11 @@
         <v>46</v>
       </c>
       <c r="B51" s="14">
-        <f>Inscritos!B49</f>
+        <f>Inscritos!B47</f>
         <v>0</v>
       </c>
       <c r="C51" s="14">
-        <f>+Inscritos!D49</f>
+        <f>+Inscritos!D47</f>
         <v>0</v>
       </c>
       <c r="D51" s="7"/>
@@ -6926,11 +6919,11 @@
         <v>47</v>
       </c>
       <c r="B52" s="14">
-        <f>Inscritos!B50</f>
+        <f>Inscritos!B48</f>
         <v>0</v>
       </c>
       <c r="C52" s="14">
-        <f>+Inscritos!D50</f>
+        <f>+Inscritos!D48</f>
         <v>0</v>
       </c>
       <c r="D52" s="7"/>
@@ -6968,11 +6961,11 @@
         <v>48</v>
       </c>
       <c r="B53" s="14">
-        <f>Inscritos!B51</f>
+        <f>Inscritos!B49</f>
         <v>0</v>
       </c>
       <c r="C53" s="14">
-        <f>+Inscritos!D51</f>
+        <f>+Inscritos!D49</f>
         <v>0</v>
       </c>
       <c r="D53" s="7"/>
@@ -7010,11 +7003,11 @@
         <v>49</v>
       </c>
       <c r="B54" s="14">
-        <f>Inscritos!B52</f>
+        <f>Inscritos!B50</f>
         <v>0</v>
       </c>
       <c r="C54" s="14">
-        <f>+Inscritos!D52</f>
+        <f>+Inscritos!D50</f>
         <v>0</v>
       </c>
       <c r="D54" s="7"/>
@@ -7052,11 +7045,11 @@
         <v>50</v>
       </c>
       <c r="B55" s="14">
-        <f>Inscritos!B53</f>
+        <f>Inscritos!B51</f>
         <v>0</v>
       </c>
       <c r="C55" s="14">
-        <f>+Inscritos!D53</f>
+        <f>+Inscritos!D51</f>
         <v>0</v>
       </c>
       <c r="D55" s="7"/>
@@ -7094,11 +7087,11 @@
         <v>51</v>
       </c>
       <c r="B56" s="14">
-        <f>Inscritos!B54</f>
+        <f>Inscritos!B52</f>
         <v>0</v>
       </c>
       <c r="C56" s="14">
-        <f>+Inscritos!D54</f>
+        <f>+Inscritos!D52</f>
         <v>0</v>
       </c>
       <c r="D56" s="7"/>
@@ -7136,11 +7129,11 @@
         <v>52</v>
       </c>
       <c r="B57" s="14">
-        <f>Inscritos!B55</f>
+        <f>Inscritos!B53</f>
         <v>0</v>
       </c>
       <c r="C57" s="14">
-        <f>+Inscritos!D55</f>
+        <f>+Inscritos!D53</f>
         <v>0</v>
       </c>
       <c r="D57" s="7"/>
@@ -7178,11 +7171,11 @@
         <v>53</v>
       </c>
       <c r="B58" s="14">
-        <f>Inscritos!B56</f>
+        <f>Inscritos!B54</f>
         <v>0</v>
       </c>
       <c r="C58" s="14">
-        <f>+Inscritos!D56</f>
+        <f>+Inscritos!D54</f>
         <v>0</v>
       </c>
       <c r="D58" s="7"/>
@@ -7220,11 +7213,11 @@
         <v>54</v>
       </c>
       <c r="B59" s="14">
-        <f>Inscritos!B57</f>
+        <f>Inscritos!B55</f>
         <v>0</v>
       </c>
       <c r="C59" s="14">
-        <f>+Inscritos!D57</f>
+        <f>+Inscritos!D55</f>
         <v>0</v>
       </c>
       <c r="D59" s="7"/>
@@ -7262,11 +7255,11 @@
         <v>55</v>
       </c>
       <c r="B60" s="14">
-        <f>Inscritos!B58</f>
+        <f>Inscritos!B56</f>
         <v>0</v>
       </c>
       <c r="C60" s="14">
-        <f>+Inscritos!D58</f>
+        <f>+Inscritos!D56</f>
         <v>0</v>
       </c>
       <c r="D60" s="7"/>
@@ -7304,11 +7297,11 @@
         <v>56</v>
       </c>
       <c r="B61" s="14">
-        <f>Inscritos!B59</f>
+        <f>Inscritos!B57</f>
         <v>0</v>
       </c>
       <c r="C61" s="14">
-        <f>+Inscritos!D59</f>
+        <f>+Inscritos!D57</f>
         <v>0</v>
       </c>
       <c r="D61" s="7"/>
@@ -7346,11 +7339,11 @@
         <v>57</v>
       </c>
       <c r="B62" s="14">
-        <f>Inscritos!B60</f>
+        <f>Inscritos!B58</f>
         <v>0</v>
       </c>
       <c r="C62" s="14">
-        <f>+Inscritos!D60</f>
+        <f>+Inscritos!D58</f>
         <v>0</v>
       </c>
       <c r="D62" s="7"/>
@@ -7388,11 +7381,11 @@
         <v>58</v>
       </c>
       <c r="B63" s="14">
-        <f>Inscritos!B61</f>
+        <f>Inscritos!B59</f>
         <v>0</v>
       </c>
       <c r="C63" s="14">
-        <f>+Inscritos!D61</f>
+        <f>+Inscritos!D59</f>
         <v>0</v>
       </c>
       <c r="D63" s="7"/>
@@ -7430,11 +7423,11 @@
         <v>59</v>
       </c>
       <c r="B64" s="14">
-        <f>Inscritos!B62</f>
+        <f>Inscritos!B60</f>
         <v>0</v>
       </c>
       <c r="C64" s="14">
-        <f>+Inscritos!D62</f>
+        <f>+Inscritos!D60</f>
         <v>0</v>
       </c>
       <c r="D64" s="7"/>
@@ -7472,11 +7465,11 @@
         <v>60</v>
       </c>
       <c r="B65" s="14">
-        <f>Inscritos!B63</f>
+        <f>Inscritos!B61</f>
         <v>0</v>
       </c>
       <c r="C65" s="14">
-        <f>+Inscritos!D63</f>
+        <f>+Inscritos!D61</f>
         <v>0</v>
       </c>
       <c r="D65" s="7"/>
@@ -7510,186 +7503,195 @@
       </c>
     </row>
     <row r="66" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D66" s="123" t="s">
+      <c r="D66" s="97" t="s">
         <v>24</v>
       </c>
-      <c r="E66" s="126" t="s">
+      <c r="E66" s="100" t="s">
         <v>12</v>
       </c>
-      <c r="G66" s="120" t="s">
+      <c r="G66" s="94" t="s">
         <v>8</v>
       </c>
-      <c r="H66" s="132" t="s">
+      <c r="H66" s="109" t="s">
         <v>9</v>
       </c>
-      <c r="I66" s="132" t="s">
+      <c r="I66" s="109" t="s">
         <v>10</v>
       </c>
-      <c r="J66" s="120" t="s">
+      <c r="J66" s="94" t="s">
         <v>11</v>
       </c>
-      <c r="L66" s="102" t="s">
+      <c r="L66" s="103" t="s">
         <v>8</v>
       </c>
-      <c r="M66" s="129" t="s">
+      <c r="M66" s="106" t="s">
         <v>9</v>
       </c>
-      <c r="N66" s="129" t="s">
+      <c r="N66" s="106" t="s">
         <v>10</v>
       </c>
-      <c r="O66" s="102" t="s">
+      <c r="O66" s="103" t="s">
         <v>11</v>
       </c>
-      <c r="Q66" s="135" t="s">
+      <c r="Q66" s="112" t="s">
         <v>24</v>
       </c>
-      <c r="R66" s="135" t="s">
+      <c r="R66" s="112" t="s">
         <v>4</v>
       </c>
-      <c r="S66" s="135" t="s">
+      <c r="S66" s="112" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="67" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D67" s="124"/>
-      <c r="E67" s="127"/>
-      <c r="G67" s="121"/>
-      <c r="H67" s="133"/>
-      <c r="I67" s="133"/>
-      <c r="J67" s="121"/>
-      <c r="L67" s="103"/>
-      <c r="M67" s="130"/>
-      <c r="N67" s="130"/>
-      <c r="O67" s="103"/>
-      <c r="Q67" s="136"/>
-      <c r="R67" s="136"/>
-      <c r="S67" s="136"/>
+      <c r="D67" s="98"/>
+      <c r="E67" s="101"/>
+      <c r="G67" s="95"/>
+      <c r="H67" s="110"/>
+      <c r="I67" s="110"/>
+      <c r="J67" s="95"/>
+      <c r="L67" s="104"/>
+      <c r="M67" s="107"/>
+      <c r="N67" s="107"/>
+      <c r="O67" s="104"/>
+      <c r="Q67" s="113"/>
+      <c r="R67" s="113"/>
+      <c r="S67" s="113"/>
     </row>
     <row r="68" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D68" s="124"/>
-      <c r="E68" s="127"/>
-      <c r="G68" s="121"/>
-      <c r="H68" s="133"/>
-      <c r="I68" s="133"/>
-      <c r="J68" s="121"/>
-      <c r="L68" s="103"/>
-      <c r="M68" s="130"/>
-      <c r="N68" s="130"/>
-      <c r="O68" s="103"/>
-      <c r="Q68" s="136"/>
-      <c r="R68" s="136"/>
-      <c r="S68" s="136"/>
+      <c r="D68" s="98"/>
+      <c r="E68" s="101"/>
+      <c r="G68" s="95"/>
+      <c r="H68" s="110"/>
+      <c r="I68" s="110"/>
+      <c r="J68" s="95"/>
+      <c r="L68" s="104"/>
+      <c r="M68" s="107"/>
+      <c r="N68" s="107"/>
+      <c r="O68" s="104"/>
+      <c r="Q68" s="113"/>
+      <c r="R68" s="113"/>
+      <c r="S68" s="113"/>
     </row>
     <row r="69" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D69" s="124"/>
-      <c r="E69" s="127"/>
-      <c r="G69" s="121"/>
-      <c r="H69" s="133"/>
-      <c r="I69" s="133"/>
-      <c r="J69" s="121"/>
-      <c r="L69" s="103"/>
-      <c r="M69" s="130"/>
-      <c r="N69" s="130"/>
-      <c r="O69" s="103"/>
-      <c r="Q69" s="136"/>
-      <c r="R69" s="136"/>
-      <c r="S69" s="136"/>
+      <c r="D69" s="98"/>
+      <c r="E69" s="101"/>
+      <c r="G69" s="95"/>
+      <c r="H69" s="110"/>
+      <c r="I69" s="110"/>
+      <c r="J69" s="95"/>
+      <c r="L69" s="104"/>
+      <c r="M69" s="107"/>
+      <c r="N69" s="107"/>
+      <c r="O69" s="104"/>
+      <c r="Q69" s="113"/>
+      <c r="R69" s="113"/>
+      <c r="S69" s="113"/>
     </row>
     <row r="70" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D70" s="124"/>
-      <c r="E70" s="127"/>
-      <c r="G70" s="121"/>
-      <c r="H70" s="133"/>
-      <c r="I70" s="133"/>
-      <c r="J70" s="121"/>
-      <c r="L70" s="103"/>
-      <c r="M70" s="130"/>
-      <c r="N70" s="130"/>
-      <c r="O70" s="103"/>
-      <c r="Q70" s="136"/>
-      <c r="R70" s="136"/>
-      <c r="S70" s="136"/>
+      <c r="D70" s="98"/>
+      <c r="E70" s="101"/>
+      <c r="G70" s="95"/>
+      <c r="H70" s="110"/>
+      <c r="I70" s="110"/>
+      <c r="J70" s="95"/>
+      <c r="L70" s="104"/>
+      <c r="M70" s="107"/>
+      <c r="N70" s="107"/>
+      <c r="O70" s="104"/>
+      <c r="Q70" s="113"/>
+      <c r="R70" s="113"/>
+      <c r="S70" s="113"/>
     </row>
     <row r="71" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D71" s="124"/>
-      <c r="E71" s="127"/>
-      <c r="G71" s="121"/>
-      <c r="H71" s="133"/>
-      <c r="I71" s="133"/>
-      <c r="J71" s="121"/>
-      <c r="L71" s="103"/>
-      <c r="M71" s="130"/>
-      <c r="N71" s="130"/>
-      <c r="O71" s="103"/>
-      <c r="Q71" s="136"/>
-      <c r="R71" s="136"/>
-      <c r="S71" s="136"/>
+      <c r="D71" s="98"/>
+      <c r="E71" s="101"/>
+      <c r="G71" s="95"/>
+      <c r="H71" s="110"/>
+      <c r="I71" s="110"/>
+      <c r="J71" s="95"/>
+      <c r="L71" s="104"/>
+      <c r="M71" s="107"/>
+      <c r="N71" s="107"/>
+      <c r="O71" s="104"/>
+      <c r="Q71" s="113"/>
+      <c r="R71" s="113"/>
+      <c r="S71" s="113"/>
     </row>
     <row r="72" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D72" s="124"/>
-      <c r="E72" s="127"/>
-      <c r="G72" s="121"/>
-      <c r="H72" s="133"/>
-      <c r="I72" s="133"/>
-      <c r="J72" s="121"/>
-      <c r="L72" s="103"/>
-      <c r="M72" s="130"/>
-      <c r="N72" s="130"/>
-      <c r="O72" s="103"/>
-      <c r="Q72" s="136"/>
-      <c r="R72" s="136"/>
-      <c r="S72" s="136"/>
+      <c r="D72" s="98"/>
+      <c r="E72" s="101"/>
+      <c r="G72" s="95"/>
+      <c r="H72" s="110"/>
+      <c r="I72" s="110"/>
+      <c r="J72" s="95"/>
+      <c r="L72" s="104"/>
+      <c r="M72" s="107"/>
+      <c r="N72" s="107"/>
+      <c r="O72" s="104"/>
+      <c r="Q72" s="113"/>
+      <c r="R72" s="113"/>
+      <c r="S72" s="113"/>
     </row>
     <row r="73" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D73" s="124"/>
-      <c r="E73" s="127"/>
-      <c r="G73" s="121"/>
-      <c r="H73" s="133"/>
-      <c r="I73" s="133"/>
-      <c r="J73" s="121"/>
-      <c r="L73" s="103"/>
-      <c r="M73" s="130"/>
-      <c r="N73" s="130"/>
-      <c r="O73" s="103"/>
-      <c r="Q73" s="136"/>
-      <c r="R73" s="136"/>
-      <c r="S73" s="136"/>
+      <c r="D73" s="98"/>
+      <c r="E73" s="101"/>
+      <c r="G73" s="95"/>
+      <c r="H73" s="110"/>
+      <c r="I73" s="110"/>
+      <c r="J73" s="95"/>
+      <c r="L73" s="104"/>
+      <c r="M73" s="107"/>
+      <c r="N73" s="107"/>
+      <c r="O73" s="104"/>
+      <c r="Q73" s="113"/>
+      <c r="R73" s="113"/>
+      <c r="S73" s="113"/>
     </row>
     <row r="74" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D74" s="124"/>
-      <c r="E74" s="127"/>
-      <c r="G74" s="121"/>
-      <c r="H74" s="133"/>
-      <c r="I74" s="133"/>
-      <c r="J74" s="121"/>
-      <c r="L74" s="103"/>
-      <c r="M74" s="130"/>
-      <c r="N74" s="130"/>
-      <c r="O74" s="103"/>
-      <c r="Q74" s="136"/>
-      <c r="R74" s="136"/>
-      <c r="S74" s="136"/>
+      <c r="D74" s="98"/>
+      <c r="E74" s="101"/>
+      <c r="G74" s="95"/>
+      <c r="H74" s="110"/>
+      <c r="I74" s="110"/>
+      <c r="J74" s="95"/>
+      <c r="L74" s="104"/>
+      <c r="M74" s="107"/>
+      <c r="N74" s="107"/>
+      <c r="O74" s="104"/>
+      <c r="Q74" s="113"/>
+      <c r="R74" s="113"/>
+      <c r="S74" s="113"/>
     </row>
     <row r="75" spans="1:20" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D75" s="125"/>
-      <c r="E75" s="128"/>
-      <c r="G75" s="122"/>
-      <c r="H75" s="134"/>
-      <c r="I75" s="134"/>
-      <c r="J75" s="122"/>
-      <c r="L75" s="104"/>
-      <c r="M75" s="131"/>
-      <c r="N75" s="131"/>
-      <c r="O75" s="104"/>
-      <c r="Q75" s="137"/>
-      <c r="R75" s="137"/>
-      <c r="S75" s="137"/>
+      <c r="D75" s="99"/>
+      <c r="E75" s="102"/>
+      <c r="G75" s="96"/>
+      <c r="H75" s="111"/>
+      <c r="I75" s="111"/>
+      <c r="J75" s="96"/>
+      <c r="L75" s="105"/>
+      <c r="M75" s="108"/>
+      <c r="N75" s="108"/>
+      <c r="O75" s="105"/>
+      <c r="Q75" s="114"/>
+      <c r="R75" s="114"/>
+      <c r="S75" s="114"/>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B6:T60">
     <sortCondition ref="B6"/>
   </sortState>
   <mergeCells count="25">
+    <mergeCell ref="G2:K2"/>
+    <mergeCell ref="D2:F2"/>
+    <mergeCell ref="Q3:T4"/>
+    <mergeCell ref="O66:O75"/>
+    <mergeCell ref="A2:A5"/>
+    <mergeCell ref="G3:K4"/>
+    <mergeCell ref="D3:F4"/>
+    <mergeCell ref="B2:B5"/>
+    <mergeCell ref="C2:C5"/>
     <mergeCell ref="B1:T1"/>
     <mergeCell ref="J66:J75"/>
     <mergeCell ref="D66:D75"/>
@@ -7706,15 +7708,6 @@
     <mergeCell ref="I66:I75"/>
     <mergeCell ref="Q2:T2"/>
     <mergeCell ref="L2:P2"/>
-    <mergeCell ref="G2:K2"/>
-    <mergeCell ref="D2:F2"/>
-    <mergeCell ref="Q3:T4"/>
-    <mergeCell ref="O66:O75"/>
-    <mergeCell ref="A2:A5"/>
-    <mergeCell ref="G3:K4"/>
-    <mergeCell ref="D3:F4"/>
-    <mergeCell ref="B2:B5"/>
-    <mergeCell ref="C2:C5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
ya saben manejas tabla de doble entrada
</commit_message>
<xml_diff>
--- a/9_asistencia_evaluacion/pivu_caucasia_notas_quices_asistencia.xlsx
+++ b/9_asistencia_evaluacion/pivu_caucasia_notas_quices_asistencia.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marco\Documentos\extension\camino-udea\9_asistencia_evaluacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C51AA121-A4C0-4B93-A344-E4CAD4B441A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{998C5AEF-2BA1-4162-AE05-A1E7D4219D72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Inscritos" sheetId="2" r:id="rId1"/>
@@ -1133,6 +1133,84 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1163,15 +1241,6 @@
     <xf numFmtId="0" fontId="7" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
@@ -1215,75 +1284,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="9" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -3374,14 +3374,14 @@
         <v>1038111245</v>
       </c>
       <c r="D14" s="13">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E14" s="13"/>
       <c r="F14" s="13"/>
       <c r="G14" s="13"/>
       <c r="H14" s="32">
         <f t="shared" si="0"/>
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="I14" s="33"/>
       <c r="J14" s="33"/>
@@ -3854,13 +3854,15 @@
         <f>+Inscritos!D21</f>
         <v>1038113598</v>
       </c>
-      <c r="D23" s="13"/>
+      <c r="D23" s="13">
+        <v>1</v>
+      </c>
       <c r="E23" s="13"/>
       <c r="F23" s="13"/>
       <c r="G23" s="13"/>
       <c r="H23" s="32">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="I23" s="33"/>
       <c r="J23" s="33"/>
@@ -4173,14 +4175,14 @@
         <v>1038109706</v>
       </c>
       <c r="D29" s="13">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E29" s="13"/>
       <c r="F29" s="13"/>
       <c r="G29" s="13"/>
       <c r="H29" s="32">
         <f t="shared" si="0"/>
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="I29" s="33"/>
       <c r="J29" s="33"/>
@@ -4336,14 +4338,14 @@
         <v>1038104210</v>
       </c>
       <c r="D32" s="13">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E32" s="13"/>
       <c r="F32" s="13"/>
       <c r="G32" s="13"/>
       <c r="H32" s="32">
         <f t="shared" si="0"/>
-        <v>0.75</v>
+        <v>1</v>
       </c>
       <c r="I32" s="33"/>
       <c r="J32" s="33"/>
@@ -4813,30 +4815,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="72.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B1" s="93" t="s">
+      <c r="B1" s="119" t="s">
         <v>18</v>
       </c>
-      <c r="C1" s="93"/>
-      <c r="D1" s="93"/>
-      <c r="E1" s="93"/>
-      <c r="F1" s="93"/>
-      <c r="G1" s="93"/>
-      <c r="H1" s="93"/>
-      <c r="I1" s="93"/>
-      <c r="J1" s="93"/>
-      <c r="K1" s="93"/>
-      <c r="L1" s="93"/>
-      <c r="M1" s="93"/>
-      <c r="N1" s="93"/>
-      <c r="O1" s="93"/>
-      <c r="P1" s="93"/>
-      <c r="Q1" s="93"/>
-      <c r="R1" s="93"/>
-      <c r="S1" s="93"/>
-      <c r="T1" s="93"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
+      <c r="E1" s="119"/>
+      <c r="F1" s="119"/>
+      <c r="G1" s="119"/>
+      <c r="H1" s="119"/>
+      <c r="I1" s="119"/>
+      <c r="J1" s="119"/>
+      <c r="K1" s="119"/>
+      <c r="L1" s="119"/>
+      <c r="M1" s="119"/>
+      <c r="N1" s="119"/>
+      <c r="O1" s="119"/>
+      <c r="P1" s="119"/>
+      <c r="Q1" s="119"/>
+      <c r="R1" s="119"/>
+      <c r="S1" s="119"/>
+      <c r="T1" s="119"/>
     </row>
     <row r="2" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="130" t="s">
+      <c r="A2" s="105" t="s">
         <v>13</v>
       </c>
       <c r="B2" s="91" t="s">
@@ -4845,89 +4847,89 @@
       <c r="C2" s="67" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="121" t="str">
+      <c r="D2" s="93" t="str">
         <f>Asistencia!D2</f>
         <v>NOMBRE DOCENTE</v>
       </c>
-      <c r="E2" s="122"/>
-      <c r="F2" s="123"/>
-      <c r="G2" s="121" t="str">
+      <c r="E2" s="94"/>
+      <c r="F2" s="95"/>
+      <c r="G2" s="93" t="str">
         <f>Asistencia!I2</f>
         <v>NOMBRE DOCENTE</v>
       </c>
-      <c r="H2" s="122"/>
-      <c r="I2" s="122"/>
-      <c r="J2" s="122"/>
-      <c r="K2" s="123"/>
-      <c r="L2" s="121" t="s">
+      <c r="H2" s="94"/>
+      <c r="I2" s="94"/>
+      <c r="J2" s="94"/>
+      <c r="K2" s="95"/>
+      <c r="L2" s="93" t="s">
         <v>19</v>
       </c>
-      <c r="M2" s="122"/>
-      <c r="N2" s="122"/>
-      <c r="O2" s="122"/>
-      <c r="P2" s="123"/>
-      <c r="Q2" s="121" t="str">
+      <c r="M2" s="94"/>
+      <c r="N2" s="94"/>
+      <c r="O2" s="94"/>
+      <c r="P2" s="95"/>
+      <c r="Q2" s="93" t="str">
         <f>Asistencia!AA2</f>
         <v>NOMBRE DOCENTE</v>
       </c>
-      <c r="R2" s="122"/>
-      <c r="S2" s="122"/>
-      <c r="T2" s="123"/>
+      <c r="R2" s="94"/>
+      <c r="S2" s="94"/>
+      <c r="T2" s="95"/>
     </row>
     <row r="3" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="131"/>
+      <c r="A3" s="106"/>
       <c r="B3" s="92"/>
       <c r="C3" s="68"/>
-      <c r="D3" s="138" t="s">
+      <c r="D3" s="113" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="139"/>
-      <c r="F3" s="140"/>
-      <c r="G3" s="132" t="s">
+      <c r="E3" s="114"/>
+      <c r="F3" s="115"/>
+      <c r="G3" s="107" t="s">
         <v>2</v>
       </c>
-      <c r="H3" s="133"/>
-      <c r="I3" s="133"/>
-      <c r="J3" s="133"/>
-      <c r="K3" s="134"/>
-      <c r="L3" s="115" t="s">
+      <c r="H3" s="108"/>
+      <c r="I3" s="108"/>
+      <c r="J3" s="108"/>
+      <c r="K3" s="109"/>
+      <c r="L3" s="138" t="s">
         <v>1</v>
       </c>
-      <c r="M3" s="116"/>
-      <c r="N3" s="116"/>
-      <c r="O3" s="116"/>
-      <c r="P3" s="117"/>
-      <c r="Q3" s="124" t="s">
-        <v>0</v>
-      </c>
-      <c r="R3" s="125"/>
-      <c r="S3" s="125"/>
-      <c r="T3" s="126"/>
+      <c r="M3" s="139"/>
+      <c r="N3" s="139"/>
+      <c r="O3" s="139"/>
+      <c r="P3" s="140"/>
+      <c r="Q3" s="96" t="s">
+        <v>0</v>
+      </c>
+      <c r="R3" s="97"/>
+      <c r="S3" s="97"/>
+      <c r="T3" s="98"/>
     </row>
     <row r="4" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="131"/>
+      <c r="A4" s="106"/>
       <c r="B4" s="92"/>
       <c r="C4" s="68"/>
-      <c r="D4" s="141"/>
-      <c r="E4" s="142"/>
-      <c r="F4" s="143"/>
-      <c r="G4" s="135"/>
-      <c r="H4" s="136"/>
-      <c r="I4" s="136"/>
-      <c r="J4" s="136"/>
-      <c r="K4" s="137"/>
-      <c r="L4" s="118"/>
-      <c r="M4" s="119"/>
-      <c r="N4" s="119"/>
-      <c r="O4" s="119"/>
-      <c r="P4" s="120"/>
-      <c r="Q4" s="127"/>
-      <c r="R4" s="128"/>
-      <c r="S4" s="128"/>
-      <c r="T4" s="129"/>
+      <c r="D4" s="116"/>
+      <c r="E4" s="117"/>
+      <c r="F4" s="118"/>
+      <c r="G4" s="110"/>
+      <c r="H4" s="111"/>
+      <c r="I4" s="111"/>
+      <c r="J4" s="111"/>
+      <c r="K4" s="112"/>
+      <c r="L4" s="141"/>
+      <c r="M4" s="142"/>
+      <c r="N4" s="142"/>
+      <c r="O4" s="142"/>
+      <c r="P4" s="143"/>
+      <c r="Q4" s="99"/>
+      <c r="R4" s="100"/>
+      <c r="S4" s="100"/>
+      <c r="T4" s="101"/>
     </row>
     <row r="5" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="131"/>
+      <c r="A5" s="106"/>
       <c r="B5" s="92"/>
       <c r="C5" s="68"/>
       <c r="D5" s="17">
@@ -7503,195 +7505,186 @@
       </c>
     </row>
     <row r="66" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D66" s="97" t="s">
+      <c r="D66" s="123" t="s">
         <v>24</v>
       </c>
-      <c r="E66" s="100" t="s">
+      <c r="E66" s="126" t="s">
         <v>12</v>
       </c>
-      <c r="G66" s="94" t="s">
+      <c r="G66" s="120" t="s">
         <v>8</v>
       </c>
-      <c r="H66" s="109" t="s">
+      <c r="H66" s="132" t="s">
         <v>9</v>
       </c>
-      <c r="I66" s="109" t="s">
+      <c r="I66" s="132" t="s">
         <v>10</v>
       </c>
-      <c r="J66" s="94" t="s">
+      <c r="J66" s="120" t="s">
         <v>11</v>
       </c>
-      <c r="L66" s="103" t="s">
+      <c r="L66" s="102" t="s">
         <v>8</v>
       </c>
-      <c r="M66" s="106" t="s">
+      <c r="M66" s="129" t="s">
         <v>9</v>
       </c>
-      <c r="N66" s="106" t="s">
+      <c r="N66" s="129" t="s">
         <v>10</v>
       </c>
-      <c r="O66" s="103" t="s">
+      <c r="O66" s="102" t="s">
         <v>11</v>
       </c>
-      <c r="Q66" s="112" t="s">
+      <c r="Q66" s="135" t="s">
         <v>24</v>
       </c>
-      <c r="R66" s="112" t="s">
+      <c r="R66" s="135" t="s">
         <v>4</v>
       </c>
-      <c r="S66" s="112" t="s">
+      <c r="S66" s="135" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="67" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D67" s="98"/>
-      <c r="E67" s="101"/>
-      <c r="G67" s="95"/>
-      <c r="H67" s="110"/>
-      <c r="I67" s="110"/>
-      <c r="J67" s="95"/>
-      <c r="L67" s="104"/>
-      <c r="M67" s="107"/>
-      <c r="N67" s="107"/>
-      <c r="O67" s="104"/>
-      <c r="Q67" s="113"/>
-      <c r="R67" s="113"/>
-      <c r="S67" s="113"/>
+      <c r="D67" s="124"/>
+      <c r="E67" s="127"/>
+      <c r="G67" s="121"/>
+      <c r="H67" s="133"/>
+      <c r="I67" s="133"/>
+      <c r="J67" s="121"/>
+      <c r="L67" s="103"/>
+      <c r="M67" s="130"/>
+      <c r="N67" s="130"/>
+      <c r="O67" s="103"/>
+      <c r="Q67" s="136"/>
+      <c r="R67" s="136"/>
+      <c r="S67" s="136"/>
     </row>
     <row r="68" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D68" s="98"/>
-      <c r="E68" s="101"/>
-      <c r="G68" s="95"/>
-      <c r="H68" s="110"/>
-      <c r="I68" s="110"/>
-      <c r="J68" s="95"/>
-      <c r="L68" s="104"/>
-      <c r="M68" s="107"/>
-      <c r="N68" s="107"/>
-      <c r="O68" s="104"/>
-      <c r="Q68" s="113"/>
-      <c r="R68" s="113"/>
-      <c r="S68" s="113"/>
+      <c r="D68" s="124"/>
+      <c r="E68" s="127"/>
+      <c r="G68" s="121"/>
+      <c r="H68" s="133"/>
+      <c r="I68" s="133"/>
+      <c r="J68" s="121"/>
+      <c r="L68" s="103"/>
+      <c r="M68" s="130"/>
+      <c r="N68" s="130"/>
+      <c r="O68" s="103"/>
+      <c r="Q68" s="136"/>
+      <c r="R68" s="136"/>
+      <c r="S68" s="136"/>
     </row>
     <row r="69" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D69" s="98"/>
-      <c r="E69" s="101"/>
-      <c r="G69" s="95"/>
-      <c r="H69" s="110"/>
-      <c r="I69" s="110"/>
-      <c r="J69" s="95"/>
-      <c r="L69" s="104"/>
-      <c r="M69" s="107"/>
-      <c r="N69" s="107"/>
-      <c r="O69" s="104"/>
-      <c r="Q69" s="113"/>
-      <c r="R69" s="113"/>
-      <c r="S69" s="113"/>
+      <c r="D69" s="124"/>
+      <c r="E69" s="127"/>
+      <c r="G69" s="121"/>
+      <c r="H69" s="133"/>
+      <c r="I69" s="133"/>
+      <c r="J69" s="121"/>
+      <c r="L69" s="103"/>
+      <c r="M69" s="130"/>
+      <c r="N69" s="130"/>
+      <c r="O69" s="103"/>
+      <c r="Q69" s="136"/>
+      <c r="R69" s="136"/>
+      <c r="S69" s="136"/>
     </row>
     <row r="70" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D70" s="98"/>
-      <c r="E70" s="101"/>
-      <c r="G70" s="95"/>
-      <c r="H70" s="110"/>
-      <c r="I70" s="110"/>
-      <c r="J70" s="95"/>
-      <c r="L70" s="104"/>
-      <c r="M70" s="107"/>
-      <c r="N70" s="107"/>
-      <c r="O70" s="104"/>
-      <c r="Q70" s="113"/>
-      <c r="R70" s="113"/>
-      <c r="S70" s="113"/>
+      <c r="D70" s="124"/>
+      <c r="E70" s="127"/>
+      <c r="G70" s="121"/>
+      <c r="H70" s="133"/>
+      <c r="I70" s="133"/>
+      <c r="J70" s="121"/>
+      <c r="L70" s="103"/>
+      <c r="M70" s="130"/>
+      <c r="N70" s="130"/>
+      <c r="O70" s="103"/>
+      <c r="Q70" s="136"/>
+      <c r="R70" s="136"/>
+      <c r="S70" s="136"/>
     </row>
     <row r="71" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D71" s="98"/>
-      <c r="E71" s="101"/>
-      <c r="G71" s="95"/>
-      <c r="H71" s="110"/>
-      <c r="I71" s="110"/>
-      <c r="J71" s="95"/>
-      <c r="L71" s="104"/>
-      <c r="M71" s="107"/>
-      <c r="N71" s="107"/>
-      <c r="O71" s="104"/>
-      <c r="Q71" s="113"/>
-      <c r="R71" s="113"/>
-      <c r="S71" s="113"/>
+      <c r="D71" s="124"/>
+      <c r="E71" s="127"/>
+      <c r="G71" s="121"/>
+      <c r="H71" s="133"/>
+      <c r="I71" s="133"/>
+      <c r="J71" s="121"/>
+      <c r="L71" s="103"/>
+      <c r="M71" s="130"/>
+      <c r="N71" s="130"/>
+      <c r="O71" s="103"/>
+      <c r="Q71" s="136"/>
+      <c r="R71" s="136"/>
+      <c r="S71" s="136"/>
     </row>
     <row r="72" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D72" s="98"/>
-      <c r="E72" s="101"/>
-      <c r="G72" s="95"/>
-      <c r="H72" s="110"/>
-      <c r="I72" s="110"/>
-      <c r="J72" s="95"/>
-      <c r="L72" s="104"/>
-      <c r="M72" s="107"/>
-      <c r="N72" s="107"/>
-      <c r="O72" s="104"/>
-      <c r="Q72" s="113"/>
-      <c r="R72" s="113"/>
-      <c r="S72" s="113"/>
+      <c r="D72" s="124"/>
+      <c r="E72" s="127"/>
+      <c r="G72" s="121"/>
+      <c r="H72" s="133"/>
+      <c r="I72" s="133"/>
+      <c r="J72" s="121"/>
+      <c r="L72" s="103"/>
+      <c r="M72" s="130"/>
+      <c r="N72" s="130"/>
+      <c r="O72" s="103"/>
+      <c r="Q72" s="136"/>
+      <c r="R72" s="136"/>
+      <c r="S72" s="136"/>
     </row>
     <row r="73" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D73" s="98"/>
-      <c r="E73" s="101"/>
-      <c r="G73" s="95"/>
-      <c r="H73" s="110"/>
-      <c r="I73" s="110"/>
-      <c r="J73" s="95"/>
-      <c r="L73" s="104"/>
-      <c r="M73" s="107"/>
-      <c r="N73" s="107"/>
-      <c r="O73" s="104"/>
-      <c r="Q73" s="113"/>
-      <c r="R73" s="113"/>
-      <c r="S73" s="113"/>
+      <c r="D73" s="124"/>
+      <c r="E73" s="127"/>
+      <c r="G73" s="121"/>
+      <c r="H73" s="133"/>
+      <c r="I73" s="133"/>
+      <c r="J73" s="121"/>
+      <c r="L73" s="103"/>
+      <c r="M73" s="130"/>
+      <c r="N73" s="130"/>
+      <c r="O73" s="103"/>
+      <c r="Q73" s="136"/>
+      <c r="R73" s="136"/>
+      <c r="S73" s="136"/>
     </row>
     <row r="74" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="D74" s="98"/>
-      <c r="E74" s="101"/>
-      <c r="G74" s="95"/>
-      <c r="H74" s="110"/>
-      <c r="I74" s="110"/>
-      <c r="J74" s="95"/>
-      <c r="L74" s="104"/>
-      <c r="M74" s="107"/>
-      <c r="N74" s="107"/>
-      <c r="O74" s="104"/>
-      <c r="Q74" s="113"/>
-      <c r="R74" s="113"/>
-      <c r="S74" s="113"/>
+      <c r="D74" s="124"/>
+      <c r="E74" s="127"/>
+      <c r="G74" s="121"/>
+      <c r="H74" s="133"/>
+      <c r="I74" s="133"/>
+      <c r="J74" s="121"/>
+      <c r="L74" s="103"/>
+      <c r="M74" s="130"/>
+      <c r="N74" s="130"/>
+      <c r="O74" s="103"/>
+      <c r="Q74" s="136"/>
+      <c r="R74" s="136"/>
+      <c r="S74" s="136"/>
     </row>
     <row r="75" spans="1:20" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D75" s="99"/>
-      <c r="E75" s="102"/>
-      <c r="G75" s="96"/>
-      <c r="H75" s="111"/>
-      <c r="I75" s="111"/>
-      <c r="J75" s="96"/>
-      <c r="L75" s="105"/>
-      <c r="M75" s="108"/>
-      <c r="N75" s="108"/>
-      <c r="O75" s="105"/>
-      <c r="Q75" s="114"/>
-      <c r="R75" s="114"/>
-      <c r="S75" s="114"/>
+      <c r="D75" s="125"/>
+      <c r="E75" s="128"/>
+      <c r="G75" s="122"/>
+      <c r="H75" s="134"/>
+      <c r="I75" s="134"/>
+      <c r="J75" s="122"/>
+      <c r="L75" s="104"/>
+      <c r="M75" s="131"/>
+      <c r="N75" s="131"/>
+      <c r="O75" s="104"/>
+      <c r="Q75" s="137"/>
+      <c r="R75" s="137"/>
+      <c r="S75" s="137"/>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B6:T60">
     <sortCondition ref="B6"/>
   </sortState>
   <mergeCells count="25">
-    <mergeCell ref="G2:K2"/>
-    <mergeCell ref="D2:F2"/>
-    <mergeCell ref="Q3:T4"/>
-    <mergeCell ref="O66:O75"/>
-    <mergeCell ref="A2:A5"/>
-    <mergeCell ref="G3:K4"/>
-    <mergeCell ref="D3:F4"/>
-    <mergeCell ref="B2:B5"/>
-    <mergeCell ref="C2:C5"/>
     <mergeCell ref="B1:T1"/>
     <mergeCell ref="J66:J75"/>
     <mergeCell ref="D66:D75"/>
@@ -7708,6 +7701,15 @@
     <mergeCell ref="I66:I75"/>
     <mergeCell ref="Q2:T2"/>
     <mergeCell ref="L2:P2"/>
+    <mergeCell ref="G2:K2"/>
+    <mergeCell ref="D2:F2"/>
+    <mergeCell ref="Q3:T4"/>
+    <mergeCell ref="O66:O75"/>
+    <mergeCell ref="A2:A5"/>
+    <mergeCell ref="G3:K4"/>
+    <mergeCell ref="D3:F4"/>
+    <mergeCell ref="B2:B5"/>
+    <mergeCell ref="C2:C5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>